<commit_message>
Remove missing verbs from dataset
</commit_message>
<xml_diff>
--- a/Dataset/Template_Unexpanded.xlsx
+++ b/Dataset/Template_Unexpanded.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F143"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1183,7 +1183,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>maghilawas</t>
+          <t>magtagay sa kalipay</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1193,17 +1193,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ang maghilawas nga mga tawo kasagaran wala'y klaro nga relasyon.; Dili maayo nga magsige ug maghilawas kay makadaot kini sa imong lawas ug isip.; Ang mga maghilawas nga binuhatan makaguba sa maayong reputasyon.; Ang mga tambag sa mga ginikanan kasagaran naglikay sa maghilawas nga binuhatan.; Ang maghilawas nga kinaiya sa uban makapalayo sa ilang mga higala ug pamilya.</t>
+          <t>Ang mga magtagay sa kalipay kasagaran makita sa mga parties ug celebrations.; Ang ilang magtagay sa kalipay nakaingon ug dakong kalipay sa tanan nga niapil.; Sa birthday ni Juan, nagmagtagay sa kalipay ang mga bisita hangtod sa kadlawn.; Ang mga magbarkada nagmagtagay sa kalipay human sa ilang reunion.; Ang mga mag-asawa nagmagtagay sa kalipay sa ilang anniversary celebration.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ang maghilawas nga mga tawo kasagaran wala'y klaro nga relasyon.; Dili maayo nga magsige ug maghilawas kay makadaot kini sa imong lawas ug isip.; Ang mga maghilawas nga binuhatan makaguba sa maayong reputasyon.; Ang mga tambag sa mga ginikanan kasagaran naglikay sa maghilawas nga binuhatan.; Ang maghilawas nga kinaiya sa uban makapalayo sa ilang mga higala ug pamilya.</t>
+          <t>Ang mga magtagay sa kalipay kasagaran makita sa mga parties ug celebrations.; Ang ilang magtagay sa kalipay nakaingon ug dakong kalipay sa tanan nga niapil.; Sa birthday ni Juan, nagmagtagay sa kalipay ang mga bisita hangtod sa kadlawn.; Ang mga magbarkada nagmagtagay sa kalipay human sa ilang reunion.; Ang mga mag-asawa nagmagtagay sa kalipay sa ilang anniversary celebration.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['magtagay']</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1213,7 +1213,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>magtagay sa kalipay</t>
+          <t>molayag sa kalipay</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1223,17 +1223,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ang mga magtagay sa kalipay kasagaran makita sa mga parties ug celebrations.; Ang ilang magtagay sa kalipay nakaingon ug dakong kalipay sa tanan nga niapil.; Sa birthday ni Juan, nagmagtagay sa kalipay ang mga bisita hangtod sa kadlawn.; Ang mga magbarkada nagmagtagay sa kalipay human sa ilang reunion.; Ang mga mag-asawa nagmagtagay sa kalipay sa ilang anniversary celebration.</t>
+          <t>Ang mga magkauban nagmolayag sa kalipay sa ilang outing sa beach.; Sa dihang nagmolayag sa kalipay ang grupo, nakalimot sila sa ilang mga problema.; Ang mga kabatan-onan nagmolayag sa kalipay human sa ilang graduation.; Ang pamilya nagmolayag sa kalipay sa ilang bakasyon sa probinsya.; Ang mga amigo nagmolayag sa kalipay sa ilang road trip.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ang mga magtagay sa kalipay kasagaran makita sa mga parties ug celebrations.; Ang ilang magtagay sa kalipay nakaingon ug dakong kalipay sa tanan nga niapil.; Sa birthday ni Juan, nagmagtagay sa kalipay ang mga bisita hangtod sa kadlawn.; Ang mga magbarkada nagmagtagay sa kalipay human sa ilang reunion.; Ang mga mag-asawa nagmagtagay sa kalipay sa ilang anniversary celebration.</t>
+          <t>Ang mga magkauban nagmolayag sa kalipay sa ilang outing sa beach.; Sa dihang nagmolayag sa kalipay ang grupo, nakalimot sila sa ilang mga problema.; Ang mga kabatan-onan nagmolayag sa kalipay human sa ilang graduation.; Ang pamilya nagmolayag sa kalipay sa ilang bakasyon sa probinsya.; Ang mga amigo nagmolayag sa kalipay sa ilang road trip.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>['magtagay']</t>
+          <t>['molayag']</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1243,27 +1243,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>molayag sa kalipay</t>
+          <t>paabang</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>sa pagpakigsekso</t>
+          <t>pag-abang</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ang mga magkauban nagmolayag sa kalipay sa ilang outing sa beach.; Sa dihang nagmolayag sa kalipay ang grupo, nakalimot sila sa ilang mga problema.; Ang mga kabatan-onan nagmolayag sa kalipay human sa ilang graduation.; Ang pamilya nagmolayag sa kalipay sa ilang bakasyon sa probinsya.; Ang mga amigo nagmolayag sa kalipay sa ilang road trip.</t>
+          <t>Gipahimutang ang iyang balay aron ipaabang sa mga bakasyonista.; Ang mga kwartong ipaabang kay dali ra kaayo mahurot ug ma-book.; Gipangita ang mga paabang nga balay nga duol sa eskwelahan.; Ang ilang negosyo nga paabang og sakyanan kay booming na kaayo karon.; Nagpaabang ug mga bisikleta ang resort para sa ilang mga bisita.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ang mga magkauban nagmolayag sa kalipay sa ilang outing sa beach.; Sa dihang nagmolayag sa kalipay ang grupo, nakalimot sila sa ilang mga problema.; Ang mga kabatan-onan nagmolayag sa kalipay human sa ilang graduation.; Ang pamilya nagmolayag sa kalipay sa ilang bakasyon sa probinsya.; Ang mga amigo nagmolayag sa kalipay sa ilang road trip.</t>
+          <t>Gipahimutang ang iyang balay aron ipaabang sa mga bakasyonista.; Ang mga kwartong ipaabang kay dali ra kaayo mahurot ug ma-book.; Gipangita ang mga paabang nga balay nga duol sa eskwelahan.; Ang ilang negosyo nga paabang og sakyanan kay booming na kaayo karon.; Nagpaabang ug mga bisikleta ang resort para sa ilang mga bisita.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>['molayag']</t>
+          <t>['paabang']</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1273,27 +1273,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>paabang</t>
+          <t>rampa</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>pag-abang</t>
+          <t>ramp</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gipahimutang ang iyang balay aron ipaabang sa mga bakasyonista.; Ang mga kwartong ipaabang kay dali ra kaayo mahurot ug ma-book.; Gipangita ang mga paabang nga balay nga duol sa eskwelahan.; Ang ilang negosyo nga paabang og sakyanan kay booming na kaayo karon.; Nagpaabang ug mga bisikleta ang resort para sa ilang mga bisita.</t>
+          <t>Nag-rampa si Ana sa fashion show ug nakadani sa mga manan-aw.; Ang mga modelo nag-rampa sa runway ug gipalakpakan sa tanan.; Si Juan ug Maria nag-rampa sa park aron mag-relax ug maglingaw-lingaw.; Ang mga dalaga ug ulitawo nag-rampa sa plaza atol sa pista.; Ang mga artista nag-rampa sa red carpet sa premiere night.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Gipahimutang ang iyang balay aron ipaabang sa mga bakasyonista.; Ang mga kwartong ipaabang kay dali ra kaayo mahurot ug ma-book.; Gipangita ang mga paabang nga balay nga duol sa eskwelahan.; Ang ilang negosyo nga paabang og sakyanan kay booming na kaayo karon.; Nagpaabang ug mga bisikleta ang resort para sa ilang mga bisita.</t>
+          <t>Nag-rampa si Ana sa fashion show ug nakadani sa mga manan-aw.; Ang mga modelo nag-rampa sa runway ug gipalakpakan sa tanan.; Si Juan ug Maria nag-rampa sa park aron mag-relax ug maglingaw-lingaw.; Ang mga dalaga ug ulitawo nag-rampa sa plaza atol sa pista.; Ang mga artista nag-rampa sa red carpet sa premiere night.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>['paabang']</t>
+          <t>['rampa']</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1303,27 +1303,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>pagkababaye</t>
+          <t>sabong</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>pagka babaye</t>
+          <t>usa ka kompetisyon</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ang iyang pagkababaye makita sa iyang pag-atiman sa pamilya.; Ang pagkababaye ni Maria nagpakita sa iyang pagka-mapinanggaon ug malumo.; Si Ana kay nagpakita sa tinuod niyang pagkababaye pinaagi sa iyang mga buhat.; Ang tinuod nga pagkababaye makita sa iyang pag-atiman ug pagpasabot sa uban.; Ang mga butang nga iyang gibuhat nagpakita sa iyang pagkababaye nga walay pagduda.</t>
+          <t>Ang sabong sa arena kay gitan-aw sa daghang mga tawo.; Ang mga manok nga ipangsabong kay gipangandaman ug maayo.; Ang mga sabong sa probinsya kasagaran ginadumog sa mga lokal nga residente.; Ang sabong sa mga manok kay paborito nga pastime sa mga kalalakin-an.; Ang mga sabong nagpakita sa abilidad sa mga magmamantala ug pag-atiman sa ilang mga manok.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ang iyang pagkababaye makita sa iyang pag-atiman sa pamilya.; Ang pagkababaye ni Maria nagpakita sa iyang pagka-mapinanggaon ug malumo.; Si Ana kay nagpakita sa tinuod niyang pagkababaye pinaagi sa iyang mga buhat.; Ang tinuod nga pagkababaye makita sa iyang pag-atiman ug pagpasabot sa uban.; Ang mga butang nga iyang gibuhat nagpakita sa iyang pagkababaye nga walay pagduda.</t>
+          <t>Ang sabong sa arena kay gitan-aw sa daghang mga tawo.; Ang mga manok nga ipangsabong kay gipangandaman ug maayo.; Ang mga sabong sa probinsya kasagaran ginadumog sa mga lokal nga residente.; Ang sabong sa mga manok kay paborito nga pastime sa mga kalalakin-an.; Ang mga sabong nagpakita sa abilidad sa mga magmamantala ug pag-atiman sa ilang mga manok.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['sabong']</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1333,27 +1333,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>rampa</t>
+          <t>taliba</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ramp</t>
+          <t>ang mga genital sa babaye</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nag-rampa si Ana sa fashion show ug nakadani sa mga manan-aw.; Ang mga modelo nag-rampa sa runway ug gipalakpakan sa tanan.; Si Juan ug Maria nag-rampa sa park aron mag-relax ug maglingaw-lingaw.; Ang mga dalaga ug ulitawo nag-rampa sa plaza atol sa pista.; Ang mga artista nag-rampa sa red carpet sa premiere night.</t>
+          <t>Ang mga pulis nag-taliba sa mga salida aron protektahan ang mga bisita.; Ang mga magtutudlo nag-taliba sa mga estudyante sa ilang field trip.; Ang mga guwardiya nag-taliba sa building adlaw ug gabii.; Ang mga volunteers nag-taliba sa event para malikayan ang mga kagubot.; Ang mga barangay tanod nag-taliba sa ilang mga area kada gabii.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Nag-rampa si Ana sa fashion show ug nakadani sa mga manan-aw.; Ang mga modelo nag-rampa sa runway ug gipalakpakan sa tanan.; Si Juan ug Maria nag-rampa sa park aron mag-relax ug maglingaw-lingaw.; Ang mga dalaga ug ulitawo nag-rampa sa plaza atol sa pista.; Ang mga artista nag-rampa sa red carpet sa premiere night.</t>
+          <t>Ang mga pulis nag-taliba sa mga salida aron protektahan ang mga bisita.; Ang mga magtutudlo nag-taliba sa mga estudyante sa ilang field trip.; Ang mga guwardiya nag-taliba sa building adlaw ug gabii.; Ang mga volunteers nag-taliba sa event para malikayan ang mga kagubot.; Ang mga barangay tanod nag-taliba sa ilang mga area kada gabii.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>['rampa']</t>
+          <t>['taliba']</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1363,27 +1363,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sabong</t>
+          <t>toyi</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>usa ka kompetisyon</t>
+          <t>coitus</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ang sabong sa arena kay gitan-aw sa daghang mga tawo.; Ang mga manok nga ipangsabong kay gipangandaman ug maayo.; Ang mga sabong sa probinsya kasagaran ginadumog sa mga lokal nga residente.; Ang sabong sa mga manok kay paborito nga pastime sa mga kalalakin-an.; Ang mga sabong nagpakita sa abilidad sa mga magmamantala ug pag-atiman sa ilang mga manok.</t>
+          <t>Ang iyang joke bahin sa toyi kay nakapatawa sa tanan.; Ang mga istorya nila bahin sa toyi kay walay kinutuban nga katawa.; Sa dihang nagbinuang siya, nagtoyi lang iyang mga amigo.; Ang ilang duwa nga toyi kay naghatag ug dako nga kalipay.; Ang iyang mga joke kay kasagaran tungkol sa toyi.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Ang sabong sa arena kay gitan-aw sa daghang mga tawo.; Ang mga manok nga ipangsabong kay gipangandaman ug maayo.; Ang mga sabong sa probinsya kasagaran ginadumog sa mga lokal nga residente.; Ang sabong sa mga manok kay paborito nga pastime sa mga kalalakin-an.; Ang mga sabong nagpakita sa abilidad sa mga magmamantala ug pag-atiman sa ilang mga manok.</t>
+          <t>Ang iyang joke bahin sa toyi kay nakapatawa sa tanan.; Ang mga istorya nila bahin sa toyi kay walay kinutuban nga katawa.; Sa dihang nagbinuang siya, nagtoyi lang iyang mga amigo.; Ang ilang duwa nga toyi kay naghatag ug dako nga kalipay.; Ang iyang mga joke kay kasagaran tungkol sa toyi.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>['sabong']</t>
+          <t>['toyi']</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1393,27 +1393,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>taga</t>
+          <t>tuslok baki</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>pag-slash</t>
+          <t>usa ka dula</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ang mga kawatan nga nadakpan kay gi-taga sa mga pulis.; Ang mga prutas gitaga ug maayo aron ma-preserve ug dili dali madaot.; Ang kahoy nga nagtapok sa likod gipangtaga para himoong kahoy pangsiga.; Ang mga kawatan nahadlok kay basin mataga sila sa mga tag-iya sa balay.; Ang mga batan-on nagpraktis ug taga sa kahoy para sa ilang project sa eskwelahan.</t>
+          <t>Ang tuslok baki nga duwa kay paborito sa mga bata sa baryo.; Kada fiesta, magdula mi ug tuslok baki aron maglingaw-lingaw.; Ang tuslok baki nga dula kay naghatag ug dakong excitement sa mga bata.; Ang mga bata nagpraktis sa tuslok baki aron mahimong champion sa dula.; Ang tuslok baki kay usa ka traditional nga dula nga gipasa-pasa sa mga henerasyon.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Ang mga kawatan nga nadakpan kay gi-taga sa mga pulis.; Ang mga prutas gitaga ug maayo aron ma-preserve ug dili dali madaot.; Ang kahoy nga nagtapok sa likod gipangtaga para himoong kahoy pangsiga.; Ang mga kawatan nahadlok kay basin mataga sila sa mga tag-iya sa balay.; Ang mga batan-on nagpraktis ug taga sa kahoy para sa ilang project sa eskwelahan.</t>
+          <t>Ang tuslok baki nga duwa kay paborito sa mga bata sa baryo.; Kada fiesta, magdula mi ug tuslok baki aron maglingaw-lingaw.; Ang tuslok baki nga dula kay naghatag ug dakong excitement sa mga bata.; Ang mga bata nagpraktis sa tuslok baki aron mahimong champion sa dula.; Ang tuslok baki kay usa ka traditional nga dula nga gipasa-pasa sa mga henerasyon.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['tuslok']</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1423,27 +1423,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>taliba</t>
+          <t>ul-ol</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ang mga genital sa babaye</t>
+          <t>sa pag- masturba Mga sinonim: batil</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ang mga pulis nag-taliba sa mga salida aron protektahan ang mga bisita.; Ang mga magtutudlo nag-taliba sa mga estudyante sa ilang field trip.; Ang mga guwardiya nag-taliba sa building adlaw ug gabii.; Ang mga volunteers nag-taliba sa event para malikayan ang mga kagubot.; Ang mga barangay tanod nag-taliba sa ilang mga area kada gabii.</t>
+          <t>Ang iyang buhat kay ul-ol kaayo, wala gyud maghunahuna.; Ayaw pag-ul-ol, kinahanglan naa kay respeto sa uban.; Ang mga ul-ol nga tawo kasagaran dili makuha ang tinuod nga punto.; Ang iyang mga ul-ol nga istorya kay naghatag ug kalibog sa tanan.; Dili maayo nga magsige ka ug ul-ol kay makadaot kini sa imong reputation.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Ang mga pulis nag-taliba sa mga salida aron protektahan ang mga bisita.; Ang mga magtutudlo nag-taliba sa mga estudyante sa ilang field trip.; Ang mga guwardiya nag-taliba sa building adlaw ug gabii.; Ang mga volunteers nag-taliba sa event para malikayan ang mga kagubot.; Ang mga barangay tanod nag-taliba sa ilang mga area kada gabii.</t>
+          <t>Ang iyang buhat kay ul-ol kaayo, wala gyud maghunahuna.; Ayaw pag-ul-ol, kinahanglan naa kay respeto sa uban.; Ang mga ul-ol nga tawo kasagaran dili makuha ang tinuod nga punto.; Ang iyang mga ul-ol nga istorya kay naghatag ug kalibog sa tanan.; Dili maayo nga magsige ka ug ul-ol kay makadaot kini sa imong reputation.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>['taliba']</t>
+          <t>['ul-ol']</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1453,27 +1453,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>tinagoan</t>
+          <t>wala nahilig</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>gitago</t>
+          <t>bisan unsang lalaki nga dili interesado sa mga relasyon nga gipahiunong</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ang mga tinagoan nga yaman sa lumang bahay kay nadiskubrehan.; Ang tinagoan nga lihim ni Juan kay nahibaw-an na sa tanan.; Ang tinagoan nga kwarta kay gikuha sa mga tulisan.; Ang tinagoan nga dokumento kay importante kaayo para sa kaso.; Ang tinagoan nga mga gamit kay kinahanglan pangitaan sa panahon sa inventory.</t>
+          <t>Si Juan wala nahilig sa mga seryosong relasyon, ganahan ra ug fling.; Ang mga wala nahilig sa seryosong relasyon kasagaran ganahan lang ug lingaw-lingaw.; Ang mga wala nahilig mag-settle down kay kasagaran naglibut-libot lang.; Dili kinahanglan pugson ang wala nahilig sa mga seryosong relasyon.; Ang mga wala nahilig kay dili gyud magdugay sa usa ka relasyon.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Ang mga tinagoan nga yaman sa lumang bahay kay nadiskubrehan.; Ang tinagoan nga lihim ni Juan kay nahibaw-an na sa tanan.; Ang tinagoan nga kwarta kay gikuha sa mga tulisan.; Ang tinagoan nga dokumento kay importante kaayo para sa kaso.; Ang tinagoan nga mga gamit kay kinahanglan pangitaan sa panahon sa inventory.</t>
+          <t>Si Juan wala nahilig sa mga seryosong relasyon, ganahan ra ug fling.; Ang mga wala nahilig sa seryosong relasyon kasagaran ganahan lang ug lingaw-lingaw.; Ang mga wala nahilig mag-settle down kay kasagaran naglibut-libot lang.; Dili kinahanglan pugson ang wala nahilig sa mga seryosong relasyon.; Ang mga wala nahilig kay dili gyud magdugay sa usa ka relasyon.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['nahilig']</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1483,27 +1483,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>toyi</t>
+          <t>abot na sa dukot</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>coitus</t>
+          <t>pag-iskrabe sa ubos sa bariles</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ang iyang joke bahin sa toyi kay nakapatawa sa tanan.; Ang mga istorya nila bahin sa toyi kay walay kinutuban nga katawa.; Sa dihang nagbinuang siya, nagtoyi lang iyang mga amigo.; Ang ilang duwa nga toyi kay naghatag ug dako nga kalipay.; Ang iyang mga joke kay kasagaran tungkol sa toyi.</t>
+          <t>Ang iyang mga problema murag abot na sa dukot, grabe na kaayo.; Ang ilang resources abot na sa dukot, kinahanglan na gyud ug tabang.; Ang mga suplay sa tindahan abot na sa dukot, hapit na mahurot.; Sa kadugay nga paghulat, ang iyang pasensya abot na sa dukot.; Ang mga isyu sa opisina abot na sa dukot, kinahanglan na gyud sulbaron.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Ang iyang joke bahin sa toyi kay nakapatawa sa tanan.; Ang mga istorya nila bahin sa toyi kay walay kinutuban nga katawa.; Sa dihang nagbinuang siya, nagtoyi lang iyang mga amigo.; Ang ilang duwa nga toyi kay naghatag ug dako nga kalipay.; Ang iyang mga joke kay kasagaran tungkol sa toyi.</t>
+          <t>Ang iyang mga problema murag abot na sa dukot, grabe na kaayo.; Ang ilang resources abot na sa dukot, kinahanglan na gyud ug tabang.; Ang mga suplay sa tindahan abot na sa dukot, hapit na mahurot.; Sa kadugay nga paghulat, ang iyang pasensya abot na sa dukot.; Ang mga isyu sa opisina abot na sa dukot, kinahanglan na gyud sulbaron.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>['toyi']</t>
+          <t>['abot', 'dukot']</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1513,27 +1513,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>tuslok baki</t>
+          <t>abot sa dalunggan ang ngisi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>usa ka dula</t>
+          <t>nga dili gayod malipay</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ang tuslok baki nga duwa kay paborito sa mga bata sa baryo.; Kada fiesta, magdula mi ug tuslok baki aron maglingaw-lingaw.; Ang tuslok baki nga dula kay naghatag ug dakong excitement sa mga bata.; Ang mga bata nagpraktis sa tuslok baki aron mahimong champion sa dula.; Ang tuslok baki kay usa ka traditional nga dula nga gipasa-pasa sa mga henerasyon.</t>
+          <t>Pagkahuman sa eksam, abot sa dalunggan ang ngisi ni Juan kay nakapasar siya.; Sa dihang nadawat siya sa trabaho, abot sa dalunggan ang ngisi ni Maria.; Ang bata, abot sa dalunggan ang ngisi sa dihang gihatagan ug dako nga regalo.; Abot sa dalunggan ang ngisi sa mga ginikanan sa ilang anak nga nag-graduate.; Sa dihang nagkita sila, abot sa dalunggan ang ngisi ni Pedro ug Ana.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ang tuslok baki nga duwa kay paborito sa mga bata sa baryo.; Kada fiesta, magdula mi ug tuslok baki aron maglingaw-lingaw.; Ang tuslok baki nga dula kay naghatag ug dakong excitement sa mga bata.; Ang mga bata nagpraktis sa tuslok baki aron mahimong champion sa dula.; Ang tuslok baki kay usa ka traditional nga dula nga gipasa-pasa sa mga henerasyon.</t>
+          <t>Pagkahuman sa eksam, abot sa dalunggan ang ngisi ni Juan kay nakapasar siya.; Sa dihang nadawat siya sa trabaho, abot sa dalunggan ang ngisi ni Maria.; Ang bata, abot sa dalunggan ang ngisi sa dihang gihatagan ug dako nga regalo.; Abot sa dalunggan ang ngisi sa mga ginikanan sa ilang anak nga nag-graduate.; Sa dihang nagkita sila, abot sa dalunggan ang ngisi ni Pedro ug Ana.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>['tuslok']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1543,27 +1543,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ul-ol</t>
+          <t>abot sa dunggan ang ngisi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>sa pag- masturba Mga sinonim: batil</t>
+          <t>nga dili gayod malipay</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ang iyang buhat kay ul-ol kaayo, wala gyud maghunahuna.; Ayaw pag-ul-ol, kinahanglan naa kay respeto sa uban.; Ang mga ul-ol nga tawo kasagaran dili makuha ang tinuod nga punto.; Ang iyang mga ul-ol nga istorya kay naghatag ug kalibog sa tanan.; Dili maayo nga magsige ka ug ul-ol kay makadaot kini sa imong reputation.</t>
+          <t>Ang among boss, abot sa dunggan ang ngisi sa dihang nadawat ang dagkong proyekto.; Abot sa dunggan ang ngisi ni Lito pagkakita sa iyang paboritong artista.; Sa dihang gihatagan siya ug award, abot sa dunggan ang ngisi ni Carla.; Ang mga bata, abot sa dunggan ang ngisi sa dihang nagkaon og ice cream.; Abot sa dunggan ang ngisi ni Manang Ines pagkakita sa iyang mga apo.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ang iyang buhat kay ul-ol kaayo, wala gyud maghunahuna.; Ayaw pag-ul-ol, kinahanglan naa kay respeto sa uban.; Ang mga ul-ol nga tawo kasagaran dili makuha ang tinuod nga punto.; Ang iyang mga ul-ol nga istorya kay naghatag ug kalibog sa tanan.; Dili maayo nga magsige ka ug ul-ol kay makadaot kini sa imong reputation.</t>
+          <t>Ang among boss, abot sa dunggan ang ngisi sa dihang nadawat ang dagkong proyekto.; Abot sa dunggan ang ngisi ni Lito pagkakita sa iyang paboritong artista.; Sa dihang gihatagan siya ug award, abot sa dunggan ang ngisi ni Carla.; Ang mga bata, abot sa dunggan ang ngisi sa dihang nagkaon og ice cream.; Abot sa dunggan ang ngisi ni Manang Ines pagkakita sa iyang mga apo.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>['ul-ol']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -1573,27 +1573,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>wala nahilig</t>
+          <t>abot sa pikas bukid</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bisan unsang lalaki nga dili interesado sa mga relasyon nga gipahiunong</t>
+          <t>usa ka tawo nga naghisgot nga makusog</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Si Juan wala nahilig sa mga seryosong relasyon, ganahan ra ug fling.; Ang mga wala nahilig sa seryosong relasyon kasagaran ganahan lang ug lingaw-lingaw.; Ang mga wala nahilig mag-settle down kay kasagaran naglibut-libot lang.; Dili kinahanglan pugson ang wala nahilig sa mga seryosong relasyon.; Ang mga wala nahilig kay dili gyud magdugay sa usa ka relasyon.</t>
+          <t>Ang mga chismosa abot sa pikas bukid ang ilang mga istorya.; Bisan asa pa sila, abot sa pikas bukid ang ilang tingog.; Ang iyang reklamo abot sa pikas bukid, grabe kaayo ug kasaba.; Ang istorya ni Pedro abot sa pikas bukid bisan dili tinuod.; Ang mga away sa ilang pamilya abot sa pikas bukid, daghan nakahibalo.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Si Juan wala nahilig sa mga seryosong relasyon, ganahan ra ug fling.; Ang mga wala nahilig sa seryosong relasyon kasagaran ganahan lang ug lingaw-lingaw.; Ang mga wala nahilig mag-settle down kay kasagaran naglibut-libot lang.; Dili kinahanglan pugson ang wala nahilig sa mga seryosong relasyon.; Ang mga wala nahilig kay dili gyud magdugay sa usa ka relasyon.</t>
+          <t>Ang mga chismosa abot sa pikas bukid ang ilang mga istorya.; Bisan asa pa sila, abot sa pikas bukid ang ilang tingog.; Ang iyang reklamo abot sa pikas bukid, grabe kaayo ug kasaba.; Ang istorya ni Pedro abot sa pikas bukid bisan dili tinuod.; Ang mga away sa ilang pamilya abot sa pikas bukid, daghan nakahibalo.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>['nahilig']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -1603,27 +1603,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>abot na sa dukot</t>
+          <t>agi sa bangag sa dagom</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>pag-iskrabe sa ubos sa bariles</t>
+          <t>pag-antos sa mga kalisdanan sa pagkab-ot sa imong tumong o damgo</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ang iyang mga problema murag abot na sa dukot, grabe na kaayo.; Ang ilang resources abot na sa dukot, kinahanglan na gyud ug tabang.; Ang mga suplay sa tindahan abot na sa dukot, hapit na mahurot.; Sa kadugay nga paghulat, ang iyang pasensya abot na sa dukot.; Ang mga isyu sa opisina abot na sa dukot, kinahanglan na gyud sulbaron.</t>
+          <t>Si Pedro agi sa bangag sa dagom aron lang makapasar sa eksam.; Ang ilang proyekto agi sa bangag sa dagom sa kalisod.; Ang iyang negosyo agi sa bangag sa dagom bago niyag napalambo.; Si Ana agi sa bangag sa dagom sa iyang pag-eskwela ug pagtrabaho.; Ang ilang relasyon agi sa bangag sa dagom sa daghang pagsulay.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ang iyang mga problema murag abot na sa dukot, grabe na kaayo.; Ang ilang resources abot na sa dukot, kinahanglan na gyud ug tabang.; Ang mga suplay sa tindahan abot na sa dukot, hapit na mahurot.; Sa kadugay nga paghulat, ang iyang pasensya abot na sa dukot.; Ang mga isyu sa opisina abot na sa dukot, kinahanglan na gyud sulbaron.</t>
+          <t>Si Pedro agi sa bangag sa dagom aron lang makapasar sa eksam.; Ang ilang proyekto agi sa bangag sa dagom sa kalisod.; Ang iyang negosyo agi sa bangag sa dagom bago niyag napalambo.; Si Ana agi sa bangag sa dagom sa iyang pag-eskwela ug pagtrabaho.; Ang ilang relasyon agi sa bangag sa dagom sa daghang pagsulay.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>['abot', 'dukot']</t>
+          <t>['agi']</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1633,27 +1633,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>abot sa dalunggan ang ngisi</t>
+          <t>awas og palad</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>nga dili gayod malipay</t>
+          <t>• awasan og palad</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Pagkahuman sa eksam, abot sa dalunggan ang ngisi ni Juan kay nakapasar siya.; Sa dihang nadawat siya sa trabaho, abot sa dalunggan ang ngisi ni Maria.; Ang bata, abot sa dalunggan ang ngisi sa dihang gihatagan ug dako nga regalo.; Abot sa dalunggan ang ngisi sa mga ginikanan sa ilang anak nga nag-graduate.; Sa dihang nagkita sila, abot sa dalunggan ang ngisi ni Pedro ug Ana.</t>
+          <t>Si Lito awas og palad, dili gyud makatigom bisan unsa ka dako ang kita.; Ang mga awas og palad kasagaran maglisod sa pagplano sa ilang kaugmaon.; Si Pedro awas og palad, pirmi lang mag-antos kay dili magtigom.; Ang mga awas og palad kasagaran maglisod sa kinabuhi kay dili kabalo magtipid.; Si Ana awas og palad, maong pirmi lang maglisod bisan taas ang sweldo.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pagkahuman sa eksam, abot sa dalunggan ang ngisi ni Juan kay nakapasar siya.; Sa dihang nadawat siya sa trabaho, abot sa dalunggan ang ngisi ni Maria.; Ang bata, abot sa dalunggan ang ngisi sa dihang gihatagan ug dako nga regalo.; Abot sa dalunggan ang ngisi sa mga ginikanan sa ilang anak nga nag-graduate.; Sa dihang nagkita sila, abot sa dalunggan ang ngisi ni Pedro ug Ana.</t>
+          <t>Si Lito awas og palad, dili gyud makatigom bisan unsa ka dako ang kita.; Ang mga awas og palad kasagaran maglisod sa pagplano sa ilang kaugmaon.; Si Pedro awas og palad, pirmi lang mag-antos kay dili magtigom.; Ang mga awas og palad kasagaran maglisod sa kinabuhi kay dili kabalo magtipid.; Si Ana awas og palad, maong pirmi lang maglisod bisan taas ang sweldo.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>['abot']</t>
+          <t>['awas']</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -1663,27 +1663,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>abot sa dunggan ang ngisi</t>
+          <t>bantay pari</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>nga dili gayod malipay</t>
+          <t>aron sa pagbantay sa usa ka tawo/usa ka butang</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ang among boss, abot sa dunggan ang ngisi sa dihang nadawat ang dagkong proyekto.; Abot sa dunggan ang ngisi ni Lito pagkakita sa iyang paboritong artista.; Sa dihang gihatagan siya ug award, abot sa dunggan ang ngisi ni Carla.; Ang mga bata, abot sa dunggan ang ngisi sa dihang nagkaon og ice cream.; Abot sa dunggan ang ngisi ni Manang Ines pagkakita sa iyang mga apo.</t>
+          <t>Si Pedro bantay pari sa ilang balay kay wala'y makalusot nga problema.; Ang mga ginikanan kasagaran bantay pari sa ilang mga anak.; Si Maria bantay pari sa iyang mga kauban sa trabaho aron dili magbinulantoy.; Ang mga bantay pari nga tawo kasagaran mahimong lider sa ilang komunidad.; Ang iyang bantay pari nga kinaiya nakapahimo nga malampuson ang ilang proyekto.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Ang among boss, abot sa dunggan ang ngisi sa dihang nadawat ang dagkong proyekto.; Abot sa dunggan ang ngisi ni Lito pagkakita sa iyang paboritong artista.; Sa dihang gihatagan siya ug award, abot sa dunggan ang ngisi ni Carla.; Ang mga bata, abot sa dunggan ang ngisi sa dihang nagkaon og ice cream.; Abot sa dunggan ang ngisi ni Manang Ines pagkakita sa iyang mga apo.</t>
+          <t>Si Pedro bantay pari sa ilang balay kay wala'y makalusot nga problema.; Ang mga ginikanan kasagaran bantay pari sa ilang mga anak.; Si Maria bantay pari sa iyang mga kauban sa trabaho aron dili magbinulantoy.; Ang mga bantay pari nga tawo kasagaran mahimong lider sa ilang komunidad.; Ang iyang bantay pari nga kinaiya nakapahimo nga malampuson ang ilang proyekto.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>['abot']</t>
+          <t>['bantay']</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -1693,27 +1693,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>abot sa pikas bukid</t>
+          <t>bukhad og palad</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>usa ka tawo nga naghisgot nga makusog</t>
+          <t>mahinatagon Synonyms: manggihatagon</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ang mga chismosa abot sa pikas bukid ang ilang mga istorya.; Bisan asa pa sila, abot sa pikas bukid ang ilang tingog.; Ang iyang reklamo abot sa pikas bukid, grabe kaayo ug kasaba.; Ang istorya ni Pedro abot sa pikas bukid bisan dili tinuod.; Ang mga away sa ilang pamilya abot sa pikas bukid, daghan nakahibalo.</t>
+          <t>Si Ana bukhad og palad, pirmi lang maghatag bisan sa mga dili kaila.; Ang mga tao nga bukhad og palad kasagaran daghan ug mga amigo.; Si Juan bukhad og palad, bisan sa iyang kalisod, pirmi lang magtabang.; Ang iyang pamilya bukhad og palad, maong daghan ang nagmahal kanila.; Ang mga tawo nga bukhad og palad kasagaran masinabtanon ug mapinanggaon.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Ang mga chismosa abot sa pikas bukid ang ilang mga istorya.; Bisan asa pa sila, abot sa pikas bukid ang ilang tingog.; Ang iyang reklamo abot sa pikas bukid, grabe kaayo ug kasaba.; Ang istorya ni Pedro abot sa pikas bukid bisan dili tinuod.; Ang mga away sa ilang pamilya abot sa pikas bukid, daghan nakahibalo.</t>
+          <t>Si Ana bukhad og palad, pirmi lang maghatag bisan sa mga dili kaila.; Ang mga tao nga bukhad og palad kasagaran daghan ug mga amigo.; Si Juan bukhad og palad, bisan sa iyang kalisod, pirmi lang magtabang.; Ang iyang pamilya bukhad og palad, maong daghan ang nagmahal kanila.; Ang mga tawo nga bukhad og palad kasagaran masinabtanon ug mapinanggaon.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>['abot']</t>
+          <t>['bukhad']</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -1723,27 +1723,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>agas og palad</t>
+          <t>buotan ra og matulog</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>usa ka manggugol</t>
+          <t>malinong</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Si Juan agas og palad, walay kwarta magdugay sa iyang kamot.; Bisan unsa kadako ang sweldo, si Ana agas og palad, dili makatigom.; Ang mga tawo nga agas og palad kasagaran dili makatigom ug insakto.; Ang iyang kinaiya nga agas og palad nagdala ug kalisod sa iyang kinabuhi.; Kinahanglan ka mag-amping sa imong kwarta, dili ka mag-agas og palad.</t>
+          <t>Si Pedro buotan ra og matulog, kay pirmi lang magbinuang sa klase.; Ang iyang anak buotan ra og matulog, kay pirmi lang mangaway sa mga silingan.; Si Juan buotan ra og matulog, kay dili gyud mahimutang kung magmata.; Ang mga bata nga buotan ra og matulog kasagaran magdala ug kasamok sa balay.; Si Ana buotan ra og matulog, kay pirmi lang magbinuang sa iyang mga igsoon.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Si Juan agas og palad, walay kwarta magdugay sa iyang kamot.; Bisan unsa kadako ang sweldo, si Ana agas og palad, dili makatigom.; Ang mga tawo nga agas og palad kasagaran dili makatigom ug insakto.; Ang iyang kinaiya nga agas og palad nagdala ug kalisod sa iyang kinabuhi.; Kinahanglan ka mag-amping sa imong kwarta, dili ka mag-agas og palad.</t>
+          <t>Si Pedro buotan ra og matulog, kay pirmi lang magbinuang sa klase.; Ang iyang anak buotan ra og matulog, kay pirmi lang mangaway sa mga silingan.; Si Juan buotan ra og matulog, kay dili gyud mahimutang kung magmata.; Ang mga bata nga buotan ra og matulog kasagaran magdala ug kasamok sa balay.; Si Ana buotan ra og matulog, kay pirmi lang magbinuang sa iyang mga igsoon.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['matulog']</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -1753,27 +1753,27 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>agi sa bangag sa dagom</t>
+          <t>dili madala og rosaryo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>pag-antos sa mga kalisdanan sa pagkab-ot sa imong tumong o damgo</t>
+          <t>usa ka hingpit nga walay paglaom nga kahimtang</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Si Pedro agi sa bangag sa dagom aron lang makapasar sa eksam.; Ang ilang proyekto agi sa bangag sa dagom sa kalisod.; Ang iyang negosyo agi sa bangag sa dagom bago niyag napalambo.; Si Ana agi sa bangag sa dagom sa iyang pag-eskwela ug pagtrabaho.; Ang ilang relasyon agi sa bangag sa dagom sa daghang pagsulay.</t>
+          <t>Ang iyang problema dili madala og rosaryo, kinahanglan gyud ug aksyon.; Si Pedro nag-atubang sa mga pagsulay nga dili madala og rosaryo.; Ang mga tawo nga naa sa kalisod kasagaran dili madala og rosaryo ilang mga problema.; Si Maria nag-antos sa mga butang nga dili madala og rosaryo.; Ang ilang sitwasyon sa negosyo dili madala og rosaryo, kinahanglan ug solusyon.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Si Pedro agi sa bangag sa dagom aron lang makapasar sa eksam.; Ang ilang proyekto agi sa bangag sa dagom sa kalisod.; Ang iyang negosyo agi sa bangag sa dagom bago niyag napalambo.; Si Ana agi sa bangag sa dagom sa iyang pag-eskwela ug pagtrabaho.; Ang ilang relasyon agi sa bangag sa dagom sa daghang pagsulay.</t>
+          <t>Ang iyang problema dili madala og rosaryo, kinahanglan gyud ug aksyon.; Si Pedro nag-atubang sa mga pagsulay nga dili madala og rosaryo.; Ang mga tawo nga naa sa kalisod kasagaran dili madala og rosaryo ilang mga problema.; Si Maria nag-antos sa mga butang nga dili madala og rosaryo.; Ang ilang sitwasyon sa negosyo dili madala og rosaryo, kinahanglan ug solusyon.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>['agi']</t>
+          <t>['madala']</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -1783,27 +1783,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>awas og palad</t>
+          <t>dili makaon og iro</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>• awasan og palad</t>
+          <t>makalilisang</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Si Lito awas og palad, dili gyud makatigom bisan unsa ka dako ang kita.; Ang mga awas og palad kasagaran maglisod sa pagplano sa ilang kaugmaon.; Si Pedro awas og palad, pirmi lang mag-antos kay dili magtigom.; Ang mga awas og palad kasagaran maglisod sa kinabuhi kay dili kabalo magtipid.; Si Ana awas og palad, maong pirmi lang maglisod bisan taas ang sweldo.</t>
+          <t>Ang iyang batasan dili makaon og iro, maong walay ganahan makighangyo niya.; Si Juan dili makaon og iro, kay pirmi lang maghimo ug gubot.; Ang mga tawo nga dili makaon og iro kasagaran walay respeto sa uban.; Si Maria dili makaon og iro, bisan unsa pa nga istorya, walay muuban niya.; Ang iyang batasan kay dili makaon og iro, maong nag-inusara siya pirmi.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Si Lito awas og palad, dili gyud makatigom bisan unsa ka dako ang kita.; Ang mga awas og palad kasagaran maglisod sa pagplano sa ilang kaugmaon.; Si Pedro awas og palad, pirmi lang mag-antos kay dili magtigom.; Ang mga awas og palad kasagaran maglisod sa kinabuhi kay dili kabalo magtipid.; Si Ana awas og palad, maong pirmi lang maglisod bisan taas ang sweldo.</t>
+          <t>Ang iyang batasan dili makaon og iro, maong walay ganahan makighangyo niya.; Si Juan dili makaon og iro, kay pirmi lang maghimo ug gubot.; Ang mga tawo nga dili makaon og iro kasagaran walay respeto sa uban.; Si Maria dili makaon og iro, bisan unsa pa nga istorya, walay muuban niya.; Ang iyang batasan kay dili makaon og iro, maong nag-inusara siya pirmi.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>['awas']</t>
+          <t>['makaon']</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -1813,27 +1813,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>bantay pari</t>
+          <t>dugay pay manguros</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>aron sa pagbantay sa usa ka tawo/usa ka butang</t>
+          <t>usa ka piraso sa cake</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Si Pedro bantay pari sa ilang balay kay wala'y makalusot nga problema.; Ang mga ginikanan kasagaran bantay pari sa ilang mga anak.; Si Maria bantay pari sa iyang mga kauban sa trabaho aron dili magbinulantoy.; Ang mga bantay pari nga tawo kasagaran mahimong lider sa ilang komunidad.; Ang iyang bantay pari nga kinaiya nakapahimo nga malampuson ang ilang proyekto.</t>
+          <t>Ang iyang trabaho dugay pay manguros, pirmi lang maghinay-hinay.; Si Juan dugay pay manguros kung magtrabaho sa opisina.; Ang mga tawo nga dugay pay manguros kasagaran maglisod sa ilang mga deadline.; Si Pedro dugay pay manguros, bisan unsa nga butang, hinay kaayo mahuman.; Ang iyang proyekto dugay pay manguros, walay klaro nga mahuman.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Si Pedro bantay pari sa ilang balay kay wala'y makalusot nga problema.; Ang mga ginikanan kasagaran bantay pari sa ilang mga anak.; Si Maria bantay pari sa iyang mga kauban sa trabaho aron dili magbinulantoy.; Ang mga bantay pari nga tawo kasagaran mahimong lider sa ilang komunidad.; Ang iyang bantay pari nga kinaiya nakapahimo nga malampuson ang ilang proyekto.</t>
+          <t>Ang iyang trabaho dugay pay manguros, pirmi lang maghinay-hinay.; Si Juan dugay pay manguros kung magtrabaho sa opisina.; Ang mga tawo nga dugay pay manguros kasagaran maglisod sa ilang mga deadline.; Si Pedro dugay pay manguros, bisan unsa nga butang, hinay kaayo mahuman.; Ang iyang proyekto dugay pay manguros, walay klaro nga mahuman.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>['bantay']</t>
+          <t>['manguros']</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -1843,27 +1843,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>bukhad og palad</t>
+          <t>dula og panit</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>mahinatagon Synonyms: manggihatagon</t>
+          <t>sa pag- masturba</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Si Ana bukhad og palad, pirmi lang maghatag bisan sa mga dili kaila.; Ang mga tao nga bukhad og palad kasagaran daghan ug mga amigo.; Si Juan bukhad og palad, bisan sa iyang kalisod, pirmi lang magtabang.; Ang iyang pamilya bukhad og palad, maong daghan ang nagmahal kanila.; Ang mga tawo nga bukhad og palad kasagaran masinabtanon ug mapinanggaon.</t>
+          <t>Si Pedro pirmi lang mag-dula og panit, bisan walay buhaton nga maayo.; Ang mga bata nga dula og panit kasagaran wala’y klaro nga padulngan.; Si Juan dula og panit, pirmi lang magtambay ug magbuot-buot.; Ang iyang barkada kay dula og panit, bisan unsa na lang nga kalipay ang gihimo.; Si Maria nagbuot-buot kay gusto siya magdula og panit pirmi.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Si Ana bukhad og palad, pirmi lang maghatag bisan sa mga dili kaila.; Ang mga tao nga bukhad og palad kasagaran daghan ug mga amigo.; Si Juan bukhad og palad, bisan sa iyang kalisod, pirmi lang magtabang.; Ang iyang pamilya bukhad og palad, maong daghan ang nagmahal kanila.; Ang mga tawo nga bukhad og palad kasagaran masinabtanon ug mapinanggaon.</t>
+          <t>Si Pedro pirmi lang mag-dula og panit, bisan walay buhaton nga maayo.; Ang mga bata nga dula og panit kasagaran wala’y klaro nga padulngan.; Si Juan dula og panit, pirmi lang magtambay ug magbuot-buot.; Ang iyang barkada kay dula og panit, bisan unsa na lang nga kalipay ang gihimo.; Si Maria nagbuot-buot kay gusto siya magdula og panit pirmi.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>['bukhad']</t>
+          <t>['dula']</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -1873,27 +1873,27 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>buotan ra og matulog</t>
+          <t>duwa og panit</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>malinong</t>
+          <t>sa pag- masturba</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Si Pedro buotan ra og matulog, kay pirmi lang magbinuang sa klase.; Ang iyang anak buotan ra og matulog, kay pirmi lang mangaway sa mga silingan.; Si Juan buotan ra og matulog, kay dili gyud mahimutang kung magmata.; Ang mga bata nga buotan ra og matulog kasagaran magdala ug kasamok sa balay.; Si Ana buotan ra og matulog, kay pirmi lang magbinuang sa iyang mga igsoon.</t>
+          <t>Si Juan pirmi lang mag-duwa og panit sa iyang kwarto.; Ang iyang mga kauban sa trabaho pirmi lang magbinuang ug magduwa og panit.; Si Pedro walay laing gihimo kundi magduwa og panit pirmi.; Ang mga bata nga nagdula sa internet pirmi lang magduwa og panit.; Si Maria naglagot kay si Juan pirmi lang magduwa og panit bisan kinahanglanon siya.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Si Pedro buotan ra og matulog, kay pirmi lang magbinuang sa klase.; Ang iyang anak buotan ra og matulog, kay pirmi lang mangaway sa mga silingan.; Si Juan buotan ra og matulog, kay dili gyud mahimutang kung magmata.; Ang mga bata nga buotan ra og matulog kasagaran magdala ug kasamok sa balay.; Si Ana buotan ra og matulog, kay pirmi lang magbinuang sa iyang mga igsoon.</t>
+          <t>Si Juan pirmi lang mag-duwa og panit sa iyang kwarto.; Ang iyang mga kauban sa trabaho pirmi lang magbinuang ug magduwa og panit.; Si Pedro walay laing gihimo kundi magduwa og panit pirmi.; Ang mga bata nga nagdula sa internet pirmi lang magduwa og panit.; Si Maria naglagot kay si Juan pirmi lang magduwa og panit bisan kinahanglanon siya.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>['matulog']</t>
+          <t>['duwa']</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -1903,27 +1903,27 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dila ray way labod</t>
+          <t>gadalag ulan</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>grabe nga nasakit</t>
+          <t>usa ka lalaki nga homoseksual</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Si Juan dila ray way labod, kay pirmi lang magsige ug kaon bisan sakit na iyang tiyan.; Ang mga bata dila ray way labod kung naa sa handaan.; Si Pedro dila ray way labod, bisan unsa na lang ang kaon nga dili na healthy.; Ang mga tawo nga dila ray way labod kasagaran maglisod sa ilang lawas.; Si Maria dila ray way labod, pirmi lang magpataka ug kaon sa mga events.</t>
+          <t>Si Juan kay gadalag ulan, maong daghan ang naglikay niya.; Ang iyang amigo gadalag ulan, maong dili siya ganahan kauban.; Si Pedro gadalag ulan, bisan unsa pa nga sitwasyon.; Ang mga tawo nga gadalag ulan kasagaran naglisod sa pagdawat sa uban.; Si Maria gadalag ulan, maong pirmi siya nag-inusara.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Si Juan dila ray way labod, kay pirmi lang magsige ug kaon bisan sakit na iyang tiyan.; Ang mga bata dila ray way labod kung naa sa handaan.; Si Pedro dila ray way labod, bisan unsa na lang ang kaon nga dili na healthy.; Ang mga tawo nga dila ray way labod kasagaran maglisod sa ilang lawas.; Si Maria dila ray way labod, pirmi lang magpataka ug kaon sa mga events.</t>
+          <t>Si Juan kay gadalag ulan, maong daghan ang naglikay niya.; Ang iyang amigo gadalag ulan, maong dili siya ganahan kauban.; Si Pedro gadalag ulan, bisan unsa pa nga sitwasyon.; Ang mga tawo nga gadalag ulan kasagaran naglisod sa pagdawat sa uban.; Si Maria gadalag ulan, maong pirmi siya nag-inusara.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['nagdala']</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -1933,27 +1933,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>dili madala og rosaryo</t>
+          <t>gadalag uwan</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>usa ka hingpit nga walay paglaom nga kahimtang</t>
+          <t>usa ka lalaki nga homoseksual</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ang iyang problema dili madala og rosaryo, kinahanglan gyud ug aksyon.; Si Pedro nag-atubang sa mga pagsulay nga dili madala og rosaryo.; Ang mga tawo nga naa sa kalisod kasagaran dili madala og rosaryo ilang mga problema.; Si Maria nag-antos sa mga butang nga dili madala og rosaryo.; Ang ilang sitwasyon sa negosyo dili madala og rosaryo, kinahanglan ug solusyon.</t>
+          <t>Si Lito gadalag uwan, pero gihigugma gihapon sa iyang pamilya.; Ang iyang silingan gadalag uwan, pero respetado gihapon sa ilang lugar.; Si Juan gadalag uwan, bisan unsa pa nga istorya, wala magpailalom.; Ang mga tao nga gadalag uwan kasagaran adunay mga pagsulay sa kinabuhi.; Si Maria gadalag uwan, pero walay mopauli sa iyang pagkatawo.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Ang iyang problema dili madala og rosaryo, kinahanglan gyud ug aksyon.; Si Pedro nag-atubang sa mga pagsulay nga dili madala og rosaryo.; Ang mga tawo nga naa sa kalisod kasagaran dili madala og rosaryo ilang mga problema.; Si Maria nag-antos sa mga butang nga dili madala og rosaryo.; Ang ilang sitwasyon sa negosyo dili madala og rosaryo, kinahanglan ug solusyon.</t>
+          <t>Si Lito gadalag uwan, pero gihigugma gihapon sa iyang pamilya.; Ang iyang silingan gadalag uwan, pero respetado gihapon sa ilang lugar.; Si Juan gadalag uwan, bisan unsa pa nga istorya, wala magpailalom.; Ang mga tao nga gadalag uwan kasagaran adunay mga pagsulay sa kinabuhi.; Si Maria gadalag uwan, pero walay mopauli sa iyang pagkatawo.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>['madala']</t>
+          <t>['nagdala']</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -1963,27 +1963,27 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>dili makaon og iro</t>
+          <t>gi-indian</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>makalilisang</t>
+          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ang iyang batasan dili makaon og iro, maong walay ganahan makighangyo niya.; Si Juan dili makaon og iro, kay pirmi lang maghimo ug gubot.; Ang mga tawo nga dili makaon og iro kasagaran walay respeto sa uban.; Si Maria dili makaon og iro, bisan unsa pa nga istorya, walay muuban niya.; Ang iyang batasan kay dili makaon og iro, maong nag-inusara siya pirmi.</t>
+          <t>Si Pedro gi-indian sa iyang uyab sa ilang sabot nga date.; Ang mga estudyante na gi-indian sa ilang maestra sa klase karon.; Si Maria nasuko kay gi-indian siya sa iyang amigo.; Ang iyang kauban sa trabaho gi-indian siya sa ilang meeting.; Si Juan gi-indian sa iyang kliyente sa ilang appointment.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Ang iyang batasan dili makaon og iro, maong walay ganahan makighangyo niya.; Si Juan dili makaon og iro, kay pirmi lang maghimo ug gubot.; Ang mga tawo nga dili makaon og iro kasagaran walay respeto sa uban.; Si Maria dili makaon og iro, bisan unsa pa nga istorya, walay muuban niya.; Ang iyang batasan kay dili makaon og iro, maong nag-inusara siya pirmi.</t>
+          <t>Si Pedro gi-indian sa iyang uyab sa ilang sabot nga date.; Ang mga estudyante na gi-indian sa ilang maestra sa klase karon.; Si Maria nasuko kay gi-indian siya sa iyang amigo.; Ang iyang kauban sa trabaho gi-indian siya sa ilang meeting.; Si Juan gi-indian sa iyang kliyente sa ilang appointment.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>['makaon']</t>
+          <t>['gi-indian']</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -1993,27 +1993,27 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>dobleg suwab ang dila</t>
+          <t>gibati og kaanyag</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>naggamit ug mapintas o makadaot nga mga pulong</t>
+          <t>prima donna</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Si Pedro dobleg suwab ang dila, pirmi lang mangaway bisan walay hinungdan.; Ang iyang amiga dobleg suwab ang dila, pirmi lang maglagot ug mangaway.; Si Juan dobleg suwab ang dila, bisan gamay nga butang, dakuon gyud.; Ang mga tawo nga dobleg suwab ang dila kasagaran magbuhat ug samok sa grupo.; Si Maria dobleg suwab ang dila, maong walay ganahan makig-istorya niya.</t>
+          <t>Si Ana gibati og kaanyag, maong pirmi siya nagbuot-buot.; Ang mga tawo nga gibati og kaanyag kasagaran magdala ug samok sa grupo.; Si Maria gibati og kaanyag, bisan unsa nga sugo, dili gyud mutuman.; Ang iyang amiga gibati og kaanyag, maong pirmi mag-away sa iyang bana.; Si Pedro gibati og kaanyag, maong pirmi magbuot sa ilang opisina.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Si Pedro dobleg suwab ang dila, pirmi lang mangaway bisan walay hinungdan.; Ang iyang amiga dobleg suwab ang dila, pirmi lang maglagot ug mangaway.; Si Juan dobleg suwab ang dila, bisan gamay nga butang, dakuon gyud.; Ang mga tawo nga dobleg suwab ang dila kasagaran magbuhat ug samok sa grupo.; Si Maria dobleg suwab ang dila, maong walay ganahan makig-istorya niya.</t>
+          <t>Si Ana gibati og kaanyag, maong pirmi siya nagbuot-buot.; Ang mga tawo nga gibati og kaanyag kasagaran magdala ug samok sa grupo.; Si Maria gibati og kaanyag, bisan unsa nga sugo, dili gyud mutuman.; Ang iyang amiga gibati og kaanyag, maong pirmi mag-away sa iyang bana.; Si Pedro gibati og kaanyag, maong pirmi magbuot sa ilang opisina.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['gibati']</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2023,27 +2023,27 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>dugay pay manguros</t>
+          <t>gigukod sa plansa</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>usa ka piraso sa cake</t>
+          <t>ang usa ka tawo nga nagsul-ob ug mga sinina</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Ang iyang trabaho dugay pay manguros, pirmi lang maghinay-hinay.; Si Juan dugay pay manguros kung magtrabaho sa opisina.; Ang mga tawo nga dugay pay manguros kasagaran maglisod sa ilang mga deadline.; Si Pedro dugay pay manguros, bisan unsa nga butang, hinay kaayo mahuman.; Ang iyang proyekto dugay pay manguros, walay klaro nga mahuman.</t>
+          <t>Si Juan pirmi lang gigukod sa plansa, kay dili siya ganahan magplantsa.; Ang iyang sinina pirmi lang gigukod sa plansa, maong bati tan-awon.; Si Pedro pirmi lang gigukod sa plansa, bisan unsa nga sinina dili mahimutang.; Ang mga tawo nga gigukod sa plansa kasagaran dili mag-atiman sa ilang kaugalingon.; Si Maria gigukod sa plansa, bisan unsa nga okasyon, dili gyud magplantsa.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Ang iyang trabaho dugay pay manguros, pirmi lang maghinay-hinay.; Si Juan dugay pay manguros kung magtrabaho sa opisina.; Ang mga tawo nga dugay pay manguros kasagaran maglisod sa ilang mga deadline.; Si Pedro dugay pay manguros, bisan unsa nga butang, hinay kaayo mahuman.; Ang iyang proyekto dugay pay manguros, walay klaro nga mahuman.</t>
+          <t>Si Juan pirmi lang gigukod sa plansa, kay dili siya ganahan magplantsa.; Ang iyang sinina pirmi lang gigukod sa plansa, maong bati tan-awon.; Si Pedro pirmi lang gigukod sa plansa, bisan unsa nga sinina dili mahimutang.; Ang mga tawo nga gigukod sa plansa kasagaran dili mag-atiman sa ilang kaugalingon.; Si Maria gigukod sa plansa, bisan unsa nga okasyon, dili gyud magplantsa.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>['manguros']</t>
+          <t>['gigukod']</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -2053,27 +2053,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>dula og panit</t>
+          <t>gigukod sa sudlay</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>nga walay buhok</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang mag-dula og panit, bisan walay buhaton nga maayo.; Ang mga bata nga dula og panit kasagaran wala’y klaro nga padulngan.; Si Juan dula og panit, pirmi lang magtambay ug magbuot-buot.; Ang iyang barkada kay dula og panit, bisan unsa na lang nga kalipay ang gihimo.; Si Maria nagbuot-buot kay gusto siya magdula og panit pirmi.</t>
+          <t>Si Ana pirmi lang gigukod sa sudlay, kay dili siya ganahan mag-comb sa iyang buhok.; Ang iyang buhok pirmi lang gigukod sa sudlay, maong bati kaayo tan-awon.; Si Pedro pirmi lang gigukod sa sudlay, bisan unsa nga event, dili mag-comb.; Ang mga tawo nga gigukod sa sudlay kasagaran dili mag-atiman sa ilang buhok.; Si Juan gigukod sa sudlay, bisan unsa nga party, dili gyud mag-comb.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang mag-dula og panit, bisan walay buhaton nga maayo.; Ang mga bata nga dula og panit kasagaran wala’y klaro nga padulngan.; Si Juan dula og panit, pirmi lang magtambay ug magbuot-buot.; Ang iyang barkada kay dula og panit, bisan unsa na lang nga kalipay ang gihimo.; Si Maria nagbuot-buot kay gusto siya magdula og panit pirmi.</t>
+          <t>Si Ana pirmi lang gigukod sa sudlay, kay dili siya ganahan mag-comb sa iyang buhok.; Ang iyang buhok pirmi lang gigukod sa sudlay, maong bati kaayo tan-awon.; Si Pedro pirmi lang gigukod sa sudlay, bisan unsa nga event, dili mag-comb.; Ang mga tawo nga gigukod sa sudlay kasagaran dili mag-atiman sa ilang buhok.; Si Juan gigukod sa sudlay, bisan unsa nga party, dili gyud mag-comb.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>['dula']</t>
+          <t>['gigukod']</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -2083,27 +2083,27 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>duwa og panit</t>
+          <t>gilawog sa tirong</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>sa pagbutang sa peligro sa usa ka tawo, ilabina</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang mag-duwa og panit sa iyang kwarto.; Ang iyang mga kauban sa trabaho pirmi lang magbinuang ug magduwa og panit.; Si Pedro walay laing gihimo kundi magduwa og panit pirmi.; Ang mga bata nga nagdula sa internet pirmi lang magduwa og panit.; Si Maria naglagot kay si Juan pirmi lang magduwa og panit bisan kinahanglanon siya.</t>
+          <t>Si Pedro gilawog sa tirong sa iyang kauban, maong nasakpan sa ilang boss.; Ang iyang amiga gilawog sa tirong, maong nahimong scapegoat sa problema.; Si Maria gilawog sa tirong sa iyang mga kauban sa trabaho.; Ang mga tawo nga gilawog sa tirong kasagaran mag-antos sa mga consequences.; Si Juan gilawog sa tirong, bisan wala siya naghimo sa sayop.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang mag-duwa og panit sa iyang kwarto.; Ang iyang mga kauban sa trabaho pirmi lang magbinuang ug magduwa og panit.; Si Pedro walay laing gihimo kundi magduwa og panit pirmi.; Ang mga bata nga nagdula sa internet pirmi lang magduwa og panit.; Si Maria naglagot kay si Juan pirmi lang magduwa og panit bisan kinahanglanon siya.</t>
+          <t>Si Pedro gilawog sa tirong sa iyang kauban, maong nasakpan sa ilang boss.; Ang iyang amiga gilawog sa tirong, maong nahimong scapegoat sa problema.; Si Maria gilawog sa tirong sa iyang mga kauban sa trabaho.; Ang mga tawo nga gilawog sa tirong kasagaran mag-antos sa mga consequences.; Si Juan gilawog sa tirong, bisan wala siya naghimo sa sayop.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>['duwa']</t>
+          <t>['gilawog']</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -2113,27 +2113,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>gadalag ulan</t>
+          <t>giluto sa kaugalingong mantika</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>usa ka lalaki nga homoseksual</t>
+          <t>sa pag-ukit sa kaugalingong lubnganan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Si Juan kay gadalag ulan, maong daghan ang naglikay niya.; Ang iyang amigo gadalag ulan, maong dili siya ganahan kauban.; Si Pedro gadalag ulan, bisan unsa pa nga sitwasyon.; Ang mga tawo nga gadalag ulan kasagaran naglisod sa pagdawat sa uban.; Si Maria gadalag ulan, maong pirmi siya nag-inusara.</t>
+          <t>Si Pedro giluto sa kaugalingong mantika sa iyang mga sala.; Ang iyang kauban giluto sa kaugalingong mantika tungod sa iyang binuhatan.; Si Maria giluto sa kaugalingong mantika sa iyang mga desisyon.; Ang mga tawo nga magbuhat ug dautan kasagaran giluto sa kaugalingong mantika.; Si Juan giluto sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Si Juan kay gadalag ulan, maong daghan ang naglikay niya.; Ang iyang amigo gadalag ulan, maong dili siya ganahan kauban.; Si Pedro gadalag ulan, bisan unsa pa nga sitwasyon.; Ang mga tawo nga gadalag ulan kasagaran naglisod sa pagdawat sa uban.; Si Maria gadalag ulan, maong pirmi siya nag-inusara.</t>
+          <t>Si Pedro giluto sa kaugalingong mantika sa iyang mga sala.; Ang iyang kauban giluto sa kaugalingong mantika tungod sa iyang binuhatan.; Si Maria giluto sa kaugalingong mantika sa iyang mga desisyon.; Ang mga tawo nga magbuhat ug dautan kasagaran giluto sa kaugalingong mantika.; Si Juan giluto sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>['nagdala']</t>
+          <t>['giluto']</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2143,27 +2143,27 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>gadalag uwan</t>
+          <t>giprito sa kaugalingong mantika</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>usa ka lalaki nga homoseksual</t>
+          <t>Alternatibo nga porma sa giluto sa kaugalingong mantika</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Si Lito gadalag uwan, pero gihigugma gihapon sa iyang pamilya.; Ang iyang silingan gadalag uwan, pero respetado gihapon sa ilang lugar.; Si Juan gadalag uwan, bisan unsa pa nga istorya, wala magpailalom.; Ang mga tao nga gadalag uwan kasagaran adunay mga pagsulay sa kinabuhi.; Si Maria gadalag uwan, pero walay mopauli sa iyang pagkatawo.</t>
+          <t>Si Ana giprito sa kaugalingong mantika tungod sa iyang mga aksyon.; Ang mga tao nga magbuhat ug dautan kasagaran giprito sa kaugalingong mantika.; Si Pedro giprito sa kaugalingong mantika sa iyang mga desisyon.; Ang iyang kauban giprito sa kaugalingong mantika sa iyang mga sala.; Si Juan giprito sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Si Lito gadalag uwan, pero gihigugma gihapon sa iyang pamilya.; Ang iyang silingan gadalag uwan, pero respetado gihapon sa ilang lugar.; Si Juan gadalag uwan, bisan unsa pa nga istorya, wala magpailalom.; Ang mga tao nga gadalag uwan kasagaran adunay mga pagsulay sa kinabuhi.; Si Maria gadalag uwan, pero walay mopauli sa iyang pagkatawo.</t>
+          <t>Si Ana giprito sa kaugalingong mantika tungod sa iyang mga aksyon.; Ang mga tao nga magbuhat ug dautan kasagaran giprito sa kaugalingong mantika.; Si Pedro giprito sa kaugalingong mantika sa iyang mga desisyon.; Ang iyang kauban giprito sa kaugalingong mantika sa iyang mga sala.; Si Juan giprito sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>['nagdala']</t>
+          <t>['giprito']</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -2173,27 +2173,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>gi-indian</t>
+          <t>gisulod sa bulsa</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
+          <t>sa paglimbong</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Si Pedro gi-indian sa iyang uyab sa ilang sabot nga date.; Ang mga estudyante na gi-indian sa ilang maestra sa klase karon.; Si Maria nasuko kay gi-indian siya sa iyang amigo.; Ang iyang kauban sa trabaho gi-indian siya sa ilang meeting.; Si Juan gi-indian sa iyang kliyente sa ilang appointment.</t>
+          <t>Si Juan gisulod sa bulsa sa iyang kauban, maong nawala ang iyang kwarta.; Ang iyang kauban gisulod sa bulsa sa ilang boss, maong napromote siya.; Si Pedro gisulod sa bulsa sa mga sindikato, maong naglisod siya karon.; Ang mga tawo nga masaligan kasagaran dili gisulod sa bulsa.; Si Maria gisulod sa bulsa, maong nag-antos siya sa iyang mga desisyon.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Si Pedro gi-indian sa iyang uyab sa ilang sabot nga date.; Ang mga estudyante na gi-indian sa ilang maestra sa klase karon.; Si Maria nasuko kay gi-indian siya sa iyang amigo.; Ang iyang kauban sa trabaho gi-indian siya sa ilang meeting.; Si Juan gi-indian sa iyang kliyente sa ilang appointment.</t>
+          <t>Si Juan gisulod sa bulsa sa iyang kauban, maong nawala ang iyang kwarta.; Ang iyang kauban gisulod sa bulsa sa ilang boss, maong napromote siya.; Si Pedro gisulod sa bulsa sa mga sindikato, maong naglisod siya karon.; Ang mga tawo nga masaligan kasagaran dili gisulod sa bulsa.; Si Maria gisulod sa bulsa, maong nag-antos siya sa iyang mga desisyon.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>['gi-indian']</t>
+          <t>['gisulod']</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -2203,27 +2203,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>gibati og kaanyag</t>
+          <t>gwapa kon magtalikod</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>prima donna</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Si Ana gibati og kaanyag, maong pirmi siya nagbuot-buot.; Ang mga tawo nga gibati og kaanyag kasagaran magdala ug samok sa grupo.; Si Maria gibati og kaanyag, bisan unsa nga sugo, dili gyud mutuman.; Ang iyang amiga gibati og kaanyag, maong pirmi mag-away sa iyang bana.; Si Pedro gibati og kaanyag, maong pirmi magbuot sa ilang opisina.</t>
+          <t>Si Ana gwapa kon magtalikod, pero pagtan-aw sa iyang nawong, lahi gyud diay.; Ang iyang kauban sa trabaho gwapa kon magtalikod, pero pag-atubang, dili na diay.; Si Maria pirmi lang ginatawgon nga gwapa kon magtalikod sa iyang mga amigo.; Ang mga tao nga gwapa kon magtalikod kasagaran maulaw kung mag-atubang.; Si Pedro pirmi lang magbuot-buot ug sulti nga gwapa kon magtalikod.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Si Ana gibati og kaanyag, maong pirmi siya nagbuot-buot.; Ang mga tawo nga gibati og kaanyag kasagaran magdala ug samok sa grupo.; Si Maria gibati og kaanyag, bisan unsa nga sugo, dili gyud mutuman.; Ang iyang amiga gibati og kaanyag, maong pirmi mag-away sa iyang bana.; Si Pedro gibati og kaanyag, maong pirmi magbuot sa ilang opisina.</t>
+          <t>Si Ana gwapa kon magtalikod, pero pagtan-aw sa iyang nawong, lahi gyud diay.; Ang iyang kauban sa trabaho gwapa kon magtalikod, pero pag-atubang, dili na diay.; Si Maria pirmi lang ginatawgon nga gwapa kon magtalikod sa iyang mga amigo.; Ang mga tao nga gwapa kon magtalikod kasagaran maulaw kung mag-atubang.; Si Pedro pirmi lang magbuot-buot ug sulti nga gwapa kon magtalikod.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>['gibati']</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -2233,27 +2233,27 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>gigukod sa plansa</t>
+          <t>gwapo kon magtalikod</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga nagsul-ob ug mga sinina</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang gigukod sa plansa, kay dili siya ganahan magplantsa.; Ang iyang sinina pirmi lang gigukod sa plansa, maong bati tan-awon.; Si Pedro pirmi lang gigukod sa plansa, bisan unsa nga sinina dili mahimutang.; Ang mga tawo nga gigukod sa plansa kasagaran dili mag-atiman sa ilang kaugalingon.; Si Maria gigukod sa plansa, bisan unsa nga okasyon, dili gyud magplantsa.</t>
+          <t>Si Juan gwapo kon magtalikod, pero dili na kaayo pag-atubang.; Ang iyang amigo gwapo kon magtalikod, pero bati diay pagtan-aw sa iyang nawong.; Si Pedro pirmi lang ginatawgon nga gwapo kon magtalikod sa iyang barkada.; Ang mga tao nga gwapo kon magtalikod kasagaran dili magdugay sa ilang relasyon.; Si Maria pirmi lang magbuot-buot ug sulti nga gwapo kon magtalikod.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang gigukod sa plansa, kay dili siya ganahan magplantsa.; Ang iyang sinina pirmi lang gigukod sa plansa, maong bati tan-awon.; Si Pedro pirmi lang gigukod sa plansa, bisan unsa nga sinina dili mahimutang.; Ang mga tawo nga gigukod sa plansa kasagaran dili mag-atiman sa ilang kaugalingon.; Si Maria gigukod sa plansa, bisan unsa nga okasyon, dili gyud magplantsa.</t>
+          <t>Si Juan gwapo kon magtalikod, pero dili na kaayo pag-atubang.; Ang iyang amigo gwapo kon magtalikod, pero bati diay pagtan-aw sa iyang nawong.; Si Pedro pirmi lang ginatawgon nga gwapo kon magtalikod sa iyang barkada.; Ang mga tao nga gwapo kon magtalikod kasagaran dili magdugay sa ilang relasyon.; Si Maria pirmi lang magbuot-buot ug sulti nga gwapo kon magtalikod.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>['gigukod']</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -2263,27 +2263,27 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>gigukod sa sudlay</t>
+          <t>habwa ang kinaon</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>nga walay buhok</t>
+          <t>pag-awhag</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang gigukod sa sudlay, kay dili siya ganahan mag-comb sa iyang buhok.; Ang iyang buhok pirmi lang gigukod sa sudlay, maong bati kaayo tan-awon.; Si Pedro pirmi lang gigukod sa sudlay, bisan unsa nga event, dili mag-comb.; Ang mga tawo nga gigukod sa sudlay kasagaran dili mag-atiman sa ilang buhok.; Si Juan gigukod sa sudlay, bisan unsa nga party, dili gyud mag-comb.</t>
+          <t>Si Juan habwa ang kinaon pagkalibang tungod sa hilab.; Ang iyang amiga naghabwa ang kinaon kay nasubraan ug kaon.; Si Pedro naghabwa ang kinaon kay nasuka.; Ang mga tawo nga magkaon ug daghan kasagaran maghabwa ang kinaon pagkalibang.; Si Maria naghabwa ang kinaon kay nagkalibanga.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang gigukod sa sudlay, kay dili siya ganahan mag-comb sa iyang buhok.; Ang iyang buhok pirmi lang gigukod sa sudlay, maong bati kaayo tan-awon.; Si Pedro pirmi lang gigukod sa sudlay, bisan unsa nga event, dili mag-comb.; Ang mga tawo nga gigukod sa sudlay kasagaran dili mag-atiman sa ilang buhok.; Si Juan gigukod sa sudlay, bisan unsa nga party, dili gyud mag-comb.</t>
+          <t>Si Juan habwa ang kinaon pagkalibang tungod sa hilab.; Ang iyang amiga naghabwa ang kinaon kay nasubraan ug kaon.; Si Pedro naghabwa ang kinaon kay nasuka.; Ang mga tawo nga magkaon ug daghan kasagaran maghabwa ang kinaon pagkalibang.; Si Maria naghabwa ang kinaon kay nagkalibanga.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>['gigukod']</t>
+          <t>['habwa', 'kinaon']</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -2293,27 +2293,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>gilawog sa tirong</t>
+          <t>hangyo kabayo</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>sa pagbutang sa peligro sa usa ka tawo, ilabina</t>
+          <t>usa ka maalamon nga paagi sa pagbaton ug usa ka butang</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Si Pedro gilawog sa tirong sa iyang kauban, maong nasakpan sa ilang boss.; Ang iyang amiga gilawog sa tirong, maong nahimong scapegoat sa problema.; Si Maria gilawog sa tirong sa iyang mga kauban sa trabaho.; Ang mga tawo nga gilawog sa tirong kasagaran mag-antos sa mga consequences.; Si Juan gilawog sa tirong, bisan wala siya naghimo sa sayop.</t>
+          <t>Si Juan hangyo kabayo, maong nakuha niya ang diskwento.; Ang iyang amiga hangyo kabayo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo kabayo, maong naangkon niya ang iyang gusto.; Ang mga tawo nga hangyo kabayo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo kabayo, maong walay makatanggi sa iyang mga pangutana.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Si Pedro gilawog sa tirong sa iyang kauban, maong nasakpan sa ilang boss.; Ang iyang amiga gilawog sa tirong, maong nahimong scapegoat sa problema.; Si Maria gilawog sa tirong sa iyang mga kauban sa trabaho.; Ang mga tawo nga gilawog sa tirong kasagaran mag-antos sa mga consequences.; Si Juan gilawog sa tirong, bisan wala siya naghimo sa sayop.</t>
+          <t>Si Juan hangyo kabayo, maong nakuha niya ang diskwento.; Ang iyang amiga hangyo kabayo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo kabayo, maong naangkon niya ang iyang gusto.; Ang mga tawo nga hangyo kabayo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo kabayo, maong walay makatanggi sa iyang mga pangutana.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>['gilawog']</t>
+          <t>['hangyo']</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -2323,27 +2323,27 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>giluto sa kaugalingong mantika</t>
+          <t>hangyo lubo</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>sa pag-ukit sa kaugalingong lubnganan</t>
+          <t>usa ka hangyo nga gihimo sa ingon nga paagi nga dili kini makalikay</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Si Pedro giluto sa kaugalingong mantika sa iyang mga sala.; Ang iyang kauban giluto sa kaugalingong mantika tungod sa iyang binuhatan.; Si Maria giluto sa kaugalingong mantika sa iyang mga desisyon.; Ang mga tawo nga magbuhat ug dautan kasagaran giluto sa kaugalingong mantika.; Si Juan giluto sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
+          <t>Si Ana hangyo lubo, maong nakuha niya ang iyang gusto.; Ang iyang kauban hangyo lubo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo lubo, maong naangkon niya ang iyang gipangayo.; Ang mga tawo nga hangyo lubo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo lubo, maong walay makatanggi sa iyang mga pangutana.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Si Pedro giluto sa kaugalingong mantika sa iyang mga sala.; Ang iyang kauban giluto sa kaugalingong mantika tungod sa iyang binuhatan.; Si Maria giluto sa kaugalingong mantika sa iyang mga desisyon.; Ang mga tawo nga magbuhat ug dautan kasagaran giluto sa kaugalingong mantika.; Si Juan giluto sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
+          <t>Si Ana hangyo lubo, maong nakuha niya ang iyang gusto.; Ang iyang kauban hangyo lubo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo lubo, maong naangkon niya ang iyang gipangayo.; Ang mga tawo nga hangyo lubo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo lubo, maong walay makatanggi sa iyang mga pangutana.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>['giluto']</t>
+          <t>['hangyo', 'lubo']</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -2353,27 +2353,27 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>giprito sa kaugalingong mantika</t>
+          <t>hatod og lubong</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Alternatibo nga porma sa giluto sa kaugalingong mantika</t>
+          <t>sa pagtambong sa usa ka paglubong o seremonya sa paghinumdom</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Si Ana giprito sa kaugalingong mantika tungod sa iyang mga aksyon.; Ang mga tao nga magbuhat ug dautan kasagaran giprito sa kaugalingong mantika.; Si Pedro giprito sa kaugalingong mantika sa iyang mga desisyon.; Ang iyang kauban giprito sa kaugalingong mantika sa iyang mga sala.; Si Juan giprito sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
+          <t>Si Juan hatod og lubong sa iyang paryente nga namatay.; Ang mga tawo nga hatod og lubong kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og lubong sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og lubong sa ilang lider.; Si Maria hatod og lubong sa iyang silingan nga namatay.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Si Ana giprito sa kaugalingong mantika tungod sa iyang mga aksyon.; Ang mga tao nga magbuhat ug dautan kasagaran giprito sa kaugalingong mantika.; Si Pedro giprito sa kaugalingong mantika sa iyang mga desisyon.; Ang iyang kauban giprito sa kaugalingong mantika sa iyang mga sala.; Si Juan giprito sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
+          <t>Si Juan hatod og lubong sa iyang paryente nga namatay.; Ang mga tawo nga hatod og lubong kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og lubong sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og lubong sa ilang lider.; Si Maria hatod og lubong sa iyang silingan nga namatay.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>['giprito']</t>
+          <t>['hatod', 'lubong']</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -2383,27 +2383,27 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>gisulod sa bulsa</t>
+          <t>hatod og patay</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>sa paglimbong</t>
+          <t>sa pagtambong sa usa ka paglubong o seremonya sa paghinumdom</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Si Juan gisulod sa bulsa sa iyang kauban, maong nawala ang iyang kwarta.; Ang iyang kauban gisulod sa bulsa sa ilang boss, maong napromote siya.; Si Pedro gisulod sa bulsa sa mga sindikato, maong naglisod siya karon.; Ang mga tawo nga masaligan kasagaran dili gisulod sa bulsa.; Si Maria gisulod sa bulsa, maong nag-antos siya sa iyang mga desisyon.</t>
+          <t>Si Juan hatod og patay sa iyang paryente nga namatay.; Ang mga tawo nga hatod og patay kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og patay sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og patay sa ilang lider.; Si Maria hatod og patay sa iyang silingan nga namatay.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Si Juan gisulod sa bulsa sa iyang kauban, maong nawala ang iyang kwarta.; Ang iyang kauban gisulod sa bulsa sa ilang boss, maong napromote siya.; Si Pedro gisulod sa bulsa sa mga sindikato, maong naglisod siya karon.; Ang mga tawo nga masaligan kasagaran dili gisulod sa bulsa.; Si Maria gisulod sa bulsa, maong nag-antos siya sa iyang mga desisyon.</t>
+          <t>Si Juan hatod og patay sa iyang paryente nga namatay.; Ang mga tawo nga hatod og patay kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og patay sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og patay sa ilang lider.; Si Maria hatod og patay sa iyang silingan nga namatay.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>['gisulod']</t>
+          <t>['hatod', 'patay']</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -2413,27 +2413,27 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>gwapa kon magtalikod</t>
+          <t>higda sa lubi</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>nindot nga tan-awon gikan sa likod</t>
+          <t>pag-ula</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Si Ana gwapa kon magtalikod, pero pagtan-aw sa iyang nawong, lahi gyud diay.; Ang iyang kauban sa trabaho gwapa kon magtalikod, pero pag-atubang, dili na diay.; Si Maria pirmi lang ginatawgon nga gwapa kon magtalikod sa iyang mga amigo.; Ang mga tao nga gwapa kon magtalikod kasagaran maulaw kung mag-atubang.; Si Pedro pirmi lang magbuot-buot ug sulti nga gwapa kon magtalikod.</t>
+          <t>Si Pedro pirmi lang higda sa lubi kung mag-inom.; Ang iyang mga kauban pirmi lang mag-higda sa lubi kung mag-party.; Si Juan higda sa lubi, pirmi lang maghubog-hubog.; Ang mga tawo nga pirmi lang mag-higda sa lubi kasagaran maglisod sa kinabuhi.; Si Maria nasuko kay si Pedro pirmi lang mag-higda sa lubi.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Si Ana gwapa kon magtalikod, pero pagtan-aw sa iyang nawong, lahi gyud diay.; Ang iyang kauban sa trabaho gwapa kon magtalikod, pero pag-atubang, dili na diay.; Si Maria pirmi lang ginatawgon nga gwapa kon magtalikod sa iyang mga amigo.; Ang mga tao nga gwapa kon magtalikod kasagaran maulaw kung mag-atubang.; Si Pedro pirmi lang magbuot-buot ug sulti nga gwapa kon magtalikod.</t>
+          <t>Si Pedro pirmi lang higda sa lubi kung mag-inom.; Ang iyang mga kauban pirmi lang mag-higda sa lubi kung mag-party.; Si Juan higda sa lubi, pirmi lang maghubog-hubog.; Ang mga tawo nga pirmi lang mag-higda sa lubi kasagaran maglisod sa kinabuhi.; Si Maria nasuko kay si Pedro pirmi lang mag-higda sa lubi.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>['magtalikod']</t>
+          <t>['higda']</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -2443,27 +2443,27 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>gwapo kon magtalikod</t>
+          <t>hinaw</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>nindot nga tan-awon gikan sa likod</t>
+          <t>sa paghunaw sa kamot sa usa o sa uban</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Si Juan gwapo kon magtalikod, pero dili na kaayo pag-atubang.; Ang iyang amigo gwapo kon magtalikod, pero bati diay pagtan-aw sa iyang nawong.; Si Pedro pirmi lang ginatawgon nga gwapo kon magtalikod sa iyang barkada.; Ang mga tao nga gwapo kon magtalikod kasagaran dili magdugay sa ilang relasyon.; Si Maria pirmi lang magbuot-buot ug sulti nga gwapo kon magtalikod.</t>
+          <t>Si Pedro naghinaw sa iyang responsibilidad pagkahuman sa proyekto.; Ang iyang kauban naghinaw sa problema kay dili siya gusto maapil.; Si Juan naghinaw sa iyang sala sa trabaho.; Ang mga tawo nga naghinaw sa ilang responsibilidad kasagaran maglisod sa pag-uli sa ilang kasal-anan.; Si Maria naghinaw sa iyang obligasyon sa pamilya.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Si Juan gwapo kon magtalikod, pero dili na kaayo pag-atubang.; Ang iyang amigo gwapo kon magtalikod, pero bati diay pagtan-aw sa iyang nawong.; Si Pedro pirmi lang ginatawgon nga gwapo kon magtalikod sa iyang barkada.; Ang mga tao nga gwapo kon magtalikod kasagaran dili magdugay sa ilang relasyon.; Si Maria pirmi lang magbuot-buot ug sulti nga gwapo kon magtalikod.</t>
+          <t>Si Pedro naghinaw sa iyang responsibilidad pagkahuman sa proyekto.; Ang iyang kauban naghinaw sa problema kay dili siya gusto maapil.; Si Juan naghinaw sa iyang sala sa trabaho.; Ang mga tawo nga naghinaw sa ilang responsibilidad kasagaran maglisod sa pag-uli sa ilang kasal-anan.; Si Maria naghinaw sa iyang obligasyon sa pamilya.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>['magtalikod']</t>
+          <t>['hinaw']</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -2473,27 +2473,27 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>habwa ang kinaon</t>
+          <t>hunaw</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>pag-awhag</t>
+          <t>sa paghunaw sa kamot sa usa o sa uban</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Si Juan habwa ang kinaon pagkalibang tungod sa hilab.; Ang iyang amiga naghabwa ang kinaon kay nasubraan ug kaon.; Si Pedro naghabwa ang kinaon kay nasuka.; Ang mga tawo nga magkaon ug daghan kasagaran maghabwa ang kinaon pagkalibang.; Si Maria naghabwa ang kinaon kay nagkalibanga.</t>
+          <t>Si Pedro naghunaw sa iyang mga sayop kay dili siya gusto ma-blame.; Ang iyang kauban naghunaw sa mga problema aron dili siya maapil.; Si Juan naghunaw sa iyang responsibilidad sa trabaho.; Ang mga tawo nga maghunaw sa ilang obligasyon kasagaran maglisod sa ilang relasyon sa uban.; Si Maria naghunaw sa iyang mga sala aron dili siya mahatagan ug parusa.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Si Juan habwa ang kinaon pagkalibang tungod sa hilab.; Ang iyang amiga naghabwa ang kinaon kay nasubraan ug kaon.; Si Pedro naghabwa ang kinaon kay nasuka.; Ang mga tawo nga magkaon ug daghan kasagaran maghabwa ang kinaon pagkalibang.; Si Maria naghabwa ang kinaon kay nagkalibanga.</t>
+          <t>Si Pedro naghunaw sa iyang mga sayop kay dili siya gusto ma-blame.; Ang iyang kauban naghunaw sa mga problema aron dili siya maapil.; Si Juan naghunaw sa iyang responsibilidad sa trabaho.; Ang mga tawo nga maghunaw sa ilang obligasyon kasagaran maglisod sa ilang relasyon sa uban.; Si Maria naghunaw sa iyang mga sala aron dili siya mahatagan ug parusa.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>['habwa', 'kinaon']</t>
+          <t>['hunaw']</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -2503,27 +2503,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>hangyo kabayo</t>
+          <t>igputi sa uwak</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>usa ka maalamon nga paagi sa pagbaton ug usa ka butang</t>
+          <t>dili gayod</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Si Juan hangyo kabayo, maong nakuha niya ang diskwento.; Ang iyang amiga hangyo kabayo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo kabayo, maong naangkon niya ang iyang gusto.; Ang mga tawo nga hangyo kabayo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo kabayo, maong walay makatanggi sa iyang mga pangutana.</t>
+          <t>Mahitabo lang na igputi sa uwak, dili gyud na matinuod.; Ang iyang pangandoy mahimong realidad igputi sa uwak pa.; Si Pedro musugot igputi sa uwak pa, dili gyud karon.; Ang mga tawo magduda sa iyang mga plano, ingnon nila nga igputi sa uwak pa na matuman.; Si Maria mutuman sa iyang sugo igputi sa uwak pa, dili gyud karon.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Si Juan hangyo kabayo, maong nakuha niya ang diskwento.; Ang iyang amiga hangyo kabayo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo kabayo, maong naangkon niya ang iyang gusto.; Ang mga tawo nga hangyo kabayo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo kabayo, maong walay makatanggi sa iyang mga pangutana.</t>
+          <t>Mahitabo lang na igputi sa uwak, dili gyud na matinuod.; Ang iyang pangandoy mahimong realidad igputi sa uwak pa.; Si Pedro musugot igputi sa uwak pa, dili gyud karon.; Ang mga tawo magduda sa iyang mga plano, ingnon nila nga igputi sa uwak pa na matuman.; Si Maria mutuman sa iyang sugo igputi sa uwak pa, dili gyud karon.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>['hangyo']</t>
+          <t>['igputi']</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -2533,27 +2533,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>hangyo lubo</t>
+          <t>ikasuga ang ihi</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>usa ka hangyo nga gihimo sa ingon nga paagi nga dili kini makalikay</t>
+          <t>alang sa usa ka babaye nga mahimong matahum kaayo</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Si Ana hangyo lubo, maong nakuha niya ang iyang gusto.; Ang iyang kauban hangyo lubo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo lubo, maong naangkon niya ang iyang gipangayo.; Ang mga tawo nga hangyo lubo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo lubo, maong walay makatanggi sa iyang mga pangutana.</t>
+          <t>Si Ana ikasuga ang ihi sa iyang kaanyag.; Ang iyang amiga ikasuga ang ihi sa iyang hitsura.; Si Pedro ikasuga ang ihi sa iyang pagkagwapo.; Ang mga tawo nga ikasuga ang ihi kasagaran daghan ug mga admirers.; Si Maria ikasuga ang ihi sa iyang pagkamahinhin.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Si Ana hangyo lubo, maong nakuha niya ang iyang gusto.; Ang iyang kauban hangyo lubo, bisan unsa nga butang iyang makuha.; Si Pedro hangyo lubo, maong naangkon niya ang iyang gipangayo.; Ang mga tawo nga hangyo lubo kasagaran magmalampuson sa ilang mga plano.; Si Maria hangyo lubo, maong walay makatanggi sa iyang mga pangutana.</t>
+          <t>Si Ana ikasuga ang ihi sa iyang kaanyag.; Ang iyang amiga ikasuga ang ihi sa iyang hitsura.; Si Pedro ikasuga ang ihi sa iyang pagkagwapo.; Ang mga tawo nga ikasuga ang ihi kasagaran daghan ug mga admirers.; Si Maria ikasuga ang ihi sa iyang pagkamahinhin.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>['hangyo', 'lubo']</t>
+          <t>['ikasuga']</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -2563,27 +2563,27 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>hatod og lubong</t>
+          <t>kakha tuka</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>sa pagtambong sa usa ka paglubong o seremonya sa paghinumdom</t>
+          <t>kamot-sa-lubong</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Si Juan hatod og lubong sa iyang paryente nga namatay.; Ang mga tawo nga hatod og lubong kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og lubong sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og lubong sa ilang lider.; Si Maria hatod og lubong sa iyang silingan nga namatay.</t>
+          <t>Si Pedro kakha tuka, walay savings ug pirmi lang magkaproblema sa kwarta.; Ang ilang pamilya kakha tuka, pirmi lang maglisod sa pagkaon.; Si Maria nagkinabuhi nga kakha tuka, walay nahabilin nga kwarta.; Ang mga tawo nga kakha tuka kasagaran maglisod sa kinabuhi.; Si Juan pirmi lang kakha tuka, walay nahabilin nga budget.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Si Juan hatod og lubong sa iyang paryente nga namatay.; Ang mga tawo nga hatod og lubong kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og lubong sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og lubong sa ilang lider.; Si Maria hatod og lubong sa iyang silingan nga namatay.</t>
+          <t>Si Pedro kakha tuka, walay savings ug pirmi lang magkaproblema sa kwarta.; Ang ilang pamilya kakha tuka, pirmi lang maglisod sa pagkaon.; Si Maria nagkinabuhi nga kakha tuka, walay nahabilin nga kwarta.; Ang mga tawo nga kakha tuka kasagaran maglisod sa kinabuhi.; Si Juan pirmi lang kakha tuka, walay nahabilin nga budget.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>['hatod', 'lubong']</t>
+          <t>['kakha', 'tuka']</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -2593,27 +2593,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>hatod og patay</t>
+          <t>kapugngan pa ang baha, dili ang biga</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>sa pagtambong sa usa ka paglubong o seremonya sa paghinumdom</t>
+          <t>dili mapugngan</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Si Juan hatod og patay sa iyang paryente nga namatay.; Ang mga tawo nga hatod og patay kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og patay sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og patay sa ilang lider.; Si Maria hatod og patay sa iyang silingan nga namatay.</t>
+          <t>Si Pedro dili mapugngan sa iyang gusto, kapugngan pa ang baha, dili ang biga.; Ang iyang determinasyon dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Juan adunay grabe kaayo nga pagnanasa, kapugngan pa ang baha, dili ang biga.; Ang iyang kalagot dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Maria adunay dakong pangandoy nga dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Si Juan hatod og patay sa iyang paryente nga namatay.; Ang mga tawo nga hatod og patay kasagaran nagpakita ug respeto sa namatay.; Si Pedro hatod og patay sa iyang kauban sa trabaho.; Ang mga kauban sa barangay naghatod og patay sa ilang lider.; Si Maria hatod og patay sa iyang silingan nga namatay.</t>
+          <t>Si Pedro dili mapugngan sa iyang gusto, kapugngan pa ang baha, dili ang biga.; Ang iyang determinasyon dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Juan adunay grabe kaayo nga pagnanasa, kapugngan pa ang baha, dili ang biga.; Ang iyang kalagot dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Maria adunay dakong pangandoy nga dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>['hatod', 'patay']</t>
+          <t>['kapugngan']</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -2623,27 +2623,27 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>higda sa lubi</t>
+          <t>kasab-itag bukag ang simod</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>pag-ula</t>
+          <t>sullen</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang higda sa lubi kung mag-inom.; Ang iyang mga kauban pirmi lang mag-higda sa lubi kung mag-party.; Si Juan higda sa lubi, pirmi lang maghubog-hubog.; Ang mga tawo nga pirmi lang mag-higda sa lubi kasagaran maglisod sa kinabuhi.; Si Maria nasuko kay si Pedro pirmi lang mag-higda sa lubi.</t>
+          <t>Si Ana pirmi lang kasab-itag bukag ang simod kung naay problema.; Ang iyang anak pirmi lang kasab-itag bukag ang simod kung walay makuha nga gusto.; Si Pedro pirmi lang kasab-itag bukag ang simod kung naa'y magbuot kaniya.; Ang mga tawo nga kasab-itag bukag ang simod kasagaran dili ganahan makig-istorya.; Si Maria pirmi lang kasab-itag bukag ang simod kung naa'y maglagot kaniya.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang higda sa lubi kung mag-inom.; Ang iyang mga kauban pirmi lang mag-higda sa lubi kung mag-party.; Si Juan higda sa lubi, pirmi lang maghubog-hubog.; Ang mga tawo nga pirmi lang mag-higda sa lubi kasagaran maglisod sa kinabuhi.; Si Maria nasuko kay si Pedro pirmi lang mag-higda sa lubi.</t>
+          <t>Si Ana pirmi lang kasab-itag bukag ang simod kung naay problema.; Ang iyang anak pirmi lang kasab-itag bukag ang simod kung walay makuha nga gusto.; Si Pedro pirmi lang kasab-itag bukag ang simod kung naa'y magbuot kaniya.; Ang mga tawo nga kasab-itag bukag ang simod kasagaran dili ganahan makig-istorya.; Si Maria pirmi lang kasab-itag bukag ang simod kung naa'y maglagot kaniya.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>['higda']</t>
+          <t>['kasab-itan']</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -2653,27 +2653,27 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>hinaw</t>
+          <t>katagakon ang mata</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>sa paghunaw sa kamot sa usa o sa uban</t>
+          <t>mag-ulog</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Si Pedro naghinaw sa iyang responsibilidad pagkahuman sa proyekto.; Ang iyang kauban naghinaw sa problema kay dili siya gusto maapil.; Si Juan naghinaw sa iyang sala sa trabaho.; Ang mga tawo nga naghinaw sa ilang responsibilidad kasagaran maglisod sa pag-uli sa ilang kasal-anan.; Si Maria naghinaw sa iyang obligasyon sa pamilya.</t>
+          <t>Si Juan katagakon ang mata human sa taas nga gabii.; Ang iyang anak katagakon ang mata human magbilar sa pagduwa sa computer.; Si Pedro katagakon ang mata human sa taas nga trabaho sa opisina.; Ang mga tawo nga katagakon ang mata kasagaran dili makamata ug sayo.; Si Maria katagakon ang mata human sa pila ka gabii nga trabaho.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Si Pedro naghinaw sa iyang responsibilidad pagkahuman sa proyekto.; Ang iyang kauban naghinaw sa problema kay dili siya gusto maapil.; Si Juan naghinaw sa iyang sala sa trabaho.; Ang mga tawo nga naghinaw sa ilang responsibilidad kasagaran maglisod sa pag-uli sa ilang kasal-anan.; Si Maria naghinaw sa iyang obligasyon sa pamilya.</t>
+          <t>Si Juan katagakon ang mata human sa taas nga gabii.; Ang iyang anak katagakon ang mata human magbilar sa pagduwa sa computer.; Si Pedro katagakon ang mata human sa taas nga trabaho sa opisina.; Ang mga tawo nga katagakon ang mata kasagaran dili makamata ug sayo.; Si Maria katagakon ang mata human sa pila ka gabii nga trabaho.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>['hinaw']</t>
+          <t>['katagakon']</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -2683,27 +2683,27 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>hunaw</t>
+          <t>kilatan</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>sa paghunaw sa kamot sa usa o sa uban</t>
+          <t>nga madalagan sa kilat</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Si Pedro naghunaw sa iyang mga sayop kay dili siya gusto ma-blame.; Ang iyang kauban naghunaw sa mga problema aron dili siya maapil.; Si Juan naghunaw sa iyang responsibilidad sa trabaho.; Ang mga tawo nga maghunaw sa ilang obligasyon kasagaran maglisod sa ilang relasyon sa uban.; Si Maria naghunaw sa iyang mga sala aron dili siya mahatagan ug parusa.</t>
+          <t>Si Pedro kilatan kay nangawat siya sa tindahan.; Ang iyang amigo kilatan kay nagbinuang sa iyang ginikanan.; Si Juan kilatan sa iyang mga kauban kay nagsumbong sa boss.; Ang mga tawo nga kilatan kasagaran magbasol sa ilang binuhatan.; Si Maria kilatan kay wala mutuman sa sugo sa iyang inahan.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Si Pedro naghunaw sa iyang mga sayop kay dili siya gusto ma-blame.; Ang iyang kauban naghunaw sa mga problema aron dili siya maapil.; Si Juan naghunaw sa iyang responsibilidad sa trabaho.; Ang mga tawo nga maghunaw sa ilang obligasyon kasagaran maglisod sa ilang relasyon sa uban.; Si Maria naghunaw sa iyang mga sala aron dili siya mahatagan ug parusa.</t>
+          <t>Si Pedro kilatan kay nangawat siya sa tindahan.; Ang iyang amigo kilatan kay nagbinuang sa iyang ginikanan.; Si Juan kilatan sa iyang mga kauban kay nagsumbong sa boss.; Ang mga tawo nga kilatan kasagaran magbasol sa ilang binuhatan.; Si Maria kilatan kay wala mutuman sa sugo sa iyang inahan.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>['hunaw']</t>
+          <t>['kilatan']</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -2713,27 +2713,27 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>igputi sa uwak</t>
+          <t>kirig</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>dili gayod</t>
+          <t>pag-awhag</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Mahitabo lang na igputi sa uwak, dili gyud na matinuod.; Ang iyang pangandoy mahimong realidad igputi sa uwak pa.; Si Pedro musugot igputi sa uwak pa, dili gyud karon.; Ang mga tawo magduda sa iyang mga plano, ingnon nila nga igputi sa uwak pa na matuman.; Si Maria mutuman sa iyang sugo igputi sa uwak pa, dili gyud karon.</t>
+          <t>Si Ana kirig sa iyang sakit nga epilepsy.; Ang iyang lola kirig tungod sa iyang katigulangon.; Si Pedro kirig human nalipong sa init.; Ang mga tawo nga naay sakit kasagaran kirig kung dili mag-amping.; Si Juan kirig sa kahadlok pagkakita sa aksidente.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Mahitabo lang na igputi sa uwak, dili gyud na matinuod.; Ang iyang pangandoy mahimong realidad igputi sa uwak pa.; Si Pedro musugot igputi sa uwak pa, dili gyud karon.; Ang mga tawo magduda sa iyang mga plano, ingnon nila nga igputi sa uwak pa na matuman.; Si Maria mutuman sa iyang sugo igputi sa uwak pa, dili gyud karon.</t>
+          <t>Si Ana kirig sa iyang sakit nga epilepsy.; Ang iyang lola kirig tungod sa iyang katigulangon.; Si Pedro kirig human nalipong sa init.; Ang mga tawo nga naay sakit kasagaran kirig kung dili mag-amping.; Si Juan kirig sa kahadlok pagkakita sa aksidente.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>['igputi']</t>
+          <t>['kirig']</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -2743,27 +2743,27 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ikasuga ang ihi</t>
+          <t>kulang sa dukol</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>alang sa usa ka babaye nga mahimong matahum kaayo</t>
+          <t>usa ka buangbuang nga tawo</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Si Ana ikasuga ang ihi sa iyang kaanyag.; Ang iyang amiga ikasuga ang ihi sa iyang hitsura.; Si Pedro ikasuga ang ihi sa iyang pagkagwapo.; Ang mga tawo nga ikasuga ang ihi kasagaran daghan ug mga admirers.; Si Maria ikasuga ang ihi sa iyang pagkamahinhin.</t>
+          <t>Si Pedro kulang sa dukol, maong pirmi lang magbinuang.; Ang iyang anak kulang sa dukol, dili gyud magtinarong sa pag-eskwela.; Si Juan kulang sa dukol, pirmi lang magtambay sa kanto.; Ang mga tawo nga kulang sa dukol kasagaran maglisod sa pagtrabaho.; Si Maria kulang sa dukol, pirmi lang magbulakbol.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Si Ana ikasuga ang ihi sa iyang kaanyag.; Ang iyang amiga ikasuga ang ihi sa iyang hitsura.; Si Pedro ikasuga ang ihi sa iyang pagkagwapo.; Ang mga tawo nga ikasuga ang ihi kasagaran daghan ug mga admirers.; Si Maria ikasuga ang ihi sa iyang pagkamahinhin.</t>
+          <t>Si Pedro kulang sa dukol, maong pirmi lang magbinuang.; Ang iyang anak kulang sa dukol, dili gyud magtinarong sa pag-eskwela.; Si Juan kulang sa dukol, pirmi lang magtambay sa kanto.; Ang mga tawo nga kulang sa dukol kasagaran maglisod sa pagtrabaho.; Si Maria kulang sa dukol, pirmi lang magbulakbol.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>['ikasuga']</t>
+          <t>['dukol']</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -2773,27 +2773,27 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>kakha tuka</t>
+          <t>kulang sa tagad</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>kamot-sa-lubong</t>
+          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Si Pedro kakha tuka, walay savings ug pirmi lang magkaproblema sa kwarta.; Ang ilang pamilya kakha tuka, pirmi lang maglisod sa pagkaon.; Si Maria nagkinabuhi nga kakha tuka, walay nahabilin nga kwarta.; Ang mga tawo nga kakha tuka kasagaran maglisod sa kinabuhi.; Si Juan pirmi lang kakha tuka, walay nahabilin nga budget.</t>
+          <t>Si Pedro kulang sa tagad, maong pirmi lang magpakitkit ug magpasikat.; Ang iyang amiga kulang sa tagad, maong pirmi lang mag-agi-agi sa ilang lugar.; Si Juan kulang sa tagad, pirmi lang magpasikat sa mga tao.; Ang mga tawo nga kulang sa tagad kasagaran magbuhat ug dautan para makuha ang attention sa uban.; Si Maria kulang sa tagad, pirmi lang magbinuang aron makuha ang atensyon sa iyang mga kauban.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Si Pedro kakha tuka, walay savings ug pirmi lang magkaproblema sa kwarta.; Ang ilang pamilya kakha tuka, pirmi lang maglisod sa pagkaon.; Si Maria nagkinabuhi nga kakha tuka, walay nahabilin nga kwarta.; Ang mga tawo nga kakha tuka kasagaran maglisod sa kinabuhi.; Si Juan pirmi lang kakha tuka, walay nahabilin nga budget.</t>
+          <t>Si Pedro kulang sa tagad, maong pirmi lang magpakitkit ug magpasikat.; Ang iyang amiga kulang sa tagad, maong pirmi lang mag-agi-agi sa ilang lugar.; Si Juan kulang sa tagad, pirmi lang magpasikat sa mga tao.; Ang mga tawo nga kulang sa tagad kasagaran magbuhat ug dautan para makuha ang attention sa uban.; Si Maria kulang sa tagad, pirmi lang magbinuang aron makuha ang atensyon sa iyang mga kauban.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>['kakha', 'tuka']</t>
+          <t>['tagad']</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -2803,27 +2803,27 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>kapugngan pa ang baha, dili ang biga</t>
+          <t>kulban sa kaldero</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>dili mapugngan</t>
+          <t>sa paghilom nga dili</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Si Pedro dili mapugngan sa iyang gusto, kapugngan pa ang baha, dili ang biga.; Ang iyang determinasyon dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Juan adunay grabe kaayo nga pagnanasa, kapugngan pa ang baha, dili ang biga.; Ang iyang kalagot dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Maria adunay dakong pangandoy nga dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
+          <t>Si Juan pirmi lang kulban sa kaldero kung makiglalis sa iyang kauban.; Ang iyang amigo kulban sa kaldero kung naa sa meeting.; Si Pedro pirmi lang kulban sa kaldero kung mag-istorya sa iyang boss.; Ang mga tawo nga kulban sa kaldero kasagaran dili makapanalipod sa ilang kaugalingon.; Si Maria pirmi lang kulban sa kaldero kung naa sa public speaking.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Si Pedro dili mapugngan sa iyang gusto, kapugngan pa ang baha, dili ang biga.; Ang iyang determinasyon dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Juan adunay grabe kaayo nga pagnanasa, kapugngan pa ang baha, dili ang biga.; Ang iyang kalagot dili mapugngan, kapugngan pa ang baha, dili ang biga.; Si Maria adunay dakong pangandoy nga dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
+          <t>Si Juan pirmi lang kulban sa kaldero kung makiglalis sa iyang kauban.; Ang iyang amigo kulban sa kaldero kung naa sa meeting.; Si Pedro pirmi lang kulban sa kaldero kung mag-istorya sa iyang boss.; Ang mga tawo nga kulban sa kaldero kasagaran dili makapanalipod sa ilang kaugalingon.; Si Maria pirmi lang kulban sa kaldero kung naa sa public speaking.</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>['kapugngan']</t>
+          <t>['kulban']</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -2833,27 +2833,27 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>kasab-itag bukag ang simod</t>
+          <t>kuskos balungos</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>sullen</t>
+          <t>pag-awhag</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang kasab-itag bukag ang simod kung naay problema.; Ang iyang anak pirmi lang kasab-itag bukag ang simod kung walay makuha nga gusto.; Si Pedro pirmi lang kasab-itag bukag ang simod kung naa'y magbuot kaniya.; Ang mga tawo nga kasab-itag bukag ang simod kasagaran dili ganahan makig-istorya.; Si Maria pirmi lang kasab-itag bukag ang simod kung naa'y maglagot kaniya.</t>
+          <t>Si Pedro pirmi lang kuskos balungos sa iyang trabaho.; Ang iyang anak kuskos balungos sa eskwela, bisan walay hinungdan.; Si Maria kuskos balungos sa balay, walay undang ang trabaho.; Ang mga tawo nga kuskos balungos kasagaran maglisod ug kapahulayan.; Si Juan pirmi lang kuskos balungos sa mga problema nga walay solusyon.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang kasab-itag bukag ang simod kung naay problema.; Ang iyang anak pirmi lang kasab-itag bukag ang simod kung walay makuha nga gusto.; Si Pedro pirmi lang kasab-itag bukag ang simod kung naa'y magbuot kaniya.; Ang mga tawo nga kasab-itag bukag ang simod kasagaran dili ganahan makig-istorya.; Si Maria pirmi lang kasab-itag bukag ang simod kung naa'y maglagot kaniya.</t>
+          <t>Si Pedro pirmi lang kuskos balungos sa iyang trabaho.; Ang iyang anak kuskos balungos sa eskwela, bisan walay hinungdan.; Si Maria kuskos balungos sa balay, walay undang ang trabaho.; Ang mga tawo nga kuskos balungos kasagaran maglisod ug kapahulayan.; Si Juan pirmi lang kuskos balungos sa mga problema nga walay solusyon.</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>['kasab-itan']</t>
+          <t>['kuskos']</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -2863,27 +2863,27 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>katagakon ang mata</t>
+          <t>kuskos-balungos</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>mag-ulog</t>
+          <t>alternatibong pagsulat sa kuskos balungos</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Si Juan katagakon ang mata human sa taas nga gabii.; Ang iyang anak katagakon ang mata human magbilar sa pagduwa sa computer.; Si Pedro katagakon ang mata human sa taas nga trabaho sa opisina.; Ang mga tawo nga katagakon ang mata kasagaran dili makamata ug sayo.; Si Maria katagakon ang mata human sa pila ka gabii nga trabaho.</t>
+          <t>Si Ana pirmi lang kuskos-balungos kung naay buhaton nga dili siya ganahan.; Ang iyang amahan kuskos-balungos sa mga butang nga wala'y hinungdan.; Si Pedro kuskos-balungos pirmi, bisan gamay nga problema.; Ang mga tawo nga kuskos-balungos kasagaran magpaluya sa ilang mga kauban.; Si Maria pirmi lang kuskos-balungos bisan unsa nga buhaton.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Si Juan katagakon ang mata human sa taas nga gabii.; Ang iyang anak katagakon ang mata human magbilar sa pagduwa sa computer.; Si Pedro katagakon ang mata human sa taas nga trabaho sa opisina.; Ang mga tawo nga katagakon ang mata kasagaran dili makamata ug sayo.; Si Maria katagakon ang mata human sa pila ka gabii nga trabaho.</t>
+          <t>Si Ana pirmi lang kuskos-balungos kung naay buhaton nga dili siya ganahan.; Ang iyang amahan kuskos-balungos sa mga butang nga wala'y hinungdan.; Si Pedro kuskos-balungos pirmi, bisan gamay nga problema.; Ang mga tawo nga kuskos-balungos kasagaran magpaluya sa ilang mga kauban.; Si Maria pirmi lang kuskos-balungos bisan unsa nga buhaton.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>['katagakon']</t>
+          <t>['kuskos']</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -2893,27 +2893,27 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>kilatan</t>
+          <t>kusog mokaon og gasolina</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>nga madalagan sa kilat</t>
+          <t>gas-gussing</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Si Pedro kilatan kay nangawat siya sa tindahan.; Ang iyang amigo kilatan kay nagbinuang sa iyang ginikanan.; Si Juan kilatan sa iyang mga kauban kay nagsumbong sa boss.; Ang mga tawo nga kilatan kasagaran magbasol sa ilang binuhatan.; Si Maria kilatan kay wala mutuman sa sugo sa iyang inahan.</t>
+          <t>Ang sakyanan ni Juan kusog mokaon og gasolina, maong mahal kaayo ang gasto.; Ang iyang motor kusog mokaon og gasolina, pirmi lang magpailis.; Si Pedro ganahan ug sakyanan nga dili kusog mokaon og gasolina.; Ang mga tawo nga mag-drive ug sakyanan nga kusog mokaon og gasolina kasagaran maglisod sa gasto.; Si Maria dili ganahan ug sakyanan nga kusog mokaon og gasolina kay mahal ang maintenance.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Si Pedro kilatan kay nangawat siya sa tindahan.; Ang iyang amigo kilatan kay nagbinuang sa iyang ginikanan.; Si Juan kilatan sa iyang mga kauban kay nagsumbong sa boss.; Ang mga tawo nga kilatan kasagaran magbasol sa ilang binuhatan.; Si Maria kilatan kay wala mutuman sa sugo sa iyang inahan.</t>
+          <t>Ang sakyanan ni Juan kusog mokaon og gasolina, maong mahal kaayo ang gasto.; Ang iyang motor kusog mokaon og gasolina, pirmi lang magpailis.; Si Pedro ganahan ug sakyanan nga dili kusog mokaon og gasolina.; Ang mga tawo nga mag-drive ug sakyanan nga kusog mokaon og gasolina kasagaran maglisod sa gasto.; Si Maria dili ganahan ug sakyanan nga kusog mokaon og gasolina kay mahal ang maintenance.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>['kilatan']</t>
+          <t>['mokaon']</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -2923,27 +2923,27 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>kirig</t>
+          <t>kuwang sa tagad</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>pag-awhag</t>
+          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Si Ana kirig sa iyang sakit nga epilepsy.; Ang iyang lola kirig tungod sa iyang katigulangon.; Si Pedro kirig human nalipong sa init.; Ang mga tawo nga naay sakit kasagaran kirig kung dili mag-amping.; Si Juan kirig sa kahadlok pagkakita sa aksidente.</t>
+          <t>Si Ana kuwang sa tagad, maong pirmi lang magpahipi sa kanto.; Ang iyang kauban sa trabaho kuwang sa tagad, maong pirmi lang magpabida.; Si Pedro kuwang sa tagad, bisan unsa nga event ganahan magpakita.; Ang mga tawo nga kuwang sa tagad kasagaran magbuhat ug mga butang aron makuha ang atensyon.; Si Juan pirmi lang magpakita sa mga tao kay kuwang sa tagad.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Si Ana kirig sa iyang sakit nga epilepsy.; Ang iyang lola kirig tungod sa iyang katigulangon.; Si Pedro kirig human nalipong sa init.; Ang mga tawo nga naay sakit kasagaran kirig kung dili mag-amping.; Si Juan kirig sa kahadlok pagkakita sa aksidente.</t>
+          <t>Si Ana kuwang sa tagad, maong pirmi lang magpahipi sa kanto.; Ang iyang kauban sa trabaho kuwang sa tagad, maong pirmi lang magpabida.; Si Pedro kuwang sa tagad, bisan unsa nga event ganahan magpakita.; Ang mga tawo nga kuwang sa tagad kasagaran magbuhat ug mga butang aron makuha ang atensyon.; Si Juan pirmi lang magpakita sa mga tao kay kuwang sa tagad.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>['kirig']</t>
+          <t>['tagad']</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -2953,27 +2953,27 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>kulang sa dukol</t>
+          <t>kuyog baboy</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>usa ka buangbuang nga tawo</t>
+          <t>usa ka tagalong</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Si Pedro kulang sa dukol, maong pirmi lang magbinuang.; Ang iyang anak kulang sa dukol, dili gyud magtinarong sa pag-eskwela.; Si Juan kulang sa dukol, pirmi lang magtambay sa kanto.; Ang mga tawo nga kulang sa dukol kasagaran maglisod sa pagtrabaho.; Si Maria kulang sa dukol, pirmi lang magbulakbol.</t>
+          <t>Si Maria pirmi lang kuyog baboy, bisan asa moadto iyang best friend naa gyud.; Ang iyang igsuon kuyog baboy pirmi kung maglakaw-lakaw.; Si Pedro dili ganahan ug kuyog baboy kay samok kaayo.; Ang mga tawo nga kuyog baboy kasagaran magpalisod sa ilang mga kauban.; Si Juan pirmi lang kuyog baboy bisan unsa nga lakaw.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Si Pedro kulang sa dukol, maong pirmi lang magbinuang.; Ang iyang anak kulang sa dukol, dili gyud magtinarong sa pag-eskwela.; Si Juan kulang sa dukol, pirmi lang magtambay sa kanto.; Ang mga tawo nga kulang sa dukol kasagaran maglisod sa pagtrabaho.; Si Maria kulang sa dukol, pirmi lang magbulakbol.</t>
+          <t>Si Maria pirmi lang kuyog baboy, bisan asa moadto iyang best friend naa gyud.; Ang iyang igsuon kuyog baboy pirmi kung maglakaw-lakaw.; Si Pedro dili ganahan ug kuyog baboy kay samok kaayo.; Ang mga tawo nga kuyog baboy kasagaran magpalisod sa ilang mga kauban.; Si Juan pirmi lang kuyog baboy bisan unsa nga lakaw.</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>['dukol']</t>
+          <t>['kuyog']</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -2983,27 +2983,27 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>kulang sa tagad</t>
+          <t>lapas na sa kalendaryo</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
+          <t>usa ka tawo nga kapin sa 31 ka tuig ang edad</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Si Pedro kulang sa tagad, maong pirmi lang magpakitkit ug magpasikat.; Ang iyang amiga kulang sa tagad, maong pirmi lang mag-agi-agi sa ilang lugar.; Si Juan kulang sa tagad, pirmi lang magpasikat sa mga tao.; Ang mga tawo nga kulang sa tagad kasagaran magbuhat ug dautan para makuha ang attention sa uban.; Si Maria kulang sa tagad, pirmi lang magbinuang aron makuha ang atensyon sa iyang mga kauban.</t>
+          <t>Si Ana lapas na sa kalendaryo, pero dili gihapon magminyo.; Ang iyang igsuon lapas na sa kalendaryo, pero dili gihapon magka-anak.; Si Pedro lapas na sa kalendaryo, pero wala gihapon trabaho.; Ang mga tawo nga lapas na sa kalendaryo kasagaran magpanikad sa ilang mga plano.; Si Juan lapas na sa kalendaryo, pero wala gihapon magtarong sa kinabuhi.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Si Pedro kulang sa tagad, maong pirmi lang magpakitkit ug magpasikat.; Ang iyang amiga kulang sa tagad, maong pirmi lang mag-agi-agi sa ilang lugar.; Si Juan kulang sa tagad, pirmi lang magpasikat sa mga tao.; Ang mga tawo nga kulang sa tagad kasagaran magbuhat ug dautan para makuha ang attention sa uban.; Si Maria kulang sa tagad, pirmi lang magbinuang aron makuha ang atensyon sa iyang mga kauban.</t>
+          <t>Si Ana lapas na sa kalendaryo, pero dili gihapon magminyo.; Ang iyang igsuon lapas na sa kalendaryo, pero dili gihapon magka-anak.; Si Pedro lapas na sa kalendaryo, pero wala gihapon trabaho.; Ang mga tawo nga lapas na sa kalendaryo kasagaran magpanikad sa ilang mga plano.; Si Juan lapas na sa kalendaryo, pero wala gihapon magtarong sa kinabuhi.</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>['tagad']</t>
+          <t>['lapas']</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -3013,27 +3013,27 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>kulban sa kaldero</t>
+          <t>lapos sa pikas dunggan</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>sa paghilom nga dili</t>
+          <t>sa pagsulod sa usa ka dalunggan ug paggawas sa laing dalunggan</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang kulban sa kaldero kung makiglalis sa iyang kauban.; Ang iyang amigo kulban sa kaldero kung naa sa meeting.; Si Pedro pirmi lang kulban sa kaldero kung mag-istorya sa iyang boss.; Ang mga tawo nga kulban sa kaldero kasagaran dili makapanalipod sa ilang kaugalingon.; Si Maria pirmi lang kulban sa kaldero kung naa sa public speaking.</t>
+          <t>Ang tambag sa iyang ginikanan lapos ra sa pikas dunggan.; Si Pedro pirmi lang lapos sa pikas dunggan ang mga lectures sa eskwela.; Ang mga sugo sa iyang boss kay lapos ra sa pikas dunggan.; Ang mga tawo nga dili magtagad kasagaran maglapos ra sa pikas dunggan ang mga pulong sa uban.; Si Maria pirmi lang maglapos ra sa pikas dunggan ang mga tambag sa iyang mga amiga.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang kulban sa kaldero kung makiglalis sa iyang kauban.; Ang iyang amigo kulban sa kaldero kung naa sa meeting.; Si Pedro pirmi lang kulban sa kaldero kung mag-istorya sa iyang boss.; Ang mga tawo nga kulban sa kaldero kasagaran dili makapanalipod sa ilang kaugalingon.; Si Maria pirmi lang kulban sa kaldero kung naa sa public speaking.</t>
+          <t>Ang tambag sa iyang ginikanan lapos ra sa pikas dunggan.; Si Pedro pirmi lang lapos sa pikas dunggan ang mga lectures sa eskwela.; Ang mga sugo sa iyang boss kay lapos ra sa pikas dunggan.; Ang mga tawo nga dili magtagad kasagaran maglapos ra sa pikas dunggan ang mga pulong sa uban.; Si Maria pirmi lang maglapos ra sa pikas dunggan ang mga tambag sa iyang mga amiga.</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>['kulban']</t>
+          <t>['lapos', 'dunggan']</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -3043,27 +3043,27 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>kuskos balungos</t>
+          <t>litik</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>pag-awhag</t>
+          <t>sa pag-aghat sa tudlo</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang kuskos balungos sa iyang trabaho.; Ang iyang anak kuskos balungos sa eskwela, bisan walay hinungdan.; Si Maria kuskos balungos sa balay, walay undang ang trabaho.; Ang mga tawo nga kuskos balungos kasagaran maglisod ug kapahulayan.; Si Juan pirmi lang kuskos balungos sa mga problema nga walay solusyon.</t>
+          <t>Si Juan naglitik sa iyang mga kalagot sa iyang kauban.; Ang iyang anak naglitik ug sugilanon nga makalipay.; Si Pedro naglitik sa iyang mga plano sa negosyo.; Ang mga tawo nga naglitik sa ilang mga pangandoy kasagaran magmalampuson.; Si Maria naglitik sa iyang mga pangandoy sa kinabuhi.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang kuskos balungos sa iyang trabaho.; Ang iyang anak kuskos balungos sa eskwela, bisan walay hinungdan.; Si Maria kuskos balungos sa balay, walay undang ang trabaho.; Ang mga tawo nga kuskos balungos kasagaran maglisod ug kapahulayan.; Si Juan pirmi lang kuskos balungos sa mga problema nga walay solusyon.</t>
+          <t>Si Juan naglitik sa iyang mga kalagot sa iyang kauban.; Ang iyang anak naglitik ug sugilanon nga makalipay.; Si Pedro naglitik sa iyang mga plano sa negosyo.; Ang mga tawo nga naglitik sa ilang mga pangandoy kasagaran magmalampuson.; Si Maria naglitik sa iyang mga pangandoy sa kinabuhi.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>['kuskos']</t>
+          <t>['litik']</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -3073,27 +3073,27 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>kuskos-balungos</t>
+          <t>lunod patay</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>alternatibong pagsulat sa kuskos balungos</t>
+          <t>dihard</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang kuskos-balungos kung naay buhaton nga dili siya ganahan.; Ang iyang amahan kuskos-balungos sa mga butang nga wala'y hinungdan.; Si Pedro kuskos-balungos pirmi, bisan gamay nga problema.; Ang mga tawo nga kuskos-balungos kasagaran magpaluya sa ilang mga kauban.; Si Maria pirmi lang kuskos-balungos bisan unsa nga buhaton.</t>
+          <t>Si Pedro lunod patay sa iyang prinsipyo, dili gyud magbag-o.; Ang iyang amigo lunod patay sa iyang pagtuo bisan pa sa mga pagsulay.; Si Juan lunod patay sa pagsuporta sa iyang pamilya.; Ang mga tawo nga lunod patay kasagaran adunay baruganan nga dili matay-og.; Si Maria lunod patay sa pagpanalipod sa iyang mga kauban.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang kuskos-balungos kung naay buhaton nga dili siya ganahan.; Ang iyang amahan kuskos-balungos sa mga butang nga wala'y hinungdan.; Si Pedro kuskos-balungos pirmi, bisan gamay nga problema.; Ang mga tawo nga kuskos-balungos kasagaran magpaluya sa ilang mga kauban.; Si Maria pirmi lang kuskos-balungos bisan unsa nga buhaton.</t>
+          <t>Si Pedro lunod patay sa iyang prinsipyo, dili gyud magbag-o.; Ang iyang amigo lunod patay sa iyang pagtuo bisan pa sa mga pagsulay.; Si Juan lunod patay sa pagsuporta sa iyang pamilya.; Ang mga tawo nga lunod patay kasagaran adunay baruganan nga dili matay-og.; Si Maria lunod patay sa pagpanalipod sa iyang mga kauban.</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>['kuskos']</t>
+          <t>['lunod', 'patay']</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -3103,27 +3103,27 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>kusog mokaon og gasolina</t>
+          <t>lupig pay ungo</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>gas-gussing</t>
+          <t>ang usa ka tawo nga wala damha moabot</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Ang sakyanan ni Juan kusog mokaon og gasolina, maong mahal kaayo ang gasto.; Ang iyang motor kusog mokaon og gasolina, pirmi lang magpailis.; Si Pedro ganahan ug sakyanan nga dili kusog mokaon og gasolina.; Ang mga tawo nga mag-drive ug sakyanan nga kusog mokaon og gasolina kasagaran maglisod sa gasto.; Si Maria dili ganahan ug sakyanan nga kusog mokaon og gasolina kay mahal ang maintenance.</t>
+          <t>Si Ana lupig pay ungo nga kalit lang nagpakita sa party.; Ang iyang kauban lupig pay ungo nga kalit lang moabot kung naay problema.; Si Pedro lupig pay ungo nga kalit lang makita sa mga event.; Ang mga tawo nga lupig pay ungo kasagaran maghatag ug katingalahan sa uban.; Si Juan lupig pay ungo nga kalit lang nagpakita sa ilang balay.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Ang sakyanan ni Juan kusog mokaon og gasolina, maong mahal kaayo ang gasto.; Ang iyang motor kusog mokaon og gasolina, pirmi lang magpailis.; Si Pedro ganahan ug sakyanan nga dili kusog mokaon og gasolina.; Ang mga tawo nga mag-drive ug sakyanan nga kusog mokaon og gasolina kasagaran maglisod sa gasto.; Si Maria dili ganahan ug sakyanan nga kusog mokaon og gasolina kay mahal ang maintenance.</t>
+          <t>Si Ana lupig pay ungo nga kalit lang nagpakita sa party.; Ang iyang kauban lupig pay ungo nga kalit lang moabot kung naay problema.; Si Pedro lupig pay ungo nga kalit lang makita sa mga event.; Ang mga tawo nga lupig pay ungo kasagaran maghatag ug katingalahan sa uban.; Si Juan lupig pay ungo nga kalit lang nagpakita sa ilang balay.</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>['mokaon']</t>
+          <t>['lupig']</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -3133,27 +3133,27 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>kuwang sa tagad</t>
+          <t>maabot sa luwa</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
+          <t>duol dili layo</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Si Ana kuwang sa tagad, maong pirmi lang magpahipi sa kanto.; Ang iyang kauban sa trabaho kuwang sa tagad, maong pirmi lang magpabida.; Si Pedro kuwang sa tagad, bisan unsa nga event ganahan magpakita.; Ang mga tawo nga kuwang sa tagad kasagaran magbuhat ug mga butang aron makuha ang atensyon.; Si Juan pirmi lang magpakita sa mga tao kay kuwang sa tagad.</t>
+          <t>Ang lugar nga ilang giadtoan kay maabot ra sa luwa, dili layo.; Ang iyang balay maabot ra sa luwa gikan sa simbahan.; Si Pedro pirmi lang maglakaw kay ang eskwelahan maabot ra sa luwa.; Ang mga tindahan nga ilang gusto adtoan kay maabot ra sa luwa gikan sa ilang lugar.; Si Maria nag-invite ug friends kay ilang balay maabot ra sa luwa.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Si Ana kuwang sa tagad, maong pirmi lang magpahipi sa kanto.; Ang iyang kauban sa trabaho kuwang sa tagad, maong pirmi lang magpabida.; Si Pedro kuwang sa tagad, bisan unsa nga event ganahan magpakita.; Ang mga tawo nga kuwang sa tagad kasagaran magbuhat ug mga butang aron makuha ang atensyon.; Si Juan pirmi lang magpakita sa mga tao kay kuwang sa tagad.</t>
+          <t>Ang lugar nga ilang giadtoan kay maabot ra sa luwa, dili layo.; Ang iyang balay maabot ra sa luwa gikan sa simbahan.; Si Pedro pirmi lang maglakaw kay ang eskwelahan maabot ra sa luwa.; Ang mga tindahan nga ilang gusto adtoan kay maabot ra sa luwa gikan sa ilang lugar.; Si Maria nag-invite ug friends kay ilang balay maabot ra sa luwa.</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>['tagad']</t>
+          <t>['maabot']</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -3163,27 +3163,27 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>kuyog baboy</t>
+          <t>mag-ihaw og lata</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>usa ka tagalong</t>
+          <t>sa pagluto sa mga pagkaon nga tinago</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Si Maria pirmi lang kuyog baboy, bisan asa moadto iyang best friend naa gyud.; Ang iyang igsuon kuyog baboy pirmi kung maglakaw-lakaw.; Si Pedro dili ganahan ug kuyog baboy kay samok kaayo.; Ang mga tawo nga kuyog baboy kasagaran magpalisod sa ilang mga kauban.; Si Juan pirmi lang kuyog baboy bisan unsa nga lakaw.</t>
+          <t>Si Ana pirmi lang mag-ihaw og lata kung walay sud-an.; Ang iyang pamilya mag-ihaw og lata kung walay kwarta.; Si Pedro mag-ihaw og lata kung walay luto nga pagkaon.; Ang mga estudyante kasagaran mag-ihaw og lata kung nagtipid.; Si Juan pirmi lang mag-ihaw og lata sa boarding house.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Si Maria pirmi lang kuyog baboy, bisan asa moadto iyang best friend naa gyud.; Ang iyang igsuon kuyog baboy pirmi kung maglakaw-lakaw.; Si Pedro dili ganahan ug kuyog baboy kay samok kaayo.; Ang mga tawo nga kuyog baboy kasagaran magpalisod sa ilang mga kauban.; Si Juan pirmi lang kuyog baboy bisan unsa nga lakaw.</t>
+          <t>Si Ana pirmi lang mag-ihaw og lata kung walay sud-an.; Ang iyang pamilya mag-ihaw og lata kung walay kwarta.; Si Pedro mag-ihaw og lata kung walay luto nga pagkaon.; Ang mga estudyante kasagaran mag-ihaw og lata kung nagtipid.; Si Juan pirmi lang mag-ihaw og lata sa boarding house.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>['kuyog']</t>
+          <t>['mag-ihaw']</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -3193,27 +3193,27 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>lapas na sa kalendaryo</t>
+          <t>mag-ugbok og mohon</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>usa ka tawo nga kapin sa 31 ka tuig ang edad</t>
+          <t>sa pagpakigsekso</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Si Ana lapas na sa kalendaryo, pero dili gihapon magminyo.; Ang iyang igsuon lapas na sa kalendaryo, pero dili gihapon magka-anak.; Si Pedro lapas na sa kalendaryo, pero wala gihapon trabaho.; Ang mga tawo nga lapas na sa kalendaryo kasagaran magpanikad sa ilang mga plano.; Si Juan lapas na sa kalendaryo, pero wala gihapon magtarong sa kinabuhi.</t>
+          <t>Si Pedro nagplano nga mag-ugbok og mohon human sa kasal.; Ang magtiayon nagdecide nga mag-ugbok og mohon sa ilang honeymoon.; Si Maria ug ang iyang bana mag-ugbok og mohon sa ilang balay.; Ang mga magtiayon nga mag-ugbok og mohon kasagaran magmalipay sa ilang relasyon.; Si Ana nagplano nga mag-ugbok og mohon sa iyang birthday.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Si Ana lapas na sa kalendaryo, pero dili gihapon magminyo.; Ang iyang igsuon lapas na sa kalendaryo, pero dili gihapon magka-anak.; Si Pedro lapas na sa kalendaryo, pero wala gihapon trabaho.; Ang mga tawo nga lapas na sa kalendaryo kasagaran magpanikad sa ilang mga plano.; Si Juan lapas na sa kalendaryo, pero wala gihapon magtarong sa kinabuhi.</t>
+          <t>Si Pedro nagplano nga mag-ugbok og mohon human sa kasal.; Ang magtiayon nagdecide nga mag-ugbok og mohon sa ilang honeymoon.; Si Maria ug ang iyang bana mag-ugbok og mohon sa ilang balay.; Ang mga magtiayon nga mag-ugbok og mohon kasagaran magmalipay sa ilang relasyon.; Si Ana nagplano nga mag-ugbok og mohon sa iyang birthday.</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>['lapas']</t>
+          <t>['mag-ugbok']</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -3223,27 +3223,27 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>lapos sa pikas dunggan</t>
+          <t>magbiko og pink</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>sa pagsulod sa usa ka dalunggan ug paggawas sa laing dalunggan</t>
+          <t>sa pagsaulog</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Ang tambag sa iyang ginikanan lapos ra sa pikas dunggan.; Si Pedro pirmi lang lapos sa pikas dunggan ang mga lectures sa eskwela.; Ang mga sugo sa iyang boss kay lapos ra sa pikas dunggan.; Ang mga tawo nga dili magtagad kasagaran maglapos ra sa pikas dunggan ang mga pulong sa uban.; Si Maria pirmi lang maglapos ra sa pikas dunggan ang mga tambag sa iyang mga amiga.</t>
+          <t>Si Pedro magbiko og pink sa iyang birthday.; Ang iyang amiga magbiko og pink sa ilang reunion.; Si Maria magbiko og pink sa ilang party sa balay.; Ang mga tawo nga magbiko og pink kasagaran maglipay sa ilang celebration.; Si Juan magbiko og pink sa iyang graduation.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Ang tambag sa iyang ginikanan lapos ra sa pikas dunggan.; Si Pedro pirmi lang lapos sa pikas dunggan ang mga lectures sa eskwela.; Ang mga sugo sa iyang boss kay lapos ra sa pikas dunggan.; Ang mga tawo nga dili magtagad kasagaran maglapos ra sa pikas dunggan ang mga pulong sa uban.; Si Maria pirmi lang maglapos ra sa pikas dunggan ang mga tambag sa iyang mga amiga.</t>
+          <t>Si Pedro magbiko og pink sa iyang birthday.; Ang iyang amiga magbiko og pink sa ilang reunion.; Si Maria magbiko og pink sa ilang party sa balay.; Ang mga tawo nga magbiko og pink kasagaran maglipay sa ilang celebration.; Si Juan magbiko og pink sa iyang graduation.</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>['lapos', 'dunggan']</t>
+          <t>['magbiko']</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -3253,27 +3253,27 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>litik</t>
+          <t>maghilak ang adlaw</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>sa pag-aghat sa tudlo</t>
+          <t>mabul-og</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Si Juan naglitik sa iyang mga kalagot sa iyang kauban.; Ang iyang anak naglitik ug sugilanon nga makalipay.; Si Pedro naglitik sa iyang mga plano sa negosyo.; Ang mga tawo nga naglitik sa ilang mga pangandoy kasagaran magmalampuson.; Si Maria naglitik sa iyang mga pangandoy sa kinabuhi.</t>
+          <t>Si Ana nagtan-aw sa bintana samtang naghilak ang adlaw.; Ang iyang pamilya nag-istorya samtang naghilak ang adlaw.; Si Pedro nagbasa ug libro samtang naghilak ang adlaw.; Ang mga tawo nag-relax sa balay samtang naghilak ang adlaw.; Si Juan naghunahuna sa iyang mga pangandoy samtang naghilak ang adlaw.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Si Juan naglitik sa iyang mga kalagot sa iyang kauban.; Ang iyang anak naglitik ug sugilanon nga makalipay.; Si Pedro naglitik sa iyang mga plano sa negosyo.; Ang mga tawo nga naglitik sa ilang mga pangandoy kasagaran magmalampuson.; Si Maria naglitik sa iyang mga pangandoy sa kinabuhi.</t>
+          <t>Si Ana nagtan-aw sa bintana samtang naghilak ang adlaw.; Ang iyang pamilya nag-istorya samtang naghilak ang adlaw.; Si Pedro nagbasa ug libro samtang naghilak ang adlaw.; Ang mga tawo nag-relax sa balay samtang naghilak ang adlaw.; Si Juan naghunahuna sa iyang mga pangandoy samtang naghilak ang adlaw.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>['litik']</t>
+          <t>['maghilak']</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -3283,27 +3283,27 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>lunod patay</t>
+          <t>magpalapad og papel</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>dihard</t>
+          <t>aron magbaton ug dungog sa buhat sa uban</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Si Pedro lunod patay sa iyang prinsipyo, dili gyud magbag-o.; Ang iyang amigo lunod patay sa iyang pagtuo bisan pa sa mga pagsulay.; Si Juan lunod patay sa pagsuporta sa iyang pamilya.; Ang mga tawo nga lunod patay kasagaran adunay baruganan nga dili matay-og.; Si Maria lunod patay sa pagpanalipod sa iyang mga kauban.</t>
+          <t>Si Pedro magpalapad og papel bisan dili siya ang nagbuhat sa proyekto.; Ang iyang kauban sa trabaho pirmi magpalapad og papel sa mga achievements sa uban.; Si Juan magpalapad og papel aron lang makakuha ug promotion.; Ang mga tawo nga magpalapad og papel kasagaran dili tinood nga maayong magtrabaho.; Si Maria magpalapad og papel bisan dili siya ang nagtrabaho sa project.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Si Pedro lunod patay sa iyang prinsipyo, dili gyud magbag-o.; Ang iyang amigo lunod patay sa iyang pagtuo bisan pa sa mga pagsulay.; Si Juan lunod patay sa pagsuporta sa iyang pamilya.; Ang mga tawo nga lunod patay kasagaran adunay baruganan nga dili matay-og.; Si Maria lunod patay sa pagpanalipod sa iyang mga kauban.</t>
+          <t>Si Pedro magpalapad og papel bisan dili siya ang nagbuhat sa proyekto.; Ang iyang kauban sa trabaho pirmi magpalapad og papel sa mga achievements sa uban.; Si Juan magpalapad og papel aron lang makakuha ug promotion.; Ang mga tawo nga magpalapad og papel kasagaran dili tinood nga maayong magtrabaho.; Si Maria magpalapad og papel bisan dili siya ang nagtrabaho sa project.</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>['lunod', 'patay']</t>
+          <t>['magpalapad']</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -3313,27 +3313,27 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>lupig pay ungo</t>
+          <t>magtumba og baka</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga wala damha moabot</t>
+          <t>sa pag-ihaw sa usa ka vaca</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Si Ana lupig pay ungo nga kalit lang nagpakita sa party.; Ang iyang kauban lupig pay ungo nga kalit lang moabot kung naay problema.; Si Pedro lupig pay ungo nga kalit lang makita sa mga event.; Ang mga tawo nga lupig pay ungo kasagaran maghatag ug katingalahan sa uban.; Si Juan lupig pay ungo nga kalit lang nagpakita sa ilang balay.</t>
+          <t>Si Pedro magtumba og baka para sa fiesta sa ilang baryo.; Ang ilang pamilya magtumba og baka kung naa’y dako nga celebration.; Si Juan nagplano nga magtumba og baka para sa birthday sa iyang anak.; Ang mga tawo nga magtumba og baka kasagaran nagselebrar ug dako nga event.; Si Maria nalipay kay magtumba og baka ang iyang pamilya para sa pasko.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Si Ana lupig pay ungo nga kalit lang nagpakita sa party.; Ang iyang kauban lupig pay ungo nga kalit lang moabot kung naay problema.; Si Pedro lupig pay ungo nga kalit lang makita sa mga event.; Ang mga tawo nga lupig pay ungo kasagaran maghatag ug katingalahan sa uban.; Si Juan lupig pay ungo nga kalit lang nagpakita sa ilang balay.</t>
+          <t>Si Pedro magtumba og baka para sa fiesta sa ilang baryo.; Ang ilang pamilya magtumba og baka kung naa’y dako nga celebration.; Si Juan nagplano nga magtumba og baka para sa birthday sa iyang anak.; Ang mga tawo nga magtumba og baka kasagaran nagselebrar ug dako nga event.; Si Maria nalipay kay magtumba og baka ang iyang pamilya para sa pasko.</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>['lupig']</t>
+          <t>['magtumba']</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -3343,27 +3343,27 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>maabot sa luwa</t>
+          <t>maibtan sa tunok</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>duol dili layo</t>
+          <t>aron mapugngan ang pag-antos o kabalaka</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Ang lugar nga ilang giadtoan kay maabot ra sa luwa, dili layo.; Ang iyang balay maabot ra sa luwa gikan sa simbahan.; Si Pedro pirmi lang maglakaw kay ang eskwelahan maabot ra sa luwa.; Ang mga tindahan nga ilang gusto adtoan kay maabot ra sa luwa gikan sa ilang lugar.; Si Maria nag-invite ug friends kay ilang balay maabot ra sa luwa.</t>
+          <t>Si Ana maibtan sa tunok human siya makapasar sa board exam.; Ang iyang pamilya maibtan sa tunok human makabayad sa ilang utang.; Si Pedro maibtan sa tunok human ma-clear ang iyang pangalan sa kaso.; Ang mga tawo nga maibtan sa tunok kasagaran magmalipay ug magrelax.; Si Maria maibtan sa tunok human magkauli ang ilang pamilya.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Ang lugar nga ilang giadtoan kay maabot ra sa luwa, dili layo.; Ang iyang balay maabot ra sa luwa gikan sa simbahan.; Si Pedro pirmi lang maglakaw kay ang eskwelahan maabot ra sa luwa.; Ang mga tindahan nga ilang gusto adtoan kay maabot ra sa luwa gikan sa ilang lugar.; Si Maria nag-invite ug friends kay ilang balay maabot ra sa luwa.</t>
+          <t>Si Ana maibtan sa tunok human siya makapasar sa board exam.; Ang iyang pamilya maibtan sa tunok human makabayad sa ilang utang.; Si Pedro maibtan sa tunok human ma-clear ang iyang pangalan sa kaso.; Ang mga tawo nga maibtan sa tunok kasagaran magmalipay ug magrelax.; Si Maria maibtan sa tunok human magkauli ang ilang pamilya.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>['maabot']</t>
+          <t>['maibtan']</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -3373,27 +3373,27 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>mag-ihaw og lata</t>
+          <t>makabugto og bra</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>sa pagluto sa mga pagkaon nga tinago</t>
+          <t>pisikal o seksuwal nga madanihon</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang mag-ihaw og lata kung walay sud-an.; Ang iyang pamilya mag-ihaw og lata kung walay kwarta.; Si Pedro mag-ihaw og lata kung walay luto nga pagkaon.; Ang mga estudyante kasagaran mag-ihaw og lata kung nagtipid.; Si Juan pirmi lang mag-ihaw og lata sa boarding house.</t>
+          <t>Si Pedro makabugto og bra tungod sa iyang pagka-sexy.; Ang artista nga iyang nakita sa TV makabugto og bra gyud.; Si Juan ganahan kaayo sa iyang uyab kay makabugto og bra.; Ang mga modelo sa magazine kasagaran makabugto og bra sa ilang porma.; Si Maria makaingon nga makabugto og bra ang iyang crush.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Si Ana pirmi lang mag-ihaw og lata kung walay sud-an.; Ang iyang pamilya mag-ihaw og lata kung walay kwarta.; Si Pedro mag-ihaw og lata kung walay luto nga pagkaon.; Ang mga estudyante kasagaran mag-ihaw og lata kung nagtipid.; Si Juan pirmi lang mag-ihaw og lata sa boarding house.</t>
+          <t>Si Pedro makabugto og bra tungod sa iyang pagka-sexy.; Ang artista nga iyang nakita sa TV makabugto og bra gyud.; Si Juan ganahan kaayo sa iyang uyab kay makabugto og bra.; Ang mga modelo sa magazine kasagaran makabugto og bra sa ilang porma.; Si Maria makaingon nga makabugto og bra ang iyang crush.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>['mag-ihaw']</t>
+          <t>['makabugto']</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -3403,27 +3403,27 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>mag-ugbok og mohon</t>
+          <t>makabugto og panty</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>sa pagpakigsekso</t>
+          <t>pisikal o seksuwal nga madanihon</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Si Pedro nagplano nga mag-ugbok og mohon human sa kasal.; Ang magtiayon nagdecide nga mag-ugbok og mohon sa ilang honeymoon.; Si Maria ug ang iyang bana mag-ugbok og mohon sa ilang balay.; Ang mga magtiayon nga mag-ugbok og mohon kasagaran magmalipay sa ilang relasyon.; Si Ana nagplano nga mag-ugbok og mohon sa iyang birthday.</t>
+          <t>Si Ana makabugto og panty sa iyang pagka-sexy.; Ang artista nga iyang nakita sa sine makabugto og panty gyud.; Si Pedro ganahan kaayo sa iyang uyab kay makabugto og panty.; Ang mga modelo sa fashion show kasagaran makabugto og panty sa ilang porma.; Si Maria makaingon nga makabugto og panty ang iyang crush.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Si Pedro nagplano nga mag-ugbok og mohon human sa kasal.; Ang magtiayon nagdecide nga mag-ugbok og mohon sa ilang honeymoon.; Si Maria ug ang iyang bana mag-ugbok og mohon sa ilang balay.; Ang mga magtiayon nga mag-ugbok og mohon kasagaran magmalipay sa ilang relasyon.; Si Ana nagplano nga mag-ugbok og mohon sa iyang birthday.</t>
+          <t>Si Ana makabugto og panty sa iyang pagka-sexy.; Ang artista nga iyang nakita sa sine makabugto og panty gyud.; Si Pedro ganahan kaayo sa iyang uyab kay makabugto og panty.; Ang mga modelo sa fashion show kasagaran makabugto og panty sa ilang porma.; Si Maria makaingon nga makabugto og panty ang iyang crush.</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>['mag-ugbok']</t>
+          <t>['makabugto']</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -3433,27 +3433,27 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>magbiko og pink</t>
+          <t>makabuhi og patay</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>sa pagsaulog</t>
+          <t>usa ka makapatikod nga bakak o sugilanon</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Si Pedro magbiko og pink sa iyang birthday.; Ang iyang amiga magbiko og pink sa ilang reunion.; Si Maria magbiko og pink sa ilang party sa balay.; Ang mga tawo nga magbiko og pink kasagaran maglipay sa ilang celebration.; Si Juan magbiko og pink sa iyang graduation.</t>
+          <t>Si Juan makabuhi og patay sa iyang mga istorya.; Ang iyang amigo makabuhi og patay kung mag-suggest ug ideas.; Si Pedro makabuhi og patay sa iyang mga jokes.; Ang mga tawo nga makabuhi og patay kasagaran maayo kaayo moistorya.; Si Maria makabuhi og patay kung mag-explain sa iyang mga pangandoy.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Si Pedro magbiko og pink sa iyang birthday.; Ang iyang amiga magbiko og pink sa ilang reunion.; Si Maria magbiko og pink sa ilang party sa balay.; Ang mga tawo nga magbiko og pink kasagaran maglipay sa ilang celebration.; Si Juan magbiko og pink sa iyang graduation.</t>
+          <t>Si Juan makabuhi og patay sa iyang mga istorya.; Ang iyang amigo makabuhi og patay kung mag-suggest ug ideas.; Si Pedro makabuhi og patay sa iyang mga jokes.; Ang mga tawo nga makabuhi og patay kasagaran maayo kaayo moistorya.; Si Maria makabuhi og patay kung mag-explain sa iyang mga pangandoy.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>['magbiko']</t>
+          <t>['makabuhi', 'patay']</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -3463,27 +3463,27 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>maghilak ang adlaw</t>
+          <t>makagisi og pitaka</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>mabul-og</t>
+          <t>mahal kaayo</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Si Ana nagtan-aw sa bintana samtang naghilak ang adlaw.; Ang iyang pamilya nag-istorya samtang naghilak ang adlaw.; Si Pedro nagbasa ug libro samtang naghilak ang adlaw.; Ang mga tawo nag-relax sa balay samtang naghilak ang adlaw.; Si Juan naghunahuna sa iyang mga pangandoy samtang naghilak ang adlaw.</t>
+          <t>Ang restaurant nga ilang giadtoan makagisi og pitaka kaayo.; Ang iyang bag-ong sapatos makagisi og pitaka tungod sa kamahal.; Si Pedro nagreklamo kay ang tuition fee sa eskwelahan makagisi og pitaka.; Ang mga luxury items kasagaran makagisi og pitaka sa ilang presyo.; Si Maria nakapalit ug bag nga makagisi og pitaka tungod sa kamahal.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Si Ana nagtan-aw sa bintana samtang naghilak ang adlaw.; Ang iyang pamilya nag-istorya samtang naghilak ang adlaw.; Si Pedro nagbasa ug libro samtang naghilak ang adlaw.; Ang mga tawo nag-relax sa balay samtang naghilak ang adlaw.; Si Juan naghunahuna sa iyang mga pangandoy samtang naghilak ang adlaw.</t>
+          <t>Ang restaurant nga ilang giadtoan makagisi og pitaka kaayo.; Ang iyang bag-ong sapatos makagisi og pitaka tungod sa kamahal.; Si Pedro nagreklamo kay ang tuition fee sa eskwelahan makagisi og pitaka.; Ang mga luxury items kasagaran makagisi og pitaka sa ilang presyo.; Si Maria nakapalit ug bag nga makagisi og pitaka tungod sa kamahal.</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>['maghilak']</t>
+          <t>['makagisi']</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -3493,27 +3493,27 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>magpalapad og papel</t>
+          <t>makakutaw og utok</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>aron magbaton ug dungog sa buhat sa uban</t>
+          <t>makapalibog</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Si Pedro magpalapad og papel bisan dili siya ang nagbuhat sa proyekto.; Ang iyang kauban sa trabaho pirmi magpalapad og papel sa mga achievements sa uban.; Si Juan magpalapad og papel aron lang makakuha ug promotion.; Ang mga tawo nga magpalapad og papel kasagaran dili tinood nga maayong magtrabaho.; Si Maria magpalapad og papel bisan dili siya ang nagtrabaho sa project.</t>
+          <t>Ang math problems nga iyang gi-atubang makakutaw og utok gyud.; Ang explanation sa iyang professor makakutaw og utok kaayo.; Si Pedro naglibog kay ang project makakutaw og utok.; Ang mga puzzles nga iyang gi-solve makakutaw og utok kaayo.; Si Maria nagreklamo kay ang instructions makakutaw og utok.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Si Pedro magpalapad og papel bisan dili siya ang nagbuhat sa proyekto.; Ang iyang kauban sa trabaho pirmi magpalapad og papel sa mga achievements sa uban.; Si Juan magpalapad og papel aron lang makakuha ug promotion.; Ang mga tawo nga magpalapad og papel kasagaran dili tinood nga maayong magtrabaho.; Si Maria magpalapad og papel bisan dili siya ang nagtrabaho sa project.</t>
+          <t>Ang math problems nga iyang gi-atubang makakutaw og utok gyud.; Ang explanation sa iyang professor makakutaw og utok kaayo.; Si Pedro naglibog kay ang project makakutaw og utok.; Ang mga puzzles nga iyang gi-solve makakutaw og utok kaayo.; Si Maria nagreklamo kay ang instructions makakutaw og utok.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>['magpalapad']</t>
+          <t>['makakutaw']</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -3523,27 +3523,27 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>magtumba og baka</t>
+          <t>makamala og sapa</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>sa pag-ihaw sa usa ka vaca</t>
+          <t>ang usa ka tawo nga may dagkong tiil</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Si Pedro magtumba og baka para sa fiesta sa ilang baryo.; Ang ilang pamilya magtumba og baka kung naa’y dako nga celebration.; Si Juan nagplano nga magtumba og baka para sa birthday sa iyang anak.; Ang mga tawo nga magtumba og baka kasagaran nagselebrar ug dako nga event.; Si Maria nalipay kay magtumba og baka ang iyang pamilya para sa pasko.</t>
+          <t>Si Juan makamala og sapa sa iyang mga tiil.; Ang iyang amigo makamala og sapa tungod sa kadako sa tiil.; Si Pedro makamala og sapa kay grabe kaayo kadako ang tiil.; Ang mga tawo nga dagko ug tiil kasagaran makamala og sapa.; Si Maria nagkatawa kay ang iyang igsuon makamala og sapa sa kadako sa tiil.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Si Pedro magtumba og baka para sa fiesta sa ilang baryo.; Ang ilang pamilya magtumba og baka kung naa’y dako nga celebration.; Si Juan nagplano nga magtumba og baka para sa birthday sa iyang anak.; Ang mga tawo nga magtumba og baka kasagaran nagselebrar ug dako nga event.; Si Maria nalipay kay magtumba og baka ang iyang pamilya para sa pasko.</t>
+          <t>Si Juan makamala og sapa sa iyang mga tiil.; Ang iyang amigo makamala og sapa tungod sa kadako sa tiil.; Si Pedro makamala og sapa kay grabe kaayo kadako ang tiil.; Ang mga tawo nga dagko ug tiil kasagaran makamala og sapa.; Si Maria nagkatawa kay ang iyang igsuon makamala og sapa sa kadako sa tiil.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>['magtumba']</t>
+          <t>['makamala']</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -3553,27 +3553,27 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>maibtan sa tunok</t>
+          <t>makawat</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>aron mapugngan ang pag-antos o kabalaka</t>
+          <t>mahimong ma-stolen</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Si Ana maibtan sa tunok human siya makapasar sa board exam.; Ang iyang pamilya maibtan sa tunok human makabayad sa ilang utang.; Si Pedro maibtan sa tunok human ma-clear ang iyang pangalan sa kaso.; Ang mga tawo nga maibtan sa tunok kasagaran magmalipay ug magrelax.; Si Maria maibtan sa tunok human magkauli ang ilang pamilya.</t>
+          <t>Ang bata ni Maria makawat kaayo, bisan kinsa lang pwede makagunit niya.; Si Pedro makawat kaayo, dali ra siya madala bisan kinsa.; Ang anak ni Juan makawat, bisan kinsa ra magpadede niya.; Si Ana makawat nga bata, dili siya mohilak bisan kinsa ang magbitbit.; Ang ilang baby makawat kaayo, bisan kinsa nga tawo dili niya kahadlukan.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Si Ana maibtan sa tunok human siya makapasar sa board exam.; Ang iyang pamilya maibtan sa tunok human makabayad sa ilang utang.; Si Pedro maibtan sa tunok human ma-clear ang iyang pangalan sa kaso.; Ang mga tawo nga maibtan sa tunok kasagaran magmalipay ug magrelax.; Si Maria maibtan sa tunok human magkauli ang ilang pamilya.</t>
+          <t>Ang bata ni Maria makawat kaayo, bisan kinsa lang pwede makagunit niya.; Si Pedro makawat kaayo, dali ra siya madala bisan kinsa.; Ang anak ni Juan makawat, bisan kinsa ra magpadede niya.; Si Ana makawat nga bata, dili siya mohilak bisan kinsa ang magbitbit.; Ang ilang baby makawat kaayo, bisan kinsa nga tawo dili niya kahadlukan.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>['maibtan']</t>
+          <t>['makawat']</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -3583,27 +3583,27 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>makabugto og bra</t>
+          <t>maliso pay buko sa kawayan</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>pisikal o seksuwal nga madanihon</t>
+          <t>dili mausab</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Si Pedro makabugto og bra tungod sa iyang pagka-sexy.; Ang artista nga iyang nakita sa TV makabugto og bra gyud.; Si Juan ganahan kaayo sa iyang uyab kay makabugto og bra.; Ang mga modelo sa magazine kasagaran makabugto og bra sa ilang porma.; Si Maria makaingon nga makabugto og bra ang iyang crush.</t>
+          <t>Ang batasan ni Pedro maliso pay buko sa kawayan, dili gyud siya magbag-o.; Ang iyang pagtuo maliso pay buko sa kawayan, dili gyud mausab.; Si Juan maliso pay buko sa kawayan ang iyang determinasyon sa paghuman sa iyang kurso.; Ang iyang kauban sa trabaho maliso pay buko sa kawayan sa pagka-strikto.; Si Maria maliso pay buko sa kawayan ang iyang pagtuo sa Diyos.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Si Pedro makabugto og bra tungod sa iyang pagka-sexy.; Ang artista nga iyang nakita sa TV makabugto og bra gyud.; Si Juan ganahan kaayo sa iyang uyab kay makabugto og bra.; Ang mga modelo sa magazine kasagaran makabugto og bra sa ilang porma.; Si Maria makaingon nga makabugto og bra ang iyang crush.</t>
+          <t>Ang batasan ni Pedro maliso pay buko sa kawayan, dili gyud siya magbag-o.; Ang iyang pagtuo maliso pay buko sa kawayan, dili gyud mausab.; Si Juan maliso pay buko sa kawayan ang iyang determinasyon sa paghuman sa iyang kurso.; Ang iyang kauban sa trabaho maliso pay buko sa kawayan sa pagka-strikto.; Si Maria maliso pay buko sa kawayan ang iyang pagtuo sa Diyos.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>['makabugto']</t>
+          <t>['maliso']</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -3613,27 +3613,27 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>makabugto og panty</t>
+          <t>mamalit og kaso</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>pisikal o seksuwal nga madanihon</t>
+          <t>aron mahimong usa ka ambulance chaser</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Si Ana makabugto og panty sa iyang pagka-sexy.; Ang artista nga iyang nakita sa sine makabugto og panty gyud.; Si Pedro ganahan kaayo sa iyang uyab kay makabugto og panty.; Ang mga modelo sa fashion show kasagaran makabugto og panty sa ilang porma.; Si Maria makaingon nga makabugto og panty ang iyang crush.</t>
+          <t>Si Ana mamalit og kaso aron lang magka-datu.; Ang abogado mamalit og kaso bisan asa nga hospital.; Si Pedro mamalit og kaso aron makakwarta sa mga biktima sa aksidente.; Ang mga tawo nga mamalit og kaso kasagaran mga abogado nga gustong magpasikat.; Si Juan mamalit og kaso aron lang magka-daghan ang iyang kliyente.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Si Ana makabugto og panty sa iyang pagka-sexy.; Ang artista nga iyang nakita sa sine makabugto og panty gyud.; Si Pedro ganahan kaayo sa iyang uyab kay makabugto og panty.; Ang mga modelo sa fashion show kasagaran makabugto og panty sa ilang porma.; Si Maria makaingon nga makabugto og panty ang iyang crush.</t>
+          <t>Si Ana mamalit og kaso aron lang magka-datu.; Ang abogado mamalit og kaso bisan asa nga hospital.; Si Pedro mamalit og kaso aron makakwarta sa mga biktima sa aksidente.; Ang mga tawo nga mamalit og kaso kasagaran mga abogado nga gustong magpasikat.; Si Juan mamalit og kaso aron lang magka-daghan ang iyang kliyente.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>['makabugto']</t>
+          <t>['mamalit']</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -3643,27 +3643,27 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>makabuhi og patay</t>
+          <t>manakop og ligid</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>usa ka makapatikod nga bakak o sugilanon</t>
+          <t>nga ang usa ka tawo naugtang sa usa ka sakyanan</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Si Juan makabuhi og patay sa iyang mga istorya.; Ang iyang amigo makabuhi og patay kung mag-suggest ug ideas.; Si Pedro makabuhi og patay sa iyang mga jokes.; Ang mga tawo nga makabuhi og patay kasagaran maayo kaayo moistorya.; Si Maria makabuhi og patay kung mag-explain sa iyang mga pangandoy.</t>
+          <t>Si Ana nasuko kay siya manakop og ligid tungod sa iyang pagkadula.; Ang iyang kauban sa trabaho pirmi lang manakop og ligid kay walay tarong nga pag-amping.; Si Pedro manakop og ligid kay nagdagan-dagan sa kalsada.; Ang mga tawo nga dili mag-amping sa dalan kasagaran manakop og ligid.; Si Juan nakasulay nga manakop og ligid human nag-away sa iyang amigo.; "Ayaw pag manakop og ligid, klaroha imong gibuhat."; "Manakop og ligid kaayo imong mga plano, walay klaro."; "Si Pedro, manakop og ligid ug walay klaro."; "Ayaw pag manakop og ligid, siguroha imong mga desisyon."; "Manakop og ligid imong mga ideas, kinahanglan pa nimo ug focus."</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Si Juan makabuhi og patay sa iyang mga istorya.; Ang iyang amigo makabuhi og patay kung mag-suggest ug ideas.; Si Pedro makabuhi og patay sa iyang mga jokes.; Ang mga tawo nga makabuhi og patay kasagaran maayo kaayo moistorya.; Si Maria makabuhi og patay kung mag-explain sa iyang mga pangandoy.</t>
+          <t>Si Ana nasuko kay siya manakop og ligid tungod sa iyang pagkadula.; Ang iyang kauban sa trabaho pirmi lang manakop og ligid kay walay tarong nga pag-amping.; Si Pedro manakop og ligid kay nagdagan-dagan sa kalsada.; Ang mga tawo nga dili mag-amping sa dalan kasagaran manakop og ligid.; Si Juan nakasulay nga manakop og ligid human nag-away sa iyang amigo.; "Ayaw pag manakop og ligid, klaroha imong gibuhat."; "Manakop og ligid kaayo imong mga plano, walay klaro."; "Si Pedro, manakop og ligid ug walay klaro."; "Ayaw pag manakop og ligid, siguroha imong mga desisyon."; "Manakop og ligid imong mga ideas, kinahanglan pa nimo ug focus."</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>['makabuhi', 'patay']</t>
+          <t>['manakop']</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -3673,27 +3673,27 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>makagisi og pitaka</t>
+          <t>mangayo og manghod</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>mahal kaayo</t>
+          <t>usa ka kaso sa bata nga nag-asuso o nag-agom sa iyang mga tudlo</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Ang restaurant nga ilang giadtoan makagisi og pitaka kaayo.; Ang iyang bag-ong sapatos makagisi og pitaka tungod sa kamahal.; Si Pedro nagreklamo kay ang tuition fee sa eskwelahan makagisi og pitaka.; Ang mga luxury items kasagaran makagisi og pitaka sa ilang presyo.; Si Maria nakapalit ug bag nga makagisi og pitaka tungod sa kamahal.</t>
+          <t>Si Ana pirmi mangayo og manghod kung magdula.; Ang iyang anak mangayo og manghod kung gutom na.; Si Pedro nakakita sa iyang anak nga mangayo og manghod sa iyang tiil.; Ang mga bata nga mangayo og manghod kasagaran mga healthy nga bata.; Si Juan nalipay kay ang iyang baby nakakat-on nga mangayo og manghod.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Ang restaurant nga ilang giadtoan makagisi og pitaka kaayo.; Ang iyang bag-ong sapatos makagisi og pitaka tungod sa kamahal.; Si Pedro nagreklamo kay ang tuition fee sa eskwelahan makagisi og pitaka.; Ang mga luxury items kasagaran makagisi og pitaka sa ilang presyo.; Si Maria nakapalit ug bag nga makagisi og pitaka tungod sa kamahal.</t>
+          <t>Si Ana pirmi mangayo og manghod kung magdula.; Ang iyang anak mangayo og manghod kung gutom na.; Si Pedro nakakita sa iyang anak nga mangayo og manghod sa iyang tiil.; Ang mga bata nga mangayo og manghod kasagaran mga healthy nga bata.; Si Juan nalipay kay ang iyang baby nakakat-on nga mangayo og manghod.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>['makagisi']</t>
+          <t>['mangayo']</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -3703,27 +3703,27 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>makakutaw og utok</t>
+          <t>manglutasay</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>makapalibog</t>
+          <t>usa ka manunulak sa mga bukog</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Ang math problems nga iyang gi-atubang makakutaw og utok gyud.; Ang explanation sa iyang professor makakutaw og utok kaayo.; Si Pedro naglibog kay ang project makakutaw og utok.; Ang mga puzzles nga iyang gi-solve makakutaw og utok kaayo.; Si Maria nagreklamo kay ang instructions makakutaw og utok.</t>
+          <t>Si Pedro pirmi manglutasay ug uyab nga mga batan-on.; Ang iyang kauban sa trabaho manglutasay sa mga kabataan.; Si Juan giingnan nga manglutasay kay ang iyang uyab mas bata kaayo.; Ang mga tawo nga manglutasay kasagaran magkatawa sa ilang kalaki.; Si Maria nalipay kay ang iyang kauban dili manglutasay.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Ang math problems nga iyang gi-atubang makakutaw og utok gyud.; Ang explanation sa iyang professor makakutaw og utok kaayo.; Si Pedro naglibog kay ang project makakutaw og utok.; Ang mga puzzles nga iyang gi-solve makakutaw og utok kaayo.; Si Maria nagreklamo kay ang instructions makakutaw og utok.</t>
+          <t>Si Pedro pirmi manglutasay ug uyab nga mga batan-on.; Ang iyang kauban sa trabaho manglutasay sa mga kabataan.; Si Juan giingnan nga manglutasay kay ang iyang uyab mas bata kaayo.; Ang mga tawo nga manglutasay kasagaran magkatawa sa ilang kalaki.; Si Maria nalipay kay ang iyang kauban dili manglutasay.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>['makakutaw']</t>
+          <t>['manglutasay']</t>
         </is>
       </c>
       <c r="F110" t="n">
@@ -3733,27 +3733,27 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>makamala og sapa</t>
+          <t>mangnukos</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga may dagkong tiil</t>
+          <t>sa pag-abli sa usa ka pista</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Si Juan makamala og sapa sa iyang mga tiil.; Ang iyang amigo makamala og sapa tungod sa kadako sa tiil.; Si Pedro makamala og sapa kay grabe kaayo kadako ang tiil.; Ang mga tawo nga dagko ug tiil kasagaran makamala og sapa.; Si Maria nagkatawa kay ang iyang igsuon makamala og sapa sa kadako sa tiil.</t>
+          <t>Si Ana nalipay kay ang iyang kauban dili mangnukos sa mga event.; Ang iyang kauban sa trabaho pirmi lang mangnukos sa mga party.; Si Pedro mangnukos sa mga events nga walay imbitasyon.; Ang mga tawo nga mangnukos kasagaran magpahimulos sa libre nga pagkaon.; Si Juan giingnan nga dili mangnukos sa party sa iyang amiga.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Si Juan makamala og sapa sa iyang mga tiil.; Ang iyang amigo makamala og sapa tungod sa kadako sa tiil.; Si Pedro makamala og sapa kay grabe kaayo kadako ang tiil.; Ang mga tawo nga dagko ug tiil kasagaran makamala og sapa.; Si Maria nagkatawa kay ang iyang igsuon makamala og sapa sa kadako sa tiil.</t>
+          <t>Si Ana nalipay kay ang iyang kauban dili mangnukos sa mga event.; Ang iyang kauban sa trabaho pirmi lang mangnukos sa mga party.; Si Pedro mangnukos sa mga events nga walay imbitasyon.; Ang mga tawo nga mangnukos kasagaran magpahimulos sa libre nga pagkaon.; Si Juan giingnan nga dili mangnukos sa party sa iyang amiga.</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>['makamala']</t>
+          <t>['mangnukos']</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -3763,27 +3763,27 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>makawat</t>
+          <t>manira sa dalan</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>mahimong ma-stolen</t>
+          <t>aron magpabilin nga magmata hangtod sa gabii</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Ang bata ni Maria makawat kaayo, bisan kinsa lang pwede makagunit niya.; Si Pedro makawat kaayo, dali ra siya madala bisan kinsa.; Ang anak ni Juan makawat, bisan kinsa ra magpadede niya.; Si Ana makawat nga bata, dili siya mohilak bisan kinsa ang magbitbit.; Ang ilang baby makawat kaayo, bisan kinsa nga tawo dili niya kahadlukan.</t>
+          <t>Si Pedro pirmi manira sa dalan kada gabii.; Ang iyang barkada manira sa dalan hangtud sa kaadlawon.; Si Juan manira sa dalan kung walay klase.; Ang mga batan-on kasagaran manira sa dalan kung walay lingaw.; Si Maria ug ang iyang mga amiga manira sa dalan human sa trabaho.; "Ayaw pag manira sa dalan, naa pa kay buhaton."; "Si Ana, sige lang manira sa dalan walay klaro."; "Manira sa dalan imong mga plano, walay padulngan."; "Ayaw pag manira sa dalan, klaroha imong mga desisyon."; "Manira sa dalan kaayo ka, kinahanglan pa nimo ug focus."</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Ang bata ni Maria makawat kaayo, bisan kinsa lang pwede makagunit niya.; Si Pedro makawat kaayo, dali ra siya madala bisan kinsa.; Ang anak ni Juan makawat, bisan kinsa ra magpadede niya.; Si Ana makawat nga bata, dili siya mohilak bisan kinsa ang magbitbit.; Ang ilang baby makawat kaayo, bisan kinsa nga tawo dili niya kahadlukan.</t>
+          <t>Si Pedro pirmi manira sa dalan kada gabii.; Ang iyang barkada manira sa dalan hangtud sa kaadlawon.; Si Juan manira sa dalan kung walay klase.; Ang mga batan-on kasagaran manira sa dalan kung walay lingaw.; Si Maria ug ang iyang mga amiga manira sa dalan human sa trabaho.; "Ayaw pag manira sa dalan, naa pa kay buhaton."; "Si Ana, sige lang manira sa dalan walay klaro."; "Manira sa dalan imong mga plano, walay padulngan."; "Ayaw pag manira sa dalan, klaroha imong mga desisyon."; "Manira sa dalan kaayo ka, kinahanglan pa nimo ug focus."</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>['makawat']</t>
+          <t>['manira']</t>
         </is>
       </c>
       <c r="F112" t="n">
@@ -3793,27 +3793,27 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>maliso pay buko sa kawayan</t>
+          <t>may tawo na ang payag</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>dili mausab</t>
+          <t>alang sa usa ka babaye nga adunay higugmaon</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Ang batasan ni Pedro maliso pay buko sa kawayan, dili gyud siya magbag-o.; Ang iyang pagtuo maliso pay buko sa kawayan, dili gyud mausab.; Si Juan maliso pay buko sa kawayan ang iyang determinasyon sa paghuman sa iyang kurso.; Ang iyang kauban sa trabaho maliso pay buko sa kawayan sa pagka-strikto.; Si Maria maliso pay buko sa kawayan ang iyang pagtuo sa Diyos.</t>
+          <t>Si Ana dili na pwede uyabon kay may tawo na ang payag.; Ang iyang crush may tawo na ang payag, mao nga dili na siya magpursige.; Si Pedro naay gipanguyaban nga may tawo na ang payag.; Ang mga batan-on kasagaran dili na mangita ug uyab kung may tawo na ang payag.; Si Maria niingon nga may tawo na ang payag mao nga dili siya ganahan sa uban.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Ang batasan ni Pedro maliso pay buko sa kawayan, dili gyud siya magbag-o.; Ang iyang pagtuo maliso pay buko sa kawayan, dili gyud mausab.; Si Juan maliso pay buko sa kawayan ang iyang determinasyon sa paghuman sa iyang kurso.; Ang iyang kauban sa trabaho maliso pay buko sa kawayan sa pagka-strikto.; Si Maria maliso pay buko sa kawayan ang iyang pagtuo sa Diyos.</t>
+          <t>Si Ana dili na pwede uyabon kay may tawo na ang payag.; Ang iyang crush may tawo na ang payag, mao nga dili na siya magpursige.; Si Pedro naay gipanguyaban nga may tawo na ang payag.; Ang mga batan-on kasagaran dili na mangita ug uyab kung may tawo na ang payag.; Si Maria niingon nga may tawo na ang payag mao nga dili siya ganahan sa uban.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>['maliso']</t>
+          <t>['may']</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -3823,27 +3823,27 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>mamalit og kaso</t>
+          <t>miulbo ang kaspa</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>aron mahimong usa ka ambulance chaser</t>
+          <t>sa pag-abli ngadto sa kasuko</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Si Ana mamalit og kaso aron lang magka-datu.; Ang abogado mamalit og kaso bisan asa nga hospital.; Si Pedro mamalit og kaso aron makakwarta sa mga biktima sa aksidente.; Ang mga tawo nga mamalit og kaso kasagaran mga abogado nga gustong magpasikat.; Si Juan mamalit og kaso aron lang magka-daghan ang iyang kliyente.</t>
+          <t>Si Ana miulbo ang kaspa human nabal-an nga gilimbongan siya.; Ang iyang boss miulbo ang kaspa tungod sa sayop nga trabaho.; Si Pedro miulbo ang kaspa human naay nakig-away niya.; Ang mga tawo nga dali masuko kasagaran miulbo ang kaspa sa gamay nga rason.; Si Maria miulbo ang kaspa kay wala siya natagaan ug hustisya.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Si Ana mamalit og kaso aron lang magka-datu.; Ang abogado mamalit og kaso bisan asa nga hospital.; Si Pedro mamalit og kaso aron makakwarta sa mga biktima sa aksidente.; Ang mga tawo nga mamalit og kaso kasagaran mga abogado nga gustong magpasikat.; Si Juan mamalit og kaso aron lang magka-daghan ang iyang kliyente.</t>
+          <t>Si Ana miulbo ang kaspa human nabal-an nga gilimbongan siya.; Ang iyang boss miulbo ang kaspa tungod sa sayop nga trabaho.; Si Pedro miulbo ang kaspa human naay nakig-away niya.; Ang mga tawo nga dali masuko kasagaran miulbo ang kaspa sa gamay nga rason.; Si Maria miulbo ang kaspa kay wala siya natagaan ug hustisya.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>['mamalit']</t>
+          <t>['miulbo']</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -3853,27 +3853,27 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>manakop og ligid</t>
+          <t>ang dili kaantos dili masantos</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>nga ang usa ka tawo naugtang sa usa ka sakyanan</t>
+          <t>walay kasakit</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Si Ana nasuko kay siya manakop og ligid tungod sa iyang pagkadula.; Ang iyang kauban sa trabaho pirmi lang manakop og ligid kay walay tarong nga pag-amping.; Si Pedro manakop og ligid kay nagdagan-dagan sa kalsada.; Ang mga tawo nga dili mag-amping sa dalan kasagaran manakop og ligid.; Si Juan nakasulay nga manakop og ligid human nag-away sa iyang amigo.; "Ayaw pag manakop og ligid, klaroha imong gibuhat."; "Manakop og ligid kaayo imong mga plano, walay klaro."; "Si Pedro, manakop og ligid ug walay klaro."; "Ayaw pag manakop og ligid, siguroha imong mga desisyon."; "Manakop og ligid imong mga ideas, kinahanglan pa nimo ug focus."</t>
+          <t>Ang mga estudyante nga dili magtuon dili gayud makapasar.; Ang mga tawo nga dili magtrabaho dili makatagamtam sa bunga sa ilang pagpaningkamot.; Ang mga atleta nga dili mag-ensayo dili makadaug sa kompetisyon.; Ang mga negosyante nga dili mag-invest dili moasinso.; Ang mga magtutudlo nga dili magplano dili makalampus sa ilang mga estudyante.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Si Ana nasuko kay siya manakop og ligid tungod sa iyang pagkadula.; Ang iyang kauban sa trabaho pirmi lang manakop og ligid kay walay tarong nga pag-amping.; Si Pedro manakop og ligid kay nagdagan-dagan sa kalsada.; Ang mga tawo nga dili mag-amping sa dalan kasagaran manakop og ligid.; Si Juan nakasulay nga manakop og ligid human nag-away sa iyang amigo.; "Ayaw pag manakop og ligid, klaroha imong gibuhat."; "Manakop og ligid kaayo imong mga plano, walay klaro."; "Si Pedro, manakop og ligid ug walay klaro."; "Ayaw pag manakop og ligid, siguroha imong mga desisyon."; "Manakop og ligid imong mga ideas, kinahanglan pa nimo ug focus."</t>
+          <t>Ang mga estudyante nga dili magtuon dili gayud makapasar.; Ang mga tawo nga dili magtrabaho dili makatagamtam sa bunga sa ilang pagpaningkamot.; Ang mga atleta nga dili mag-ensayo dili makadaug sa kompetisyon.; Ang mga negosyante nga dili mag-invest dili moasinso.; Ang mga magtutudlo nga dili magplano dili makalampus sa ilang mga estudyante.</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>['manakop']</t>
+          <t>['makaantos, masantos']</t>
         </is>
       </c>
       <c r="F115" t="n">
@@ -3883,27 +3883,27 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>mangayo og manghod</t>
+          <t>ang gaba dili magsaba</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>usa ka kaso sa bata nga nag-asuso o nag-agom sa iyang mga tudlo</t>
+          <t>ang silot tungod sa iyang mga sayop o mga paglapas moabut sa wala damha</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Si Ana pirmi mangayo og manghod kung magdula.; Ang iyang anak mangayo og manghod kung gutom na.; Si Pedro nakakita sa iyang anak nga mangayo og manghod sa iyang tiil.; Ang mga bata nga mangayo og manghod kasagaran mga healthy nga bata.; Si Juan nalipay kay ang iyang baby nakakat-on nga mangayo og manghod.</t>
+          <t>Ang mga nagpakasala magulat lang kay ang gaba dili magsaba.; Si Pedro nabulabog kay nasuko ang iyang giilad, ang gaba dili magsaba.; Si Juan nakabalo nga ang iyang gibuhat nga dili maayo mibalik kaniya, ang gaba dili magsaba.; Ang mga tawo nga nagbuhat ug dautan maghulat sa ilang gaba kay ang gaba dili magsaba.; Si Ana nabulabog kay ang gaba dili magsaba sa iyang gibuhat nga sayop.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Si Ana pirmi mangayo og manghod kung magdula.; Ang iyang anak mangayo og manghod kung gutom na.; Si Pedro nakakita sa iyang anak nga mangayo og manghod sa iyang tiil.; Ang mga bata nga mangayo og manghod kasagaran mga healthy nga bata.; Si Juan nalipay kay ang iyang baby nakakat-on nga mangayo og manghod.</t>
+          <t>Ang mga nagpakasala magulat lang kay ang gaba dili magsaba.; Si Pedro nabulabog kay nasuko ang iyang giilad, ang gaba dili magsaba.; Si Juan nakabalo nga ang iyang gibuhat nga dili maayo mibalik kaniya, ang gaba dili magsaba.; Ang mga tawo nga nagbuhat ug dautan maghulat sa ilang gaba kay ang gaba dili magsaba.; Si Ana nabulabog kay ang gaba dili magsaba sa iyang gibuhat nga sayop.</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>['mangayo']</t>
+          <t>['magsaba']</t>
         </is>
       </c>
       <c r="F116" t="n">
@@ -3913,27 +3913,27 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>manglutasay</t>
+          <t>ayaw adto og gubat kon wala kay bala</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>usa ka manunulak sa mga bukog</t>
+          <t>ayaw pagbuhat ug dili-andam</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi manglutasay ug uyab nga mga batan-on.; Ang iyang kauban sa trabaho manglutasay sa mga kabataan.; Si Juan giingnan nga manglutasay kay ang iyang uyab mas bata kaayo.; Ang mga tawo nga manglutasay kasagaran magkatawa sa ilang kalaki.; Si Maria nalipay kay ang iyang kauban dili manglutasay.</t>
+          <t>Si Juan giingnan nga ayaw adto og gubat kon wala kay bala kay walay ayo.; Ang mga negosyante giingnan nga ayaw adto og gubat kon wala kay bala sa kompetisyon.; Si Pedro giandam ang tanan sa pag-adto sa exam, ayaw adto og gubat kon wala kay bala.; Ang mga estudyante kinahanglan magtuon kay ayaw adto og gubat kon wala kay bala.; Si Ana nagplano sa iyang project aron dili ma-unsa, ayaw adto og gubat kon wala kay bala.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi manglutasay ug uyab nga mga batan-on.; Ang iyang kauban sa trabaho manglutasay sa mga kabataan.; Si Juan giingnan nga manglutasay kay ang iyang uyab mas bata kaayo.; Ang mga tawo nga manglutasay kasagaran magkatawa sa ilang kalaki.; Si Maria nalipay kay ang iyang kauban dili manglutasay.</t>
+          <t>Si Juan giingnan nga ayaw adto og gubat kon wala kay bala kay walay ayo.; Ang mga negosyante giingnan nga ayaw adto og gubat kon wala kay bala sa kompetisyon.; Si Pedro giandam ang tanan sa pag-adto sa exam, ayaw adto og gubat kon wala kay bala.; Ang mga estudyante kinahanglan magtuon kay ayaw adto og gubat kon wala kay bala.; Si Ana nagplano sa iyang project aron dili ma-unsa, ayaw adto og gubat kon wala kay bala.</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>['manglutasay']</t>
+          <t>['adto']</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -3943,27 +3943,27 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>mangnukos</t>
+          <t>bisan ang kabaw nga naay upat ka tiil masipyat</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>sa pag-abli sa usa ka pista</t>
+          <t>kitang tanan magkamali</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Si Ana nalipay kay ang iyang kauban dili mangnukos sa mga event.; Ang iyang kauban sa trabaho pirmi lang mangnukos sa mga party.; Si Pedro mangnukos sa mga events nga walay imbitasyon.; Ang mga tawo nga mangnukos kasagaran magpahimulos sa libre nga pagkaon.; Si Juan giingnan nga dili mangnukos sa party sa iyang amiga.</t>
+          <t>Si Ana nakasala sa iyang trabaho, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang iyang amigo nakalimot sa meeting, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Pedro nasipyat sa exam, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang mga tawo kasagaran maghimo og sayop, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Maria nasipyat sa pagplano, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Si Ana nalipay kay ang iyang kauban dili mangnukos sa mga event.; Ang iyang kauban sa trabaho pirmi lang mangnukos sa mga party.; Si Pedro mangnukos sa mga events nga walay imbitasyon.; Ang mga tawo nga mangnukos kasagaran magpahimulos sa libre nga pagkaon.; Si Juan giingnan nga dili mangnukos sa party sa iyang amiga.</t>
+          <t>Si Ana nakasala sa iyang trabaho, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang iyang amigo nakalimot sa meeting, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Pedro nasipyat sa exam, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang mga tawo kasagaran maghimo og sayop, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Maria nasipyat sa pagplano, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>['mangnukos']</t>
+          <t>['naay', 'masipyat']</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -3973,27 +3973,27 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>manira sa dalan</t>
+          <t>buhat ang pasulti-on dili sulti ang pabuhaton</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>aron magpabilin nga magmata hangtod sa gabii</t>
+          <t>Maglakaw sa paghisgot</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi manira sa dalan kada gabii.; Ang iyang barkada manira sa dalan hangtud sa kaadlawon.; Si Juan manira sa dalan kung walay klase.; Ang mga batan-on kasagaran manira sa dalan kung walay lingaw.; Si Maria ug ang iyang mga amiga manira sa dalan human sa trabaho.; "Ayaw pag manira sa dalan, naa pa kay buhaton."; "Si Ana, sige lang manira sa dalan walay klaro."; "Manira sa dalan imong mga plano, walay padulngan."; "Ayaw pag manira sa dalan, klaroha imong mga desisyon."; "Manira sa dalan kaayo ka, kinahanglan pa nimo ug focus."</t>
+          <t>Si Juan giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa iyang trabaho.; Ang mga estudyante giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa ilang proyekto.; Si Pedro nagpakita nga maayo siya sa trabaho, buhat ang pasulti-on dili sulti ang pabuhaton.; Ang mga tawo nga buhat ang pasulti-on dili sulti ang pabuhaton kasagaran magmalampuson.; Si Ana nagpakita sa iyang abilidad sa pagtrabaho, buhat ang pasulti-on dili sulti ang pabuhaton.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi manira sa dalan kada gabii.; Ang iyang barkada manira sa dalan hangtud sa kaadlawon.; Si Juan manira sa dalan kung walay klase.; Ang mga batan-on kasagaran manira sa dalan kung walay lingaw.; Si Maria ug ang iyang mga amiga manira sa dalan human sa trabaho.; "Ayaw pag manira sa dalan, naa pa kay buhaton."; "Si Ana, sige lang manira sa dalan walay klaro."; "Manira sa dalan imong mga plano, walay padulngan."; "Ayaw pag manira sa dalan, klaroha imong mga desisyon."; "Manira sa dalan kaayo ka, kinahanglan pa nimo ug focus."</t>
+          <t>Si Juan giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa iyang trabaho.; Ang mga estudyante giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa ilang proyekto.; Si Pedro nagpakita nga maayo siya sa trabaho, buhat ang pasulti-on dili sulti ang pabuhaton.; Ang mga tawo nga buhat ang pasulti-on dili sulti ang pabuhaton kasagaran magmalampuson.; Si Ana nagpakita sa iyang abilidad sa pagtrabaho, buhat ang pasulti-on dili sulti ang pabuhaton.</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>['manira']</t>
+          <t>['pasulti-on, pabuhaton']</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -4003,27 +4003,27 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>may tawo na ang payag</t>
+          <t>dili na mabalik ang baha paingon sa bukid</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>alang sa usa ka babaye nga adunay higugmaon</t>
+          <t>Ang nahimo dili mahimong malikayan</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Si Ana dili na pwede uyabon kay may tawo na ang payag.; Ang iyang crush may tawo na ang payag, mao nga dili na siya magpursige.; Si Pedro naay gipanguyaban nga may tawo na ang payag.; Ang mga batan-on kasagaran dili na mangita ug uyab kung may tawo na ang payag.; Si Maria niingon nga may tawo na ang payag mao nga dili siya ganahan sa uban.</t>
+          <t>Si Juan nasayod nga dili na mabalik ang baha paingon sa bukid, mao nga nagpadayon na siya.; Ang mga tawo giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na.; Si Pedro giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga naghinuktok na lang.; Ang mga estudyante nakabalo nga dili na mabalik ang baha paingon sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na sa iyang kinabuhi.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Si Ana dili na pwede uyabon kay may tawo na ang payag.; Ang iyang crush may tawo na ang payag, mao nga dili na siya magpursige.; Si Pedro naay gipanguyaban nga may tawo na ang payag.; Ang mga batan-on kasagaran dili na mangita ug uyab kung may tawo na ang payag.; Si Maria niingon nga may tawo na ang payag mao nga dili siya ganahan sa uban.</t>
+          <t>Si Juan nasayod nga dili na mabalik ang baha paingon sa bukid, mao nga nagpadayon na siya.; Ang mga tawo giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na.; Si Pedro giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga naghinuktok na lang.; Ang mga estudyante nakabalo nga dili na mabalik ang baha paingon sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na sa iyang kinabuhi.</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>['may']</t>
+          <t>['mabalik']</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -4033,27 +4033,27 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>miulbo ang kaspa</t>
+          <t>dili na nimo mabalik ang baha sa bukid</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>sa pag-abli ngadto sa kasuko</t>
+          <t>Ang nahimo nahimo na</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Si Ana miulbo ang kaspa human nabal-an nga gilimbongan siya.; Ang iyang boss miulbo ang kaspa tungod sa sayop nga trabaho.; Si Pedro miulbo ang kaspa human naay nakig-away niya.; Ang mga tawo nga dali masuko kasagaran miulbo ang kaspa sa gamay nga rason.; Si Maria miulbo ang kaspa kay wala siya natagaan ug hustisya.</t>
+          <t>Si Pedro giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga naghinuktok na lang siya.; Ang mga estudyante nakabalo nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na nimo mabalik ang baha sa bukid, mao nga nag-move on na siya.; Ang iyang pamilya giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila og tarong.; Si Maria giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagpadayon na sa iyang mga plano.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Si Ana miulbo ang kaspa human nabal-an nga gilimbongan siya.; Ang iyang boss miulbo ang kaspa tungod sa sayop nga trabaho.; Si Pedro miulbo ang kaspa human naay nakig-away niya.; Ang mga tawo nga dali masuko kasagaran miulbo ang kaspa sa gamay nga rason.; Si Maria miulbo ang kaspa kay wala siya natagaan ug hustisya.</t>
+          <t>Si Pedro giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga naghinuktok na lang siya.; Ang mga estudyante nakabalo nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na nimo mabalik ang baha sa bukid, mao nga nag-move on na siya.; Ang iyang pamilya giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila og tarong.; Si Maria giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagpadayon na sa iyang mga plano.</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>['miulbo']</t>
+          <t>['mabalik']</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -4063,27 +4063,27 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ang dili kaantos dili masantos</t>
+          <t>dili tanang butang sili nga mohalang dayon</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>walay kasakit</t>
+          <t>Dili tanan mahitabo sa usa ka higayon</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Ang mga estudyante nga dili magtuon dili gayud makapasar.; Ang mga tawo nga dili magtrabaho dili makatagamtam sa bunga sa ilang pagpaningkamot.; Ang mga atleta nga dili mag-ensayo dili makadaug sa kompetisyon.; Ang mga negosyante nga dili mag-invest dili moasinso.; Ang mga magtutudlo nga dili magplano dili makalampus sa ilang mga estudyante.</t>
+          <t>Si Pedro naghinuktok nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.; Ang mga estudyante giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan magtuon pag-ayo.; Si Ana nakasabot nga dili tanang butang sili nga mohalang dayon, mao nga nagplano og maayo.; Ang mga tawo nga dili tanang butang sili nga mohalang dayon kasagaran magmalampuson sa ilang mga plano.; Si Maria giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Ang mga estudyante nga dili magtuon dili gayud makapasar.; Ang mga tawo nga dili magtrabaho dili makatagamtam sa bunga sa ilang pagpaningkamot.; Ang mga atleta nga dili mag-ensayo dili makadaug sa kompetisyon.; Ang mga negosyante nga dili mag-invest dili moasinso.; Ang mga magtutudlo nga dili magplano dili makalampus sa ilang mga estudyante.</t>
+          <t>Si Pedro naghinuktok nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.; Ang mga estudyante giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan magtuon pag-ayo.; Si Ana nakasabot nga dili tanang butang sili nga mohalang dayon, mao nga nagplano og maayo.; Ang mga tawo nga dili tanang butang sili nga mohalang dayon kasagaran magmalampuson sa ilang mga plano.; Si Maria giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>['makaantos, masantos']</t>
+          <t>['mohalang']</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -4093,27 +4093,27 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ang gaba dili magsaba</t>
+          <t>maayo pa ang kwarta naay tawo, ang tawo wala</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>ang silot tungod sa iyang mga sayop o mga paglapas moabut sa wala damha</t>
+          <t>ang usa tingali makaagi ug malisod nga mga panahon</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Ang mga nagpakasala magulat lang kay ang gaba dili magsaba.; Si Pedro nabulabog kay nasuko ang iyang giilad, ang gaba dili magsaba.; Si Juan nakabalo nga ang iyang gibuhat nga dili maayo mibalik kaniya, ang gaba dili magsaba.; Ang mga tawo nga nagbuhat ug dautan maghulat sa ilang gaba kay ang gaba dili magsaba.; Si Ana nabulabog kay ang gaba dili magsaba sa iyang gibuhat nga sayop.</t>
+          <t>Si Juan nagpasalamat nga naa siyay kwarta kay lisod ang panahon, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Pedro nagkalisod tungod kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang pamilya naglisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Ana nagstruggle kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang mga negosyante nagkalisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Ang mga nagpakasala magulat lang kay ang gaba dili magsaba.; Si Pedro nabulabog kay nasuko ang iyang giilad, ang gaba dili magsaba.; Si Juan nakabalo nga ang iyang gibuhat nga dili maayo mibalik kaniya, ang gaba dili magsaba.; Ang mga tawo nga nagbuhat ug dautan maghulat sa ilang gaba kay ang gaba dili magsaba.; Si Ana nabulabog kay ang gaba dili magsaba sa iyang gibuhat nga sayop.</t>
+          <t>Si Juan nagpasalamat nga naa siyay kwarta kay lisod ang panahon, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Pedro nagkalisod tungod kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang pamilya naglisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Ana nagstruggle kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang mga negosyante nagkalisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>['magsaba']</t>
+          <t>['naay']</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -4123,27 +4123,27 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ayaw adto og gubat kon wala kay bala</t>
+          <t>madala nimo ang baka sa suba apan dili nimo mainom</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ayaw pagbuhat ug dili-andam</t>
+          <t>Mahimo nimong pagdala ang kabayo ngadto sa tubig</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Si Juan giingnan nga ayaw adto og gubat kon wala kay bala kay walay ayo.; Ang mga negosyante giingnan nga ayaw adto og gubat kon wala kay bala sa kompetisyon.; Si Pedro giandam ang tanan sa pag-adto sa exam, ayaw adto og gubat kon wala kay bala.; Ang mga estudyante kinahanglan magtuon kay ayaw adto og gubat kon wala kay bala.; Si Ana nagplano sa iyang project aron dili ma-unsa, ayaw adto og gubat kon wala kay bala.</t>
+          <t>Si Pedro giingnan nga bisan unsaon pagdasig, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga estudyante kinahanglan magtuon, madala nimo ang baka sa suba apan dili nimo mainom.; Si Ana giingnan nga kinahanglan siya magpursige, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga tawo nga dili magpaningkamot dili gyud magmalampuson, madala nimo ang baka sa suba apan dili nimo mainom.; Si Maria giingnan nga kinahanglan siya mag-uban sa pagpaningkamot, madala nimo ang baka sa suba apan dili nimo mainom.</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Si Juan giingnan nga ayaw adto og gubat kon wala kay bala kay walay ayo.; Ang mga negosyante giingnan nga ayaw adto og gubat kon wala kay bala sa kompetisyon.; Si Pedro giandam ang tanan sa pag-adto sa exam, ayaw adto og gubat kon wala kay bala.; Ang mga estudyante kinahanglan magtuon kay ayaw adto og gubat kon wala kay bala.; Si Ana nagplano sa iyang project aron dili ma-unsa, ayaw adto og gubat kon wala kay bala.</t>
+          <t>Si Pedro giingnan nga bisan unsaon pagdasig, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga estudyante kinahanglan magtuon, madala nimo ang baka sa suba apan dili nimo mainom.; Si Ana giingnan nga kinahanglan siya magpursige, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga tawo nga dili magpaningkamot dili gyud magmalampuson, madala nimo ang baka sa suba apan dili nimo mainom.; Si Maria giingnan nga kinahanglan siya mag-uban sa pagpaningkamot, madala nimo ang baka sa suba apan dili nimo mainom.</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>['adto']</t>
+          <t>['madala', 'mainom']</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -4153,27 +4153,27 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>bisan ang kabaw nga naay upat ka tiil masipyat</t>
+          <t>sa usa ka bulig naa gayod usa ka buang</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>kitang tanan magkamali</t>
+          <t>Adunay usa ka putli nga mansanas sa matag bariles</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Si Ana nakasala sa iyang trabaho, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang iyang amigo nakalimot sa meeting, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Pedro nasipyat sa exam, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang mga tawo kasagaran maghimo og sayop, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Maria nasipyat sa pagplano, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
+          <t>Ang grupo nga magkatapok kasagaran naa gyud usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Pedro nagpakatawa sa iyang grupo, sa usa ka bulig naa gayod usa ka buang.; Ang mga kauban sa trabaho kasagaran naa'y usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Ana nagpakatawa sa iyang mga amiga, sa usa ka bulig naa gayod usa ka buang.; Ang pamilya kasagaran naa gyud usa ka buang nga magpatawa, sa usa ka bulig naa gayod usa ka buang.</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Si Ana nakasala sa iyang trabaho, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang iyang amigo nakalimot sa meeting, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Pedro nasipyat sa exam, bisan ang kabaw nga naay upat ka tiil masipyat.; Ang mga tawo kasagaran maghimo og sayop, bisan ang kabaw nga naay upat ka tiil masipyat.; Si Maria nasipyat sa pagplano, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
+          <t>Ang grupo nga magkatapok kasagaran naa gyud usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Pedro nagpakatawa sa iyang grupo, sa usa ka bulig naa gayod usa ka buang.; Ang mga kauban sa trabaho kasagaran naa'y usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Ana nagpakatawa sa iyang mga amiga, sa usa ka bulig naa gayod usa ka buang.; Ang pamilya kasagaran naa gyud usa ka buang nga magpatawa, sa usa ka bulig naa gayod usa ka buang.</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>['naay', 'masipyat']</t>
+          <t>['naa']</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -4183,27 +4183,27 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>buhat ang pasulti-on dili sulti ang pabuhaton</t>
+          <t>walay aso makumkom</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Maglakaw sa paghisgot</t>
+          <t>walay sekreto nga magpabilin nga sekreto</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Si Juan giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa iyang trabaho.; Ang mga estudyante giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa ilang proyekto.; Si Pedro nagpakita nga maayo siya sa trabaho, buhat ang pasulti-on dili sulti ang pabuhaton.; Ang mga tawo nga buhat ang pasulti-on dili sulti ang pabuhaton kasagaran magmalampuson.; Si Ana nagpakita sa iyang abilidad sa pagtrabaho, buhat ang pasulti-on dili sulti ang pabuhaton.</t>
+          <t>Si Pedro nasayod nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.; Ang mga tawo giingnan nga walay aso makumkom, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay aso makumkom, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay aso makumkom, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Si Juan giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa iyang trabaho.; Ang mga estudyante giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa ilang proyekto.; Si Pedro nagpakita nga maayo siya sa trabaho, buhat ang pasulti-on dili sulti ang pabuhaton.; Ang mga tawo nga buhat ang pasulti-on dili sulti ang pabuhaton kasagaran magmalampuson.; Si Ana nagpakita sa iyang abilidad sa pagtrabaho, buhat ang pasulti-on dili sulti ang pabuhaton.</t>
+          <t>Si Pedro nasayod nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.; Ang mga tawo giingnan nga walay aso makumkom, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay aso makumkom, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay aso makumkom, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>['pasulti-on, pabuhaton']</t>
+          <t>['makumkom']</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -4213,7 +4213,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>dili na mabalik ang baha paingon sa bukid</t>
+          <t>walay mahay nga gauna</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -4223,17 +4223,17 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Si Juan nasayod nga dili na mabalik ang baha paingon sa bukid, mao nga nagpadayon na siya.; Ang mga tawo giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na.; Si Pedro giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga naghinuktok na lang.; Ang mga estudyante nakabalo nga dili na mabalik ang baha paingon sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na sa iyang kinabuhi.</t>
+          <t>Si Pedro nakasabot nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay mahay nga gauna, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay mahay nga gauna, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay mahay nga gauna, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Si Juan nasayod nga dili na mabalik ang baha paingon sa bukid, mao nga nagpadayon na siya.; Ang mga tawo giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na.; Si Pedro giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga naghinuktok na lang.; Ang mga estudyante nakabalo nga dili na mabalik ang baha paingon sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na sa iyang kinabuhi.</t>
+          <t>Si Pedro nakasabot nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay mahay nga gauna, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay mahay nga gauna, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay mahay nga gauna, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>['mabalik']</t>
+          <t>['gauna']</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -4243,27 +4243,27 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>dili na nimo mabalik ang baha sa bukid</t>
+          <t>walay man kardaba mamunga og tundan</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Ang nahimo nahimo na</t>
+          <t>ang mansanas dili mahulog nga layo sa kahoy</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Si Pedro giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga naghinuktok na lang siya.; Ang mga estudyante nakabalo nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na nimo mabalik ang baha sa bukid, mao nga nag-move on na siya.; Ang iyang pamilya giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila og tarong.; Si Maria giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagpadayon na sa iyang mga plano.</t>
+          <t>Si Pedro nasayod nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay man kardaba mamunga og tundan, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay man kardaba mamunga og tundan, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay man kardaba mamunga og tundan, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Si Pedro giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga naghinuktok na lang siya.; Ang mga estudyante nakabalo nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila pag-ayo.; Si Ana nakasabot nga dili na nimo mabalik ang baha sa bukid, mao nga nag-move on na siya.; Ang iyang pamilya giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagplano na sila og tarong.; Si Maria giingnan nga dili na nimo mabalik ang baha sa bukid, mao nga nagpadayon na sa iyang mga plano.</t>
+          <t>Si Pedro nasayod nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay man kardaba mamunga og tundan, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay man kardaba mamunga og tundan, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay man kardaba mamunga og tundan, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>['mabalik']</t>
+          <t>['mamunga']</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -4273,27 +4273,27 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>dili tanang butang sili nga mohalang dayon</t>
+          <t>gidaman</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Dili tanan mahitabo sa usa ka higayon</t>
+          <t>sa pag-aturog o pag-aturog</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Si Pedro naghinuktok nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.; Ang mga estudyante giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan magtuon pag-ayo.; Si Ana nakasabot nga dili tanang butang sili nga mohalang dayon, mao nga nagplano og maayo.; Ang mga tawo nga dili tanang butang sili nga mohalang dayon kasagaran magmalampuson sa ilang mga plano.; Si Maria giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.</t>
+          <t>"Gidaman na pud si Pedro, daghan kaayo siya og storya."; "Kung mangutana ka og ing-ana, murag gidaman ka."; "Gidaman na ba ka? Daghan kaayo kag opinion."; "Gidaman na si Juan, sige lang siya og panaway."; "Ayaw ko gidam-i, klaro kaayo imong mga istorya."</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Si Pedro naghinuktok nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.; Ang mga estudyante giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan magtuon pag-ayo.; Si Ana nakasabot nga dili tanang butang sili nga mohalang dayon, mao nga nagplano og maayo.; Ang mga tawo nga dili tanang butang sili nga mohalang dayon kasagaran magmalampuson sa ilang mga plano.; Si Maria giingnan nga dili tanang butang sili nga mohalang dayon, kinahanglan gyud og pagpaningkamot.</t>
+          <t>"Gidaman na pud si Pedro, daghan kaayo siya og storya."; "Kung mangutana ka og ing-ana, murag gidaman ka."; "Gidaman na ba ka? Daghan kaayo kag opinion."; "Gidaman na si Juan, sige lang siya og panaway."; "Ayaw ko gidam-i, klaro kaayo imong mga istorya."</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>['mohalang']</t>
+          <t>['gidaman']</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -4303,27 +4303,27 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>maayo pa ang kwarta naay tawo, ang tawo wala</t>
+          <t>isdaa</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>ang usa tingali makaagi ug malisod nga mga panahon</t>
+          <t>isda</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Si Juan nagpasalamat nga naa siyay kwarta kay lisod ang panahon, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Pedro nagkalisod tungod kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang pamilya naglisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Ana nagstruggle kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang mga negosyante nagkalisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.</t>
+          <t>"Isdaa, ngano magbuhat ka ana?"; "Isdaa, unsa may imong plano?"; "Isdaa, unsa man diay imong gusto mahibal-an?"; "Isdaa, nganong mangutana man ka ana?"; "Isdaa, walay klaro imong pangutana."</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Si Juan nagpasalamat nga naa siyay kwarta kay lisod ang panahon, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Pedro nagkalisod tungod kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang pamilya naglisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.; Si Ana nagstruggle kay walay kwarta, maayo pa ang kwarta naay tawo, ang tawo wala.; Ang mga negosyante nagkalisod tungod sa kawad-on, maayo pa ang kwarta naay tawo, ang tawo wala.</t>
+          <t>"Isdaa, ngano magbuhat ka ana?"; "Isdaa, unsa may imong plano?"; "Isdaa, unsa man diay imong gusto mahibal-an?"; "Isdaa, nganong mangutana man ka ana?"; "Isdaa, walay klaro imong pangutana."</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>['naay']</t>
+          <t>['isdaa']</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -4333,27 +4333,27 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>madala nimo ang baka sa suba apan dili nimo mainom</t>
+          <t>lamoy</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Mahimo nimong pagdala ang kabayo ngadto sa tubig</t>
+          <t>pag-abot</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Si Pedro giingnan nga bisan unsaon pagdasig, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga estudyante kinahanglan magtuon, madala nimo ang baka sa suba apan dili nimo mainom.; Si Ana giingnan nga kinahanglan siya magpursige, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga tawo nga dili magpaningkamot dili gyud magmalampuson, madala nimo ang baka sa suba apan dili nimo mainom.; Si Maria giingnan nga kinahanglan siya mag-uban sa pagpaningkamot, madala nimo ang baka sa suba apan dili nimo mainom.</t>
+          <t>"Lamoya nalang na imong gibuhat, walay gamit."; "Si Ana, sige lang lamoy walay klaro."; "Lamoy nalang na imong giingon, walay unod."; "Lamoy kaayo ka, bisan asa nalang dapita."; "Lamoy imong mga plano, walay klaro."</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Si Pedro giingnan nga bisan unsaon pagdasig, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga estudyante kinahanglan magtuon, madala nimo ang baka sa suba apan dili nimo mainom.; Si Ana giingnan nga kinahanglan siya magpursige, madala nimo ang baka sa suba apan dili nimo mainom.; Ang mga tawo nga dili magpaningkamot dili gyud magmalampuson, madala nimo ang baka sa suba apan dili nimo mainom.; Si Maria giingnan nga kinahanglan siya mag-uban sa pagpaningkamot, madala nimo ang baka sa suba apan dili nimo mainom.</t>
+          <t>"Lamoya nalang na imong gibuhat, walay gamit."; "Si Ana, sige lang lamoy walay klaro."; "Lamoy nalang na imong giingon, walay unod."; "Lamoy kaayo ka, bisan asa nalang dapita."; "Lamoy imong mga plano, walay klaro."</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>['madala', 'mainom']</t>
+          <t>['lamoy']</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -4363,27 +4363,27 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>sa usa ka bulig naa gayod usa ka buang</t>
+          <t>mura og halas nga nagluno</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Adunay usa ka putli nga mansanas sa matag bariles</t>
+          <t>ang usa ka tawo nga magbiya sa iyang mahugaw nga sinina sa tanang dapit sa balay</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Ang grupo nga magkatapok kasagaran naa gyud usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Pedro nagpakatawa sa iyang grupo, sa usa ka bulig naa gayod usa ka buang.; Ang mga kauban sa trabaho kasagaran naa'y usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Ana nagpakatawa sa iyang mga amiga, sa usa ka bulig naa gayod usa ka buang.; Ang pamilya kasagaran naa gyud usa ka buang nga magpatawa, sa usa ka bulig naa gayod usa ka buang.</t>
+          <t>"Ang iyang mga sinina nagkatag mura og halas nga nagluno."; "Ang kwarto sa bata mura og halas nga nagluno, walay nasunod nga kalimpyo."; "Ang sala murag halas nga nagluno, kay gikalat niya tanan iyang mga butang."; "Ang balay ni Pedro mura og halas nga nagluno, nagkatag tanan."; "Ang silingan namo mura og halas nga nagluno, walay tarong pagbutang sa mga gamit."</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Ang grupo nga magkatapok kasagaran naa gyud usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Pedro nagpakatawa sa iyang grupo, sa usa ka bulig naa gayod usa ka buang.; Ang mga kauban sa trabaho kasagaran naa'y usa ka buang, sa usa ka bulig naa gayod usa ka buang.; Si Ana nagpakatawa sa iyang mga amiga, sa usa ka bulig naa gayod usa ka buang.; Ang pamilya kasagaran naa gyud usa ka buang nga magpatawa, sa usa ka bulig naa gayod usa ka buang.</t>
+          <t>"Ang iyang mga sinina nagkatag mura og halas nga nagluno."; "Ang kwarto sa bata mura og halas nga nagluno, walay nasunod nga kalimpyo."; "Ang sala murag halas nga nagluno, kay gikalat niya tanan iyang mga butang."; "Ang balay ni Pedro mura og halas nga nagluno, nagkatag tanan."; "Ang silingan namo mura og halas nga nagluno, walay tarong pagbutang sa mga gamit."</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>['naa']</t>
+          <t>['nagluno']</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -4393,27 +4393,27 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>walay aso makumkom</t>
+          <t>murag gitilapan og iring</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>walay sekreto nga magpabilin nga sekreto</t>
+          <t>walay sapayan</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Si Pedro nasayod nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.; Ang mga tawo giingnan nga walay aso makumkom, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay aso makumkom, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay aso makumkom, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.</t>
+          <t>"Ang iyang sapatos murag gitilapan og iring, limpyo kaayo."; "Ang lamesa sa balay ni Ana murag gitilapan og iring, limpyo kaayo."; "Ang awto ni Pedro murag gitilapan og iring, walay bahid sa hugaw."; "Ang iyang kwarto murag gitilapan og iring, limpyo kaayo."; "Ang iyang mga gamit sa opisina murag gitilapan og iring, limpyo ug hapsay."</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Si Pedro nasayod nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.; Ang mga tawo giingnan nga walay aso makumkom, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay aso makumkom, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay aso makumkom, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.</t>
+          <t>"Ang iyang sapatos murag gitilapan og iring, limpyo kaayo."; "Ang lamesa sa balay ni Ana murag gitilapan og iring, limpyo kaayo."; "Ang awto ni Pedro murag gitilapan og iring, walay bahid sa hugaw."; "Ang iyang kwarto murag gitilapan og iring, limpyo kaayo."; "Ang iyang mga gamit sa opisina murag gitilapan og iring, limpyo ug hapsay."</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>['makumkom']</t>
+          <t>['gitilapan']</t>
         </is>
       </c>
       <c r="F133" t="n">
@@ -4423,27 +4423,27 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>walay mahay nga gauna</t>
+          <t>murag langaw nga nakatugdon sa kabaw</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Ang nahimo dili mahimong malikayan</t>
+          <t>nouveau riche</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Si Pedro nakasabot nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay mahay nga gauna, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay mahay nga gauna, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay mahay nga gauna, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga lihok.</t>
+          <t>"Siya karon murag langaw nga nakatugdon sa kabaw, taas kaayo og pride."; "Ang bag-ong kwartahan murag langaw nga nakatugdon sa kabaw, wala pa kasuway sa kwarta."; "Si Ana, gikan sa pagka-pobre, murag langaw nga nakatugdon sa kabaw karon."; "Ang mga tawo nga bag-o rang nakuhaan ug jackpot murag langaw nga nakatugdon sa kabaw."; "Ang mga bag-o rang nigraduate ug ni trabaho, murag langaw nga nakatugdon sa kabaw."</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Si Pedro nakasabot nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay mahay nga gauna, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay mahay nga gauna, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay mahay nga gauna, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga lihok.</t>
+          <t>"Siya karon murag langaw nga nakatugdon sa kabaw, taas kaayo og pride."; "Ang bag-ong kwartahan murag langaw nga nakatugdon sa kabaw, wala pa kasuway sa kwarta."; "Si Ana, gikan sa pagka-pobre, murag langaw nga nakatugdon sa kabaw karon."; "Ang mga tawo nga bag-o rang nakuhaan ug jackpot murag langaw nga nakatugdon sa kabaw."; "Ang mga bag-o rang nigraduate ug ni trabaho, murag langaw nga nakatugdon sa kabaw."</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>['gauna']</t>
+          <t>['nakatugdon']</t>
         </is>
       </c>
       <c r="F134" t="n">
@@ -4453,27 +4453,27 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>walay man kardaba mamunga og tundan</t>
+          <t>murag namatyag iring</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ang mansanas dili mahulog nga layo sa kahoy</t>
+          <t>gigamit sa paghulagway sa usa ka tawo nga nagtangis nga nagtangis o nagtangis nga nagtangis</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Si Pedro nasayod nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay man kardaba mamunga og tundan, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay man kardaba mamunga og tundan, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay man kardaba mamunga og tundan, mao nga nagmatngon siya sa iyang mga lihok.</t>
+          <t>"Si Pedro murag namatyag iring, sige lang hilak."; "Ang bata murag namatyag iring, hilak kaayo pagnalaya."; "Si Ana murag namatyag iring, dili madala ang iyang hilak."; "Ang iyang asawa murag namatyag iring pagkahibalo nga naay problema."; "Ang mga bata murag namatyag iring pagkahuman sa dula."</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Si Pedro nasayod nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga tawo giingnan nga walay man kardaba mamunga og tundan, mao nga magmatngon sila sa ilang mga buhaton.; Si Ana nakasabot nga walay man kardaba mamunga og tundan, mao nga nagbantay siya sa iyang mga desisyon.; Ang mga estudyante giingnan nga walay man kardaba mamunga og tundan, mao nga magtuon sila pag-ayo.; Si Maria giingnan nga walay man kardaba mamunga og tundan, mao nga nagmatngon siya sa iyang mga lihok.</t>
+          <t>"Si Pedro murag namatyag iring, sige lang hilak."; "Ang bata murag namatyag iring, hilak kaayo pagnalaya."; "Si Ana murag namatyag iring, dili madala ang iyang hilak."; "Ang iyang asawa murag namatyag iring pagkahibalo nga naay problema."; "Ang mga bata murag namatyag iring pagkahuman sa dula."</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>['mamunga']</t>
+          <t>['namatyag']</t>
         </is>
       </c>
       <c r="F135" t="n">
@@ -4483,240 +4483,30 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>gidaman</t>
+          <t>murag namiya og tai</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>sa pag-aturog o pag-aturog</t>
+          <t>Usa ka tawo nga mibiya sa dili-iasa nga walay iyang pulong</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>"Gidaman na pud si Pedro, daghan kaayo siya og storya."; "Kung mangutana ka og ing-ana, murag gidaman ka."; "Gidaman na ba ka? Daghan kaayo kag opinion."; "Gidaman na si Juan, sige lang siya og panaway."; "Ayaw ko gidam-i, klaro kaayo imong mga istorya."</t>
+          <t>"Siya kalit lang murag namiya og tai, wala na gani nagpahibalo."; "Ang bata murag namiya og tai, kalit lang nawala."; "Si Pedro murag namiya og tai, wala na gani nagpahibalo sa iyang mga kauban."; "Ang silingan murag namiya og tai, kalit lang wala."; "Si Ana murag namiya og tai, wala na gani nagpahibalo sa iyang mga plano."</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>"Gidaman na pud si Pedro, daghan kaayo siya og storya."; "Kung mangutana ka og ing-ana, murag gidaman ka."; "Gidaman na ba ka? Daghan kaayo kag opinion."; "Gidaman na si Juan, sige lang siya og panaway."; "Ayaw ko gidam-i, klaro kaayo imong mga istorya."</t>
+          <t>"Siya kalit lang murag namiya og tai, wala na gani nagpahibalo."; "Ang bata murag namiya og tai, kalit lang nawala."; "Si Pedro murag namiya og tai, wala na gani nagpahibalo sa iyang mga kauban."; "Ang silingan murag namiya og tai, kalit lang wala."; "Si Ana murag namiya og tai, wala na gani nagpahibalo sa iyang mga plano."</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>['gidaman']</t>
+          <t>['namiya']</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>isdaa</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>isda</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>"Isdaa, ngano magbuhat ka ana?"; "Isdaa, unsa may imong plano?"; "Isdaa, unsa man diay imong gusto mahibal-an?"; "Isdaa, nganong mangutana man ka ana?"; "Isdaa, walay klaro imong pangutana."</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>"Isdaa, ngano magbuhat ka ana?"; "Isdaa, unsa may imong plano?"; "Isdaa, unsa man diay imong gusto mahibal-an?"; "Isdaa, nganong mangutana man ka ana?"; "Isdaa, walay klaro imong pangutana."</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>['isdaa']</t>
-        </is>
-      </c>
-      <c r="F137" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>lamoy</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>pag-abot</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>"Lamoya nalang na imong gibuhat, walay gamit."; "Si Ana, sige lang lamoy walay klaro."; "Lamoy nalang na imong giingon, walay unod."; "Lamoy kaayo ka, bisan asa nalang dapita."; "Lamoy imong mga plano, walay klaro."</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>"Lamoya nalang na imong gibuhat, walay gamit."; "Si Ana, sige lang lamoy walay klaro."; "Lamoy nalang na imong giingon, walay unod."; "Lamoy kaayo ka, bisan asa nalang dapita."; "Lamoy imong mga plano, walay klaro."</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>['lamoy']</t>
-        </is>
-      </c>
-      <c r="F138" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>mura og halas nga nagluno</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>ang usa ka tawo nga magbiya sa iyang mahugaw nga sinina sa tanang dapit sa balay</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>"Ang iyang mga sinina nagkatag mura og halas nga nagluno."; "Ang kwarto sa bata mura og halas nga nagluno, walay nasunod nga kalimpyo."; "Ang sala murag halas nga nagluno, kay gikalat niya tanan iyang mga butang."; "Ang balay ni Pedro mura og halas nga nagluno, nagkatag tanan."; "Ang silingan namo mura og halas nga nagluno, walay tarong pagbutang sa mga gamit."</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>"Ang iyang mga sinina nagkatag mura og halas nga nagluno."; "Ang kwarto sa bata mura og halas nga nagluno, walay nasunod nga kalimpyo."; "Ang sala murag halas nga nagluno, kay gikalat niya tanan iyang mga butang."; "Ang balay ni Pedro mura og halas nga nagluno, nagkatag tanan."; "Ang silingan namo mura og halas nga nagluno, walay tarong pagbutang sa mga gamit."</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>['nagluno']</t>
-        </is>
-      </c>
-      <c r="F139" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>murag gitilapan og iring</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>walay sapayan</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>"Ang iyang sapatos murag gitilapan og iring, limpyo kaayo."; "Ang lamesa sa balay ni Ana murag gitilapan og iring, limpyo kaayo."; "Ang awto ni Pedro murag gitilapan og iring, walay bahid sa hugaw."; "Ang iyang kwarto murag gitilapan og iring, limpyo kaayo."; "Ang iyang mga gamit sa opisina murag gitilapan og iring, limpyo ug hapsay."</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>"Ang iyang sapatos murag gitilapan og iring, limpyo kaayo."; "Ang lamesa sa balay ni Ana murag gitilapan og iring, limpyo kaayo."; "Ang awto ni Pedro murag gitilapan og iring, walay bahid sa hugaw."; "Ang iyang kwarto murag gitilapan og iring, limpyo kaayo."; "Ang iyang mga gamit sa opisina murag gitilapan og iring, limpyo ug hapsay."</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>['gitilapan']</t>
-        </is>
-      </c>
-      <c r="F140" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>murag langaw nga nakatugdon sa kabaw</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>nouveau riche</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>"Siya karon murag langaw nga nakatugdon sa kabaw, taas kaayo og pride."; "Ang bag-ong kwartahan murag langaw nga nakatugdon sa kabaw, wala pa kasuway sa kwarta."; "Si Ana, gikan sa pagka-pobre, murag langaw nga nakatugdon sa kabaw karon."; "Ang mga tawo nga bag-o rang nakuhaan ug jackpot murag langaw nga nakatugdon sa kabaw."; "Ang mga bag-o rang nigraduate ug ni trabaho, murag langaw nga nakatugdon sa kabaw."</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>"Siya karon murag langaw nga nakatugdon sa kabaw, taas kaayo og pride."; "Ang bag-ong kwartahan murag langaw nga nakatugdon sa kabaw, wala pa kasuway sa kwarta."; "Si Ana, gikan sa pagka-pobre, murag langaw nga nakatugdon sa kabaw karon."; "Ang mga tawo nga bag-o rang nakuhaan ug jackpot murag langaw nga nakatugdon sa kabaw."; "Ang mga bag-o rang nigraduate ug ni trabaho, murag langaw nga nakatugdon sa kabaw."</t>
-        </is>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>['nakatugdon']</t>
-        </is>
-      </c>
-      <c r="F141" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>murag namatyag iring</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>gigamit sa paghulagway sa usa ka tawo nga nagtangis nga nagtangis o nagtangis nga nagtangis</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>"Si Pedro murag namatyag iring, sige lang hilak."; "Ang bata murag namatyag iring, hilak kaayo pagnalaya."; "Si Ana murag namatyag iring, dili madala ang iyang hilak."; "Ang iyang asawa murag namatyag iring pagkahibalo nga naay problema."; "Ang mga bata murag namatyag iring pagkahuman sa dula."</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>"Si Pedro murag namatyag iring, sige lang hilak."; "Ang bata murag namatyag iring, hilak kaayo pagnalaya."; "Si Ana murag namatyag iring, dili madala ang iyang hilak."; "Ang iyang asawa murag namatyag iring pagkahibalo nga naay problema."; "Ang mga bata murag namatyag iring pagkahuman sa dula."</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>['namatyag']</t>
-        </is>
-      </c>
-      <c r="F142" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>murag namiya og tai</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>Usa ka tawo nga mibiya sa dili-iasa nga walay iyang pulong</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>"Siya kalit lang murag namiya og tai, wala na gani nagpahibalo."; "Ang bata murag namiya og tai, kalit lang nawala."; "Si Pedro murag namiya og tai, wala na gani nagpahibalo sa iyang mga kauban."; "Ang silingan murag namiya og tai, kalit lang wala."; "Si Ana murag namiya og tai, wala na gani nagpahibalo sa iyang mga plano."</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>"Siya kalit lang murag namiya og tai, wala na gani nagpahibalo."; "Ang bata murag namiya og tai, kalit lang nawala."; "Si Pedro murag namiya og tai, wala na gani nagpahibalo sa iyang mga kauban."; "Ang silingan murag namiya og tai, kalit lang wala."; "Si Ana murag namiya og tai, wala na gani nagpahibalo sa iyang mga plano."</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>['namiya']</t>
-        </is>
-      </c>
-      <c r="F143" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>